<commit_message>
added 3d models, added more resistors, added 16X2 LCD module, modified Pico 2 footprint
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\russe\Repositories\MIL\MIL-Altium\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB364E85-36F3-4680-B92F-F6C1D0BE1D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F81F15F8-F8E2-4C0F-9B99-826A01E46FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="630" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="5" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="7" activeTab="13" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="272">
   <si>
     <t>Capacitance</t>
   </si>
@@ -771,9 +771,6 @@
     <t>Misc Components</t>
   </si>
   <si>
-    <t>M3 MountHole</t>
-  </si>
-  <si>
     <t>Default mount hole</t>
   </si>
   <si>
@@ -844,6 +841,36 @@
   </si>
   <si>
     <t>Pi 5 w/ active cooler</t>
+  </si>
+  <si>
+    <t>LCD</t>
+  </si>
+  <si>
+    <t>16x2 LCD Display</t>
+  </si>
+  <si>
+    <t>16x2 LCD, no driver, only parallel pins</t>
+  </si>
+  <si>
+    <t>M3 Mount Hole</t>
+  </si>
+  <si>
+    <t>3386T-1-103LF</t>
+  </si>
+  <si>
+    <t>10 kOhms 0.5W, 1/2W PC Pins Through Hole Trimmer Potentiometer Cermet 1.0 Turn Top Adjustment</t>
+  </si>
+  <si>
+    <t>1/4W</t>
+  </si>
+  <si>
+    <t>MFR-25FTF52-100K</t>
+  </si>
+  <si>
+    <t>100 kOhms ±1% 0.25W, 1/4W Through Hole Resistor Axial Metal Film</t>
+  </si>
+  <si>
+    <t>100k</t>
   </si>
 </sst>
 </file>
@@ -969,24 +996,7 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
@@ -1072,7 +1082,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
@@ -1085,7 +1095,7 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
@@ -1095,7 +1105,7 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
@@ -1120,28 +1130,28 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
@@ -1169,7 +1179,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
@@ -1184,6 +1194,23 @@
       </extLst>
     </dxf>
     <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1211,7 +1238,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
@@ -1227,7 +1254,7 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
@@ -1264,8 +1291,8 @@
   </bag>
   <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
     <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
       <bagId>5</bagId>
-      <bagId>2</bagId>
     </a>
   </bag>
 </FeaturePropertyBags>
@@ -1293,10 +1320,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:G10" totalsRowShown="0">
   <autoFilter ref="A1:G10" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="26"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="25"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -1308,8 +1335,11 @@
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{7B88261C-6B3D-4539-9169-7D9FC231B64A}" name="Misc" displayName="Misc" ref="A1:D13" totalsRowShown="0">
   <autoFilter ref="A1:D13" xr:uid="{7B88261C-6B3D-4539-9169-7D9FC231B64A}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D13">
+    <sortCondition ref="B1:B13"/>
+  </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="24"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -1319,37 +1349,37 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="24"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="22"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="21"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="20"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="19"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="18"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="17"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="16"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="15"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H22" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H22" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A1:H22" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H22">
     <sortCondition ref="C1:C22"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="12"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="10">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="7">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -1357,11 +1387,11 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1371,7 +1401,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}" name="Switches" displayName="Switches" ref="A1:G11" totalsRowShown="0">
   <autoFilter ref="A1:G11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="1"/>
     <tableColumn id="1" xr3:uid="{C868B851-3D2D-4863-96B3-5412E9A862E1}" name="Function"/>
     <tableColumn id="6" xr3:uid="{D6EA3AC7-CEF9-4E2A-800B-297C8C002273}" name="Circuit"/>
     <tableColumn id="2" xr3:uid="{5048C5E7-258E-4EC2-B0BD-C338C4D84C91}" name="Part Number"/>
@@ -1387,7 +1417,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{82CFED5E-627B-4A23-9BFA-C489CEA32F25}" name="Voltage_Regulators" displayName="Voltage_Regulators" ref="A1:H12" totalsRowShown="0">
   <autoFilter ref="A1:H12" xr:uid="{82CFED5E-627B-4A23-9BFA-C489CEA32F25}"/>
   <tableColumns count="8">
-    <tableColumn id="3" xr3:uid="{DD7A1A9A-DE5A-4766-9947-A308E87BA7FD}" name="Added to Altium?" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{DD7A1A9A-DE5A-4766-9947-A308E87BA7FD}" name="Added to Altium?" dataDxfId="0"/>
     <tableColumn id="1" xr3:uid="{7B7659A2-8D22-4954-B10E-C811D8D29B99}" name="Type"/>
     <tableColumn id="7" xr3:uid="{24DD5DAD-1853-4138-AB66-BA5667E60D26}" name="Operation"/>
     <tableColumn id="8" xr3:uid="{C0E1C407-BC33-4018-B09E-15A16329D7C6}" name="Input Voltage"/>
@@ -1453,11 +1483,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Diodes3" displayName="Diodes3" ref="A1:F7" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Diodes3" displayName="Diodes3" ref="A1:F7" totalsRowShown="0" headerRowDxfId="46">
   <autoFilter ref="A1:F7" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="45"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="44"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -1468,25 +1498,25 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="43">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="45"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:G10" totalsRowShown="0" headerRowDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:G10" totalsRowShown="0" headerRowDxfId="37">
   <autoFilter ref="A1:G10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="39"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="36"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="35"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
     <tableColumn id="3" xr3:uid="{7EDCBE59-D502-4146-84D0-ACB598015CAD}" name="Max Voltage"/>
@@ -1501,8 +1531,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}" name="ICs" displayName="ICs" ref="A1:E10" totalsRowShown="0">
   <autoFilter ref="A1:E10" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}"/>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="33"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -1512,14 +1542,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="32">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="34"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2226,49 +2256,58 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C2" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
       <c r="D2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>136</v>
+        <v>265</v>
       </c>
       <c r="C3" t="s">
-        <v>137</v>
+        <v>208</v>
       </c>
       <c r="D3" t="s">
-        <v>138</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>240</v>
+        <v>136</v>
       </c>
       <c r="C4" t="s">
-        <v>241</v>
+        <v>137</v>
       </c>
       <c r="D4" t="s">
-        <v>242</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C5" t="s">
+        <v>266</v>
+      </c>
+      <c r="D5" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -2520,7 +2559,7 @@
         <v>27</v>
       </c>
       <c r="C2" s="17">
-        <f t="shared" ref="C2:C22" si="0">IF(ISNUMBER(B2),
+        <f>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
 IF(RIGHT(B2,1)="k",1000,
@@ -2552,7 +2591,12 @@
         <v>33</v>
       </c>
       <c r="C3" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B3),
+IF(B3=0,"",B3),
+VALUE(LEFT(B3,LEN(B3)-1))*
+IF(RIGHT(B3,1)="k",1000,
+IF(RIGHT(B3,1)="M",1000000,
+IF(RIGHT(B3,1)="m",0.001,1))))</f>
         <v>33</v>
       </c>
       <c r="D3" s="16" t="s">
@@ -2579,7 +2623,12 @@
         <v>100</v>
       </c>
       <c r="C4" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B4),
+IF(B4=0,"",B4),
+VALUE(LEFT(B4,LEN(B4)-1))*
+IF(RIGHT(B4,1)="k",1000,
+IF(RIGHT(B4,1)="M",1000000,
+IF(RIGHT(B4,1)="m",0.001,1))))</f>
         <v>100</v>
       </c>
       <c r="D4" s="16" t="s">
@@ -2592,10 +2641,10 @@
         <v>199</v>
       </c>
       <c r="G4" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="H4" s="16" t="s">
         <v>243</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -2606,7 +2655,12 @@
         <v>220</v>
       </c>
       <c r="C5" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B5),
+IF(B5=0,"",B5),
+VALUE(LEFT(B5,LEN(B5)-1))*
+IF(RIGHT(B5,1)="k",1000,
+IF(RIGHT(B5,1)="M",1000000,
+IF(RIGHT(B5,1)="m",0.001,1))))</f>
         <v>220</v>
       </c>
       <c r="D5" s="16" t="s">
@@ -2633,7 +2687,12 @@
         <v>220</v>
       </c>
       <c r="C6" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B6),
+IF(B6=0,"",B6),
+VALUE(LEFT(B6,LEN(B6)-1))*
+IF(RIGHT(B6,1)="k",1000,
+IF(RIGHT(B6,1)="M",1000000,
+IF(RIGHT(B6,1)="m",0.001,1))))</f>
         <v>220</v>
       </c>
       <c r="D6" s="16" t="s">
@@ -2660,7 +2719,12 @@
         <v>61</v>
       </c>
       <c r="C7" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B7),
+IF(B7=0,"",B7),
+VALUE(LEFT(B7,LEN(B7)-1))*
+IF(RIGHT(B7,1)="k",1000,
+IF(RIGHT(B7,1)="M",1000000,
+IF(RIGHT(B7,1)="m",0.001,1))))</f>
         <v>1000</v>
       </c>
       <c r="D7" s="16" t="s">
@@ -2687,7 +2751,12 @@
         <v>61</v>
       </c>
       <c r="C8" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B8),
+IF(B8=0,"",B8),
+VALUE(LEFT(B8,LEN(B8)-1))*
+IF(RIGHT(B8,1)="k",1000,
+IF(RIGHT(B8,1)="M",1000000,
+IF(RIGHT(B8,1)="m",0.001,1))))</f>
         <v>1000</v>
       </c>
       <c r="D8" s="16" t="s">
@@ -2714,7 +2783,12 @@
         <v>70</v>
       </c>
       <c r="C9" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B9),
+IF(B9=0,"",B9),
+VALUE(LEFT(B9,LEN(B9)-1))*
+IF(RIGHT(B9,1)="k",1000,
+IF(RIGHT(B9,1)="M",1000000,
+IF(RIGHT(B9,1)="m",0.001,1))))</f>
         <v>2000</v>
       </c>
       <c r="D9" s="16" t="s">
@@ -2741,7 +2815,12 @@
         <v>53</v>
       </c>
       <c r="C10" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B10),
+IF(B10=0,"",B10),
+VALUE(LEFT(B10,LEN(B10)-1))*
+IF(RIGHT(B10,1)="k",1000,
+IF(RIGHT(B10,1)="M",1000000,
+IF(RIGHT(B10,1)="m",0.001,1))))</f>
         <v>5100</v>
       </c>
       <c r="D10" s="16" t="s">
@@ -2768,7 +2847,12 @@
         <v>139</v>
       </c>
       <c r="C11" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B11),
+IF(B11=0,"",B11),
+VALUE(LEFT(B11,LEN(B11)-1))*
+IF(RIGHT(B11,1)="k",1000,
+IF(RIGHT(B11,1)="M",1000000,
+IF(RIGHT(B11,1)="m",0.001,1))))</f>
         <v>10000</v>
       </c>
       <c r="D11" s="16" t="s">
@@ -2795,7 +2879,12 @@
         <v>139</v>
       </c>
       <c r="C12" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B12),
+IF(B12=0,"",B12),
+VALUE(LEFT(B12,LEN(B12)-1))*
+IF(RIGHT(B12,1)="k",1000,
+IF(RIGHT(B12,1)="M",1000000,
+IF(RIGHT(B12,1)="m",0.001,1))))</f>
         <v>10000</v>
       </c>
       <c r="D12" s="16" t="s">
@@ -2822,7 +2911,12 @@
         <v>144</v>
       </c>
       <c r="C13" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B13),
+IF(B13=0,"",B13),
+VALUE(LEFT(B13,LEN(B13)-1))*
+IF(RIGHT(B13,1)="k",1000,
+IF(RIGHT(B13,1)="M",1000000,
+IF(RIGHT(B13,1)="m",0.001,1))))</f>
         <v>52300</v>
       </c>
       <c r="D13" s="16" t="s">
@@ -2843,20 +2937,35 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="B14" s="15">
-        <v>0</v>
-      </c>
-      <c r="C14" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
+        <v>1</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>271</v>
+      </c>
+      <c r="C14" s="17">
+        <f>IF(ISNUMBER(B14),
+IF(B14=0,"",B14),
+VALUE(LEFT(B14,LEN(B14)-1))*
+IF(RIGHT(B14,1)="k",1000,
+IF(RIGHT(B14,1)="M",1000000,
+IF(RIGHT(B14,1)="m",0.001,1))))</f>
+        <v>100000</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>268</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>269</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>270</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="18" t="b">
@@ -2866,7 +2975,12 @@
         <v>0</v>
       </c>
       <c r="C15" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B15),
+IF(B15=0,"",B15),
+VALUE(LEFT(B15,LEN(B15)-1))*
+IF(RIGHT(B15,1)="k",1000,
+IF(RIGHT(B15,1)="M",1000000,
+IF(RIGHT(B15,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D15" s="16"/>
@@ -2883,7 +2997,12 @@
         <v>0</v>
       </c>
       <c r="C16" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B16),
+IF(B16=0,"",B16),
+VALUE(LEFT(B16,LEN(B16)-1))*
+IF(RIGHT(B16,1)="k",1000,
+IF(RIGHT(B16,1)="M",1000000,
+IF(RIGHT(B16,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D16" s="16"/>
@@ -2900,7 +3019,12 @@
         <v>0</v>
       </c>
       <c r="C17" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B17),
+IF(B17=0,"",B17),
+VALUE(LEFT(B17,LEN(B17)-1))*
+IF(RIGHT(B17,1)="k",1000,
+IF(RIGHT(B17,1)="M",1000000,
+IF(RIGHT(B17,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D17" s="16"/>
@@ -2917,7 +3041,12 @@
         <v>0</v>
       </c>
       <c r="C18" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B18),
+IF(B18=0,"",B18),
+VALUE(LEFT(B18,LEN(B18)-1))*
+IF(RIGHT(B18,1)="k",1000,
+IF(RIGHT(B18,1)="M",1000000,
+IF(RIGHT(B18,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D18" s="16"/>
@@ -2934,7 +3063,12 @@
         <v>0</v>
       </c>
       <c r="C19" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B19),
+IF(B19=0,"",B19),
+VALUE(LEFT(B19,LEN(B19)-1))*
+IF(RIGHT(B19,1)="k",1000,
+IF(RIGHT(B19,1)="M",1000000,
+IF(RIGHT(B19,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D19" s="16"/>
@@ -2951,7 +3085,12 @@
         <v>0</v>
       </c>
       <c r="C20" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B20),
+IF(B20=0,"",B20),
+VALUE(LEFT(B20,LEN(B20)-1))*
+IF(RIGHT(B20,1)="k",1000,
+IF(RIGHT(B20,1)="M",1000000,
+IF(RIGHT(B20,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D20" s="16"/>
@@ -2968,7 +3107,12 @@
         <v>0</v>
       </c>
       <c r="C21" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B21),
+IF(B21=0,"",B21),
+VALUE(LEFT(B21,LEN(B21)-1))*
+IF(RIGHT(B21,1)="k",1000,
+IF(RIGHT(B21,1)="M",1000000,
+IF(RIGHT(B21,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D21" s="16"/>
@@ -2985,7 +3129,12 @@
         <v>0</v>
       </c>
       <c r="C22" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B22),
+IF(B22=0,"",B22),
+VALUE(LEFT(B22,LEN(B22)-1))*
+IF(RIGHT(B22,1)="k",1000,
+IF(RIGHT(B22,1)="M",1000000,
+IF(RIGHT(B22,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D22" s="16"/>
@@ -3660,7 +3809,7 @@
         <v>153</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>157</v>
@@ -3703,7 +3852,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C3" s="12">
         <v>9</v>
@@ -3712,13 +3861,13 @@
         <v>158</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>246</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -4059,7 +4208,7 @@
         <v>96</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>97</v>
@@ -4392,7 +4541,8 @@
     <col min="4" max="4" width="15.7265625" customWidth="1"/>
     <col min="5" max="5" width="19.54296875" customWidth="1"/>
     <col min="6" max="6" width="31.54296875" customWidth="1"/>
-    <col min="7" max="8" width="8.7265625" hidden="1"/>
+    <col min="7" max="8" width="8.7265625" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="0" hidden="1" customWidth="1"/>
     <col min="10" max="16384" width="8.7265625" hidden="1"/>
   </cols>
   <sheetData>
@@ -4401,10 +4551,10 @@
         <v>203</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>87</v>
@@ -4421,16 +4571,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C2" t="s">
         <v>252</v>
       </c>
-      <c r="C2" t="s">
-        <v>253</v>
-      </c>
       <c r="D2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F2" t="s">
         <v>255</v>
-      </c>
-      <c r="F2" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -4438,19 +4588,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C3" t="s">
+        <v>257</v>
+      </c>
+      <c r="D3" t="s">
+        <v>256</v>
+      </c>
+      <c r="E3" t="s">
         <v>258</v>
       </c>
-      <c r="D3" t="s">
-        <v>257</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>259</v>
-      </c>
-      <c r="F3" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -4458,21 +4608,33 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D4" t="s">
+        <v>254</v>
+      </c>
+      <c r="F4" t="s">
         <v>261</v>
-      </c>
-      <c r="D4" t="s">
-        <v>255</v>
-      </c>
-      <c r="F4" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>262</v>
+      </c>
+      <c r="C5" t="s">
+        <v>263</v>
+      </c>
+      <c r="D5" t="s">
+        <v>262</v>
+      </c>
+      <c r="F5" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
added more new parts
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCCB022D-9FF7-4806-929F-E0FB4CC45DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5C6B81-9926-4547-920E-034227F104A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="13" activeTab="16" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="8" activeTab="10" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="373">
   <si>
     <t>Capacitance</t>
   </si>
@@ -1114,6 +1114,69 @@
   </si>
   <si>
     <t>White PC Test Point, Multipurpose Phosphor Bronze Silver Plating Through Hole Mounting Type</t>
+  </si>
+  <si>
+    <t>1000uF</t>
+  </si>
+  <si>
+    <t>35V</t>
+  </si>
+  <si>
+    <t>35PK1000MEFC10X20</t>
+  </si>
+  <si>
+    <t>TB002-500-05BE</t>
+  </si>
+  <si>
+    <t>5 Position Wire to Board Terminal Block Horizontal with Board 0.197" (5.00mm) Through Hole</t>
+  </si>
+  <si>
+    <t>TB002-500-04BE</t>
+  </si>
+  <si>
+    <t>4 Position Wire to Board Terminal Block Horizontal with Board 0.197" (5.00mm) Through Hole</t>
+  </si>
+  <si>
+    <t>TB002-500-06BE</t>
+  </si>
+  <si>
+    <t>6 Position Wire to Board Terminal Block Horizontal with Board 0.197" (5.00mm) Through Hole</t>
+  </si>
+  <si>
+    <t>TB002-500-10BE</t>
+  </si>
+  <si>
+    <t>10 Position Wire to Board Terminal Block Horizontal with Board 0.197" (5.00mm) Through Hole</t>
+  </si>
+  <si>
+    <t>3mm Diameter</t>
+  </si>
+  <si>
+    <t>151031VS06000</t>
+  </si>
+  <si>
+    <t>CFR-25JR-52-220R</t>
+  </si>
+  <si>
+    <t>220 Ohms ±5% 0.25W, 1/4W Through Hole Resistor Axial Automotive AEC-Q200 Carbon Film</t>
+  </si>
+  <si>
+    <t>Neopixel (Single)</t>
+  </si>
+  <si>
+    <t>LED</t>
+  </si>
+  <si>
+    <t>5x5mm</t>
+  </si>
+  <si>
+    <t>Clear</t>
+  </si>
+  <si>
+    <t>RGB</t>
+  </si>
+  <si>
+    <t>Addressable Lighting - LED Serial NRZ (Shift Register) Red, Green, Blue (RGB) 5.00mm L x 5.00mm W</t>
   </si>
 </sst>
 </file>
@@ -1249,15 +1312,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="68">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="69">
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1284,6 +1339,21 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1412,6 +1482,21 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -1419,22 +1504,11 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <extLst>
@@ -1557,11 +1631,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <extLst>
@@ -1614,13 +1684,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I26" totalsRowShown="0">
   <autoFilter ref="A1:I26" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="65"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="66"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="64"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="65"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="63"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="62"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="64"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="63"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -1629,13 +1699,14 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:G10" totalsRowShown="0">
-  <autoFilter ref="A1:G10" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
-  <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H10" totalsRowShown="0">
+  <autoFilter ref="A1:H10" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
+  <tableColumns count="8">
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="0"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="67"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -1645,10 +1716,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="31">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="30"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -1667,7 +1738,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="29"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -1677,37 +1748,37 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="25"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="20"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="19"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="23"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="22"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="21"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="20"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H22" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H22" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="A1:H22" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H22">
     <sortCondition ref="C1:C22"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="13"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="11">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="12">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -1715,11 +1786,11 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1729,7 +1800,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}" name="Switches" displayName="Switches" ref="A1:G11" totalsRowShown="0">
   <autoFilter ref="A1:G11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="6"/>
     <tableColumn id="1" xr3:uid="{C868B851-3D2D-4863-96B3-5412E9A862E1}" name="Function"/>
     <tableColumn id="6" xr3:uid="{D6EA3AC7-CEF9-4E2A-800B-297C8C002273}" name="Circuit"/>
     <tableColumn id="2" xr3:uid="{5048C5E7-258E-4EC2-B0BD-C338C4D84C91}" name="Part Number"/>
@@ -1742,10 +1813,10 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{C800FF98-41EA-493F-A089-14FECFF39D7A}" name="Test_Points" displayName="Test_Points" ref="A1:F11" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{C800FF98-41EA-493F-A089-14FECFF39D7A}" name="Test_Points" displayName="Test_Points" ref="A1:F11" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:F11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{5FA1F5D0-B5EA-4DAB-B07A-643BF29E8565}" name="Added to Altium?" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{5FA1F5D0-B5EA-4DAB-B07A-643BF29E8565}" name="Added to Altium?" dataDxfId="4"/>
     <tableColumn id="1" xr3:uid="{CC1FCF46-8E52-4166-BC69-286FE8778BAA}" name="Mounting Type"/>
     <tableColumn id="3" xr3:uid="{25F97020-E67A-4F9F-99D3-71374E9FAEC5}" name="# of pads/points"/>
     <tableColumn id="6" xr3:uid="{6395E911-E7EB-4DC7-B232-C23AAD6F19AF}" name="Series"/>
@@ -1757,10 +1828,10 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{261C41B4-4EE2-4BF0-B2F3-2F2A51D3792A}" name="Transistors" displayName="Transistors" ref="A1:H11" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{261C41B4-4EE2-4BF0-B2F3-2F2A51D3792A}" name="Transistors" displayName="Transistors" ref="A1:H11" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:H11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{3A0D6614-B80A-4184-9ADE-5206B38A06E5}" name="Added to Altium?" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{3A0D6614-B80A-4184-9ADE-5206B38A06E5}" name="Added to Altium?" dataDxfId="2"/>
     <tableColumn id="1" xr3:uid="{05D09AC3-5445-495F-8B8E-1C98473F2758}" name="Technology"/>
     <tableColumn id="6" xr3:uid="{F919A207-76D0-435F-BB24-020D391F6DB9}" name="Configuration"/>
     <tableColumn id="8" xr3:uid="{4CC17C6A-1F84-408C-8AAD-69C3E5F234CA}" name="Max Voltage"/>
@@ -1777,7 +1848,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{82CFED5E-627B-4A23-9BFA-C489CEA32F25}" name="Voltage_Regulators" displayName="Voltage_Regulators" ref="A1:H12" totalsRowShown="0">
   <autoFilter ref="A1:H12" xr:uid="{82CFED5E-627B-4A23-9BFA-C489CEA32F25}"/>
   <tableColumns count="8">
-    <tableColumn id="3" xr3:uid="{DD7A1A9A-DE5A-4766-9947-A308E87BA7FD}" name="Added to Altium?" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{DD7A1A9A-DE5A-4766-9947-A308E87BA7FD}" name="Added to Altium?" dataDxfId="1"/>
     <tableColumn id="1" xr3:uid="{7B7659A2-8D22-4954-B10E-C811D8D29B99}" name="Type"/>
     <tableColumn id="7" xr3:uid="{24DD5DAD-1853-4138-AB66-BA5667E60D26}" name="Operation"/>
     <tableColumn id="8" xr3:uid="{C0E1C407-BC33-4018-B09E-15A16329D7C6}" name="Input Voltage"/>
@@ -1791,20 +1862,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H30" totalsRowShown="0" headerRowDxfId="61">
-  <autoFilter ref="A1:H30" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H30">
-    <sortCondition ref="B1:B30"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H31" totalsRowShown="0" headerRowDxfId="62">
+  <autoFilter ref="A1:H31" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H31">
+    <sortCondition ref="B1:B31"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="60"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="59"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="56"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="55"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="54"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="53"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="61"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="59"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="58"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="57"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="56"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="55"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1827,10 +1898,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G7" totalsRowShown="0" headerRowDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G7" totalsRowShown="0" headerRowDxfId="53">
   <autoFilter ref="A1:G7" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="52"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -1843,11 +1914,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Diodes3" displayName="Diodes3" ref="A1:F7" totalsRowShown="0" headerRowDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Diodes3" displayName="Diodes3" ref="A1:F7" totalsRowShown="0" headerRowDxfId="51">
   <autoFilter ref="A1:F7" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="49"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="48"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="49"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -1858,25 +1929,25 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="48">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="46"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="42">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="40"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="41"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="40"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -1893,8 +1964,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}" name="ICs" displayName="ICs" ref="A1:E10" totalsRowShown="0">
   <autoFilter ref="A1:E10" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}"/>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="67"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="66"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="38"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -1904,14 +1975,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="37">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="37"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="36"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2452,143 +2523,197 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9362198B-44BD-4E55-B62E-439143EC0CFE}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="8.7265625" customWidth="1"/>
-    <col min="3" max="3" width="16.36328125" customWidth="1"/>
-    <col min="4" max="4" width="14.36328125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="17.453125" customWidth="1"/>
-    <col min="6" max="6" width="31.81640625" customWidth="1"/>
-    <col min="7" max="7" width="43.26953125" customWidth="1"/>
-    <col min="8" max="16384" width="8.7265625" hidden="1"/>
+    <col min="1" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" customWidth="1"/>
+    <col min="5" max="5" width="14.36328125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="17.453125" customWidth="1"/>
+    <col min="7" max="7" width="31.81640625" customWidth="1"/>
+    <col min="8" max="8" width="43.26953125" customWidth="1"/>
+    <col min="9" max="16384" width="8.7265625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>203</v>
       </c>
       <c r="B1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" t="s">
         <v>20</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>198</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>22</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>368</v>
+      </c>
+      <c r="C2" t="s">
         <v>21</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>107</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>23</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>368</v>
+      </c>
+      <c r="C3" t="s">
         <v>26</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>23</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B4" t="s">
+        <v>368</v>
+      </c>
+      <c r="C4" t="s">
         <v>28</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>23</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>368</v>
+      </c>
+      <c r="C5" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>107</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>23</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>368</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" t="s">
+        <v>129</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="F6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>367</v>
+      </c>
+      <c r="C7" t="s">
+        <v>371</v>
+      </c>
+      <c r="D7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="F7" t="s">
+        <v>370</v>
+      </c>
+      <c r="G7">
+        <v>16347</v>
+      </c>
+      <c r="H7" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="b">
         <v>0</v>
       </c>
@@ -3042,7 +3167,7 @@
         <v>27</v>
       </c>
       <c r="C2" s="17">
-        <f t="shared" ref="C2:C22" si="0">IF(ISNUMBER(B2),
+        <f>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
 IF(RIGHT(B2,1)="k",1000,
@@ -3074,7 +3199,12 @@
         <v>33</v>
       </c>
       <c r="C3" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B3),
+IF(B3=0,"",B3),
+VALUE(LEFT(B3,LEN(B3)-1))*
+IF(RIGHT(B3,1)="k",1000,
+IF(RIGHT(B3,1)="M",1000000,
+IF(RIGHT(B3,1)="m",0.001,1))))</f>
         <v>33</v>
       </c>
       <c r="D3" s="16" t="s">
@@ -3101,7 +3231,12 @@
         <v>100</v>
       </c>
       <c r="C4" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B4),
+IF(B4=0,"",B4),
+VALUE(LEFT(B4,LEN(B4)-1))*
+IF(RIGHT(B4,1)="k",1000,
+IF(RIGHT(B4,1)="M",1000000,
+IF(RIGHT(B4,1)="m",0.001,1))))</f>
         <v>100</v>
       </c>
       <c r="D4" s="16" t="s">
@@ -3128,7 +3263,12 @@
         <v>220</v>
       </c>
       <c r="C5" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B5),
+IF(B5=0,"",B5),
+VALUE(LEFT(B5,LEN(B5)-1))*
+IF(RIGHT(B5,1)="k",1000,
+IF(RIGHT(B5,1)="M",1000000,
+IF(RIGHT(B5,1)="m",0.001,1))))</f>
         <v>220</v>
       </c>
       <c r="D5" s="16" t="s">
@@ -3155,7 +3295,12 @@
         <v>220</v>
       </c>
       <c r="C6" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B6),
+IF(B6=0,"",B6),
+VALUE(LEFT(B6,LEN(B6)-1))*
+IF(RIGHT(B6,1)="k",1000,
+IF(RIGHT(B6,1)="M",1000000,
+IF(RIGHT(B6,1)="m",0.001,1))))</f>
         <v>220</v>
       </c>
       <c r="D6" s="16" t="s">
@@ -3178,27 +3323,32 @@
       <c r="A7" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>61</v>
+      <c r="B7" s="15">
+        <v>220</v>
       </c>
       <c r="C7" s="17">
-        <f t="shared" si="0"/>
-        <v>1000</v>
+        <f>IF(ISNUMBER(B7),
+IF(B7=0,"",B7),
+VALUE(LEFT(B7,LEN(B7)-1))*
+IF(RIGHT(B7,1)="k",1000,
+IF(RIGHT(B7,1)="M",1000000,
+IF(RIGHT(B7,1)="m",0.001,1))))</f>
+        <v>220</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>54</v>
+        <v>140</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>9</v>
+        <v>129</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>199</v>
+        <v>268</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>59</v>
+        <v>365</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>60</v>
+        <v>366</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -3209,23 +3359,28 @@
         <v>61</v>
       </c>
       <c r="C8" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B8),
+IF(B8=0,"",B8),
+VALUE(LEFT(B8,LEN(B8)-1))*
+IF(RIGHT(B8,1)="k",1000,
+IF(RIGHT(B8,1)="M",1000000,
+IF(RIGHT(B8,1)="m",0.001,1))))</f>
         <v>1000</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F8" s="16" t="s">
         <v>199</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>134</v>
+        <v>59</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>135</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -3233,26 +3388,31 @@
         <v>1</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C9" s="17">
-        <f t="shared" si="0"/>
-        <v>2000</v>
+        <f>IF(ISNUMBER(B9),
+IF(B9=0,"",B9),
+VALUE(LEFT(B9,LEN(B9)-1))*
+IF(RIGHT(B9,1)="k",1000,
+IF(RIGHT(B9,1)="M",1000000,
+IF(RIGHT(B9,1)="m",0.001,1))))</f>
+        <v>1000</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F9" s="16" t="s">
         <v>199</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>68</v>
+        <v>134</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>69</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -3260,14 +3420,19 @@
         <v>1</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="C10" s="17">
-        <f t="shared" si="0"/>
-        <v>5100</v>
+        <f>IF(ISNUMBER(B10),
+IF(B10=0,"",B10),
+VALUE(LEFT(B10,LEN(B10)-1))*
+IF(RIGHT(B10,1)="k",1000,
+IF(RIGHT(B10,1)="M",1000000,
+IF(RIGHT(B10,1)="m",0.001,1))))</f>
+        <v>2000</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="E10" s="16" t="s">
         <v>9</v>
@@ -3276,10 +3441,10 @@
         <v>199</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
@@ -3287,26 +3452,31 @@
         <v>1</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>139</v>
+        <v>53</v>
       </c>
       <c r="C11" s="17">
-        <f t="shared" si="0"/>
-        <v>10000</v>
+        <f>IF(ISNUMBER(B11),
+IF(B11=0,"",B11),
+VALUE(LEFT(B11,LEN(B11)-1))*
+IF(RIGHT(B11,1)="k",1000,
+IF(RIGHT(B11,1)="M",1000000,
+IF(RIGHT(B11,1)="m",0.001,1))))</f>
+        <v>5100</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>140</v>
+        <v>54</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>141</v>
+        <v>199</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>142</v>
+        <v>55</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>143</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -3317,23 +3487,28 @@
         <v>139</v>
       </c>
       <c r="C12" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B12),
+IF(B12=0,"",B12),
+VALUE(LEFT(B12,LEN(B12)-1))*
+IF(RIGHT(B12,1)="k",1000,
+IF(RIGHT(B12,1)="M",1000000,
+IF(RIGHT(B12,1)="m",0.001,1))))</f>
         <v>10000</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>54</v>
+        <v>140</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>199</v>
+        <v>141</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>168</v>
+        <v>142</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -3341,11 +3516,16 @@
         <v>1</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>333</v>
+        <v>139</v>
       </c>
       <c r="C13" s="17">
-        <f t="shared" si="0"/>
-        <v>47000</v>
+        <f>IF(ISNUMBER(B13),
+IF(B13=0,"",B13),
+VALUE(LEFT(B13,LEN(B13)-1))*
+IF(RIGHT(B13,1)="k",1000,
+IF(RIGHT(B13,1)="M",1000000,
+IF(RIGHT(B13,1)="m",0.001,1))))</f>
+        <v>10000</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>54</v>
@@ -3357,10 +3537,10 @@
         <v>199</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>334</v>
+        <v>168</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>335</v>
+        <v>167</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
@@ -3368,26 +3548,31 @@
         <v>1</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>144</v>
+        <v>333</v>
       </c>
       <c r="C14" s="17">
-        <f t="shared" si="0"/>
-        <v>52300</v>
+        <f>IF(ISNUMBER(B14),
+IF(B14=0,"",B14),
+VALUE(LEFT(B14,LEN(B14)-1))*
+IF(RIGHT(B14,1)="k",1000,
+IF(RIGHT(B14,1)="M",1000000,
+IF(RIGHT(B14,1)="m",0.001,1))))</f>
+        <v>47000</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>54</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>141</v>
+        <v>199</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>145</v>
+        <v>334</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>146</v>
+        <v>335</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -3395,26 +3580,31 @@
         <v>1</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>271</v>
+        <v>144</v>
       </c>
       <c r="C15" s="17">
-        <f t="shared" si="0"/>
-        <v>100000</v>
+        <f>IF(ISNUMBER(B15),
+IF(B15=0,"",B15),
+VALUE(LEFT(B15,LEN(B15)-1))*
+IF(RIGHT(B15,1)="k",1000,
+IF(RIGHT(B15,1)="M",1000000,
+IF(RIGHT(B15,1)="m",0.001,1))))</f>
+        <v>52300</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>54</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>129</v>
+        <v>25</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>268</v>
+        <v>141</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>269</v>
+        <v>145</v>
       </c>
       <c r="H15" s="16" t="s">
-        <v>270</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -3422,26 +3612,31 @@
         <v>1</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>295</v>
+        <v>271</v>
       </c>
       <c r="C16" s="17">
-        <f t="shared" si="0"/>
-        <v>680000</v>
+        <f>IF(ISNUMBER(B16),
+IF(B16=0,"",B16),
+VALUE(LEFT(B16,LEN(B16)-1))*
+IF(RIGHT(B16,1)="k",1000,
+IF(RIGHT(B16,1)="M",1000000,
+IF(RIGHT(B16,1)="m",0.001,1))))</f>
+        <v>100000</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>140</v>
+        <v>54</v>
       </c>
       <c r="E16" s="16" t="s">
         <v>129</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>293</v>
+        <v>268</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>296</v>
+        <v>269</v>
       </c>
       <c r="H16" s="16" t="s">
-        <v>298</v>
+        <v>270</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -3449,11 +3644,16 @@
         <v>1</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C17" s="17">
-        <f t="shared" si="0"/>
-        <v>1000000</v>
+        <f>IF(ISNUMBER(B17),
+IF(B17=0,"",B17),
+VALUE(LEFT(B17,LEN(B17)-1))*
+IF(RIGHT(B17,1)="k",1000,
+IF(RIGHT(B17,1)="M",1000000,
+IF(RIGHT(B17,1)="m",0.001,1))))</f>
+        <v>680000</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>140</v>
@@ -3465,10 +3665,10 @@
         <v>293</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="H17" s="16" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
@@ -3479,41 +3679,61 @@
         <v>292</v>
       </c>
       <c r="C18" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B18),
+IF(B18=0,"",B18),
+VALUE(LEFT(B18,LEN(B18)-1))*
+IF(RIGHT(B18,1)="k",1000,
+IF(RIGHT(B18,1)="M",1000000,
+IF(RIGHT(B18,1)="m",0.001,1))))</f>
         <v>1000000</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>54</v>
+        <v>140</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>9</v>
+        <v>129</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>199</v>
+        <v>293</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>327</v>
+        <v>294</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>328</v>
+        <v>297</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="B19" s="15">
-        <v>0</v>
-      </c>
-      <c r="C19" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
+        <v>1</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>292</v>
+      </c>
+      <c r="C19" s="17">
+        <f>IF(ISNUMBER(B19),
+IF(B19=0,"",B19),
+VALUE(LEFT(B19,LEN(B19)-1))*
+IF(RIGHT(B19,1)="k",1000,
+IF(RIGHT(B19,1)="M",1000000,
+IF(RIGHT(B19,1)="m",0.001,1))))</f>
+        <v>1000000</v>
+      </c>
+      <c r="D19" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="G19" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="H19" s="16" t="s">
+        <v>328</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="18" t="b">
@@ -3523,7 +3743,12 @@
         <v>0</v>
       </c>
       <c r="C20" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B20),
+IF(B20=0,"",B20),
+VALUE(LEFT(B20,LEN(B20)-1))*
+IF(RIGHT(B20,1)="k",1000,
+IF(RIGHT(B20,1)="M",1000000,
+IF(RIGHT(B20,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D20" s="16"/>
@@ -3540,7 +3765,12 @@
         <v>0</v>
       </c>
       <c r="C21" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B21),
+IF(B21=0,"",B21),
+VALUE(LEFT(B21,LEN(B21)-1))*
+IF(RIGHT(B21,1)="k",1000,
+IF(RIGHT(B21,1)="M",1000000,
+IF(RIGHT(B21,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D21" s="16"/>
@@ -3557,7 +3787,12 @@
         <v>0</v>
       </c>
       <c r="C22" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B22),
+IF(B22=0,"",B22),
+VALUE(LEFT(B22,LEN(B22)-1))*
+IF(RIGHT(B22,1)="k",1000,
+IF(RIGHT(B22,1)="M",1000000,
+IF(RIGHT(B22,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D22" s="16"/>
@@ -3717,6 +3952,7 @@
     <col min="4" max="4" width="13.81640625" customWidth="1"/>
     <col min="5" max="5" width="19.26953125" customWidth="1"/>
     <col min="6" max="6" width="41.81640625" customWidth="1"/>
+    <col min="7" max="8" width="0" hidden="1" customWidth="1"/>
     <col min="9" max="16384" width="8.7265625" hidden="1"/>
   </cols>
   <sheetData>
@@ -4430,7 +4666,31 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B12" t="s">
+        <v>352</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D12" t="s">
+        <v>353</v>
+      </c>
+      <c r="E12" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="H12" t="s">
+        <v>116</v>
+      </c>
+      <c r="I12" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
@@ -4514,7 +4774,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31311A32-7C4D-4571-8105-957397FF3475}">
-  <dimension ref="A1:XDX30"/>
+  <dimension ref="A1:XDX31"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.1796875" style="3" customWidth="1"/>
@@ -4923,6 +5183,12 @@
       <c r="D22" s="3" t="s">
         <v>338</v>
       </c>
+      <c r="E22" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="b">
@@ -4932,11 +5198,17 @@
         <v>154</v>
       </c>
       <c r="C23" s="12">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>338</v>
       </c>
+      <c r="E23" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>356</v>
+      </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="b">
@@ -4946,33 +5218,36 @@
         <v>154</v>
       </c>
       <c r="C24" s="12">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>338</v>
       </c>
+      <c r="E24" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>360</v>
+      </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="10" t="b">
         <v>1</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>272</v>
+        <v>154</v>
       </c>
       <c r="C25" s="12">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>338</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>340</v>
+        <v>361</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>274</v>
+        <v>362</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
@@ -4980,20 +5255,22 @@
         <v>1</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="C26" s="12"/>
+        <v>272</v>
+      </c>
+      <c r="C26" s="12">
+        <v>4</v>
+      </c>
       <c r="D26" s="3" t="s">
         <v>338</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>96</v>
+        <v>273</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>249</v>
+        <v>340</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>97</v>
+        <v>274</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
@@ -5001,22 +5278,20 @@
         <v>1</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="C27" s="12">
-        <v>4</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="C27" s="12"/>
       <c r="D27" s="3" t="s">
         <v>338</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>339</v>
+        <v>96</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>340</v>
+        <v>249</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>341</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
@@ -5024,35 +5299,58 @@
         <v>1</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="C28" s="12">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>338</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>340</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C29" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="C29" s="12">
+        <v>8</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>344</v>
+      </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C30" s="12"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C31" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
moved over some reference designs
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64EC9B8D-22F5-4C63-BB5A-9326518A4DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73EDB4D6-2521-4D8F-86F3-7EE1239D5DD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1910" windowWidth="12090" windowHeight="8170" firstSheet="14" activeTab="14" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="2" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="456">
   <si>
     <t>Capacitance</t>
   </si>
@@ -1396,6 +1396,36 @@
   </si>
   <si>
     <t>15 kOhms ±1% 0.125W, 1/8W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
+    <t>CRCW0603680RFKEA</t>
+  </si>
+  <si>
+    <t>680 Ohms ±1% 0.125W, 1/8W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
+    <t>302-S161</t>
+  </si>
+  <si>
+    <t>Mezzanine</t>
+  </si>
+  <si>
+    <t>DF40C-12DP-0.4V(51)</t>
+  </si>
+  <si>
+    <t>Pitch = 0.40mm</t>
+  </si>
+  <si>
+    <t>12 Position Connector Receptacle, Center Strip Contacts Surface Mount Gold</t>
+  </si>
+  <si>
+    <t>12 Position Connector Plug, Outer Shroud Contacts Surface Mount Gold</t>
+  </si>
+  <si>
+    <t>Height = 2.0mm Pitch = 0.40mm</t>
+  </si>
+  <si>
+    <t>DF40B(2.0)-12DS-0.4V(51)</t>
   </si>
 </sst>
 </file>
@@ -1787,12 +1817,45 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="1"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -1825,39 +1888,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1903,13 +1933,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I26" totalsRowShown="0">
   <autoFilter ref="A1:I26" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="65"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="59"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="64"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="58"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="63"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="62"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="57"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="56"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -2081,20 +2111,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="68">
   <autoFilter ref="A1:H50" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H31">
     <sortCondition ref="B1:B31"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="60"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="59"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="56"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="55"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="54"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="53"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="67"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="66"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="65"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="63"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="62"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="61"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="60"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2117,10 +2147,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G7" totalsRowShown="0" headerRowDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G7" totalsRowShown="0" headerRowDxfId="55">
   <autoFilter ref="A1:G7" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="54"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -2133,11 +2163,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="68">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="53">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="66"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="52"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="51"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -4045,7 +4075,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>443</v>
@@ -4072,20 +4102,30 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B25" s="15">
-        <v>0</v>
-      </c>
-      <c r="C25" s="17" t="str">
+        <v>680</v>
+      </c>
+      <c r="C25" s="17">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
+        <v>680</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="E25" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="G25" s="16" t="s">
+        <v>446</v>
+      </c>
+      <c r="H25" s="16" t="s">
+        <v>447</v>
+      </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="18" t="b">
@@ -6341,97 +6381,148 @@
         <v>424</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C33" s="12"/>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="C33" s="12">
+        <v>16</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="C34" s="12"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B34" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="C34" s="12">
+        <v>12</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="C35" s="12"/>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B35" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="C35" s="12">
+        <v>12</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C36" s="12"/>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C37" s="12"/>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C38" s="12"/>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C39" s="12"/>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C40" s="12"/>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C41" s="12"/>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C42" s="12"/>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C43" s="12"/>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C44" s="12"/>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C45" s="12"/>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C46" s="12"/>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C47" s="12"/>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="10" t="b">
         <v>0</v>
       </c>
@@ -6451,8 +6542,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Added new parts, created "Mounts, Pads, Vias" library
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73EDB4D6-2521-4D8F-86F3-7EE1239D5DD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2D90D2E-583E-4A93-BD6C-E91571F84E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="2" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-28920" yWindow="5700" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="13" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -26,12 +26,13 @@
     <sheet name="LEDs" sheetId="5" r:id="rId11"/>
     <sheet name="Memory" sheetId="17" r:id="rId12"/>
     <sheet name="Misc Components" sheetId="14" r:id="rId13"/>
-    <sheet name="MCUs" sheetId="6" r:id="rId14"/>
-    <sheet name="Resistors" sheetId="2" r:id="rId15"/>
-    <sheet name="Switches" sheetId="11" r:id="rId16"/>
-    <sheet name="Test Points" sheetId="19" r:id="rId17"/>
-    <sheet name="Transistors" sheetId="18" r:id="rId18"/>
-    <sheet name="Voltage Regulators" sheetId="4" r:id="rId19"/>
+    <sheet name="Mounts, Pads, Vias" sheetId="20" r:id="rId14"/>
+    <sheet name="MCUs" sheetId="6" r:id="rId15"/>
+    <sheet name="Resistors" sheetId="2" r:id="rId16"/>
+    <sheet name="Switches" sheetId="11" r:id="rId17"/>
+    <sheet name="Test Points" sheetId="19" r:id="rId18"/>
+    <sheet name="Transistors" sheetId="18" r:id="rId19"/>
+    <sheet name="Voltage Regulators" sheetId="4" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Capacitors'!$B$1:$I$9</definedName>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="502">
   <si>
     <t>Capacitance</t>
   </si>
@@ -1426,6 +1427,144 @@
   </si>
   <si>
     <t>DF40B(2.0)-12DS-0.4V(51)</t>
+  </si>
+  <si>
+    <t>1kbit</t>
+  </si>
+  <si>
+    <t>128 x 8/64 x 16</t>
+  </si>
+  <si>
+    <t>3-Wire</t>
+  </si>
+  <si>
+    <t>FLASH</t>
+  </si>
+  <si>
+    <t>M93C46-WMN6TP</t>
+  </si>
+  <si>
+    <t>EEPROM Memory IC 1Kbit Microwire 2 MHz 8-SOIC</t>
+  </si>
+  <si>
+    <t>22pF</t>
+  </si>
+  <si>
+    <t>CC0603JRNPO9BN220</t>
+  </si>
+  <si>
+    <t>1.5k</t>
+  </si>
+  <si>
+    <t>CR0603-FX-1501ELF</t>
+  </si>
+  <si>
+    <t>1.5 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Moisture Resistant Thick Film</t>
+  </si>
+  <si>
+    <t>DF40HC(3.5)-20DS-0.4V(51)</t>
+  </si>
+  <si>
+    <t>DF40C-20DP-0.4V(51)</t>
+  </si>
+  <si>
+    <t>Height = 3.5mm</t>
+  </si>
+  <si>
+    <t>SOD-123</t>
+  </si>
+  <si>
+    <t>B5819W-TP</t>
+  </si>
+  <si>
+    <t>Diode 40 V 1A Surface Mount SOD-123</t>
+  </si>
+  <si>
+    <t>Zener</t>
+  </si>
+  <si>
+    <t>5.6V</t>
+  </si>
+  <si>
+    <t>N/A, rated for 1W</t>
+  </si>
+  <si>
+    <t>DO-214AC</t>
+  </si>
+  <si>
+    <t>SMAZ5V6-13-F</t>
+  </si>
+  <si>
+    <t>Zener Diode 5.6 V 1 W ±5% Surface Mount SMA</t>
+  </si>
+  <si>
+    <t>Optocoupler</t>
+  </si>
+  <si>
+    <t>4N26S</t>
+  </si>
+  <si>
+    <t>Optoisolator Transistor with Base Output 1500Vrms 1 Channel 6-SMD</t>
+  </si>
+  <si>
+    <t>DF40C-30DP-0.4V(51)</t>
+  </si>
+  <si>
+    <t>DF40HC(3.5)-30DS-0.4V(51)</t>
+  </si>
+  <si>
+    <t>30 Position Connector Receptacle, Center Strip Contacts Surface Mount Gold</t>
+  </si>
+  <si>
+    <t>30 Position Connector Plug, Outer Shroud Contacts Surface Mount Gold</t>
+  </si>
+  <si>
+    <t>USB-B Mini</t>
+  </si>
+  <si>
+    <t>MUSB-05-S-B-SM-A-K-TR</t>
+  </si>
+  <si>
+    <t>USB - mini B USB 2.0 Receptacle Connector 5 Position Surface Mount, Right Angle</t>
+  </si>
+  <si>
+    <t>Via</t>
+  </si>
+  <si>
+    <t>Signal Via</t>
+  </si>
+  <si>
+    <t>Shape</t>
+  </si>
+  <si>
+    <t>Round</t>
+  </si>
+  <si>
+    <t>Hole Size (diameter)</t>
+  </si>
+  <si>
+    <t>3.5mm</t>
+  </si>
+  <si>
+    <t>Copper X-Size</t>
+  </si>
+  <si>
+    <t>Copper Y-Size</t>
+  </si>
+  <si>
+    <t>6mm</t>
+  </si>
+  <si>
+    <t>0.3mm</t>
+  </si>
+  <si>
+    <t>0.7mm</t>
+  </si>
+  <si>
+    <t>Thru-hole via for signal connection.</t>
+  </si>
+  <si>
+    <t>Use for board mounting points. Place 4.5mm from board edges.</t>
   </si>
 </sst>
 </file>
@@ -1491,7 +1630,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1557,12 +1696,26 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="69">
+  <dxfs count="78">
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -1570,9 +1723,31 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
@@ -1587,7 +1762,7 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
@@ -1602,7 +1777,7 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
@@ -1688,7 +1863,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
@@ -1701,14 +1876,14 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
@@ -1726,14 +1901,14 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
@@ -1758,28 +1933,14 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
@@ -1807,7 +1968,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
@@ -1817,14 +1978,14 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="2"/>
         </ext>
       </extLst>
     </dxf>
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
@@ -1834,28 +1995,12 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -1882,12 +2027,42 @@
       <numFmt numFmtId="30" formatCode="@"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="1"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="1"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="1"/>
+        </ext>
+      </extLst>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1920,10 +2095,15 @@
   <bag type="XFComplement">
     <bagId k="XFControls">4</bagId>
   </bag>
+  <bag type="XFControls"/>
+  <bag type="XFComplement">
+    <bagId k="XFControls">6</bagId>
+  </bag>
   <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
     <a k="MappedFeaturePropertyBags">
+      <bagId>5</bagId>
       <bagId>2</bagId>
-      <bagId>5</bagId>
+      <bagId>7</bagId>
     </a>
   </bag>
 </FeaturePropertyBags>
@@ -1933,13 +2113,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I26" totalsRowShown="0">
   <autoFilter ref="A1:I26" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="59"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="75"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="58"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="74"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="57"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="73"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="72"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -1951,11 +2131,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H10" totalsRowShown="0">
   <autoFilter ref="A1:H10" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="33"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="32"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="42"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="41"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="40"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -1965,10 +2145,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="39">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="38"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -1987,7 +2167,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="37"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -1997,37 +2177,54 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:H11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
+  <tableColumns count="8">
+    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="4"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="25"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="20"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="19"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="31"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="29"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="28"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="A1:H50" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="C1:C50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="13"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="11">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="20">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -2035,21 +2232,21 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}" name="Switches" displayName="Switches" ref="A1:G11" totalsRowShown="0">
   <autoFilter ref="A1:G11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="14"/>
     <tableColumn id="1" xr3:uid="{C868B851-3D2D-4863-96B3-5412E9A862E1}" name="Function"/>
     <tableColumn id="6" xr3:uid="{D6EA3AC7-CEF9-4E2A-800B-297C8C002273}" name="Circuit"/>
     <tableColumn id="2" xr3:uid="{5048C5E7-258E-4EC2-B0BD-C338C4D84C91}" name="Part Number"/>
@@ -2061,11 +2258,11 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{C800FF98-41EA-493F-A089-14FECFF39D7A}" name="Test_Points" displayName="Test_Points" ref="A1:F11" totalsRowShown="0" headerRowDxfId="4">
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{C800FF98-41EA-493F-A089-14FECFF39D7A}" name="Test_Points" displayName="Test_Points" ref="A1:F11" totalsRowShown="0" headerRowDxfId="13">
   <autoFilter ref="A1:F11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{5FA1F5D0-B5EA-4DAB-B07A-643BF29E8565}" name="Added to Altium?" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{5FA1F5D0-B5EA-4DAB-B07A-643BF29E8565}" name="Added to Altium?" dataDxfId="12"/>
     <tableColumn id="1" xr3:uid="{CC1FCF46-8E52-4166-BC69-286FE8778BAA}" name="Mounting Type"/>
     <tableColumn id="3" xr3:uid="{25F97020-E67A-4F9F-99D3-71374E9FAEC5}" name="# of pads/points"/>
     <tableColumn id="6" xr3:uid="{6395E911-E7EB-4DC7-B232-C23AAD6F19AF}" name="Series"/>
@@ -2076,11 +2273,11 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{261C41B4-4EE2-4BF0-B2F3-2F2A51D3792A}" name="Transistors" displayName="Transistors" ref="A1:H11" totalsRowShown="0" headerRowDxfId="2">
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{261C41B4-4EE2-4BF0-B2F3-2F2A51D3792A}" name="Transistors" displayName="Transistors" ref="A1:H11" totalsRowShown="0" headerRowDxfId="11">
   <autoFilter ref="A1:H11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{3A0D6614-B80A-4184-9ADE-5206B38A06E5}" name="Added to Altium?" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{3A0D6614-B80A-4184-9ADE-5206B38A06E5}" name="Added to Altium?" dataDxfId="10"/>
     <tableColumn id="1" xr3:uid="{05D09AC3-5445-495F-8B8E-1C98473F2758}" name="Technology"/>
     <tableColumn id="6" xr3:uid="{F919A207-76D0-435F-BB24-020D391F6DB9}" name="Configuration"/>
     <tableColumn id="8" xr3:uid="{4CC17C6A-1F84-408C-8AAD-69C3E5F234CA}" name="Max Voltage"/>
@@ -2093,11 +2290,11 @@
 </table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{82CFED5E-627B-4A23-9BFA-C489CEA32F25}" name="Voltage_Regulators" displayName="Voltage_Regulators" ref="A1:H12" totalsRowShown="0">
   <autoFilter ref="A1:H12" xr:uid="{82CFED5E-627B-4A23-9BFA-C489CEA32F25}"/>
   <tableColumns count="8">
-    <tableColumn id="3" xr3:uid="{DD7A1A9A-DE5A-4766-9947-A308E87BA7FD}" name="Added to Altium?" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{DD7A1A9A-DE5A-4766-9947-A308E87BA7FD}" name="Added to Altium?" dataDxfId="9"/>
     <tableColumn id="1" xr3:uid="{7B7659A2-8D22-4954-B10E-C811D8D29B99}" name="Type"/>
     <tableColumn id="7" xr3:uid="{24DD5DAD-1853-4138-AB66-BA5667E60D26}" name="Operation"/>
     <tableColumn id="8" xr3:uid="{C0E1C407-BC33-4018-B09E-15A16329D7C6}" name="Input Voltage"/>
@@ -2111,20 +2308,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="68">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="71">
   <autoFilter ref="A1:H50" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H31">
     <sortCondition ref="B1:B31"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="67"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="66"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="65"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="63"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="62"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="61"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="60"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="70"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="68"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2147,10 +2344,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G7" totalsRowShown="0" headerRowDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G7" totalsRowShown="0" headerRowDxfId="62">
   <autoFilter ref="A1:G7" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="61"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -2163,11 +2360,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="53">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="60">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="52"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="59"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="58"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -2178,25 +2375,25 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="57">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="49"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="56"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="54"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="44">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="51">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="42"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="49"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -2216,8 +2413,8 @@
     <sortCondition ref="B1:B10"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="41"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="77"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="76"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -2227,14 +2424,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="48">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="38"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="37"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3092,12 +3289,26 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>458</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="F3" t="s">
+        <v>460</v>
+      </c>
+      <c r="G3" t="s">
+        <v>461</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="b">
@@ -3136,8 +3347,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3282,6 +3494,147 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22B86CF3-50F4-4B19-99AD-AF8E53CE9DBA}">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="15.54296875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="21.1796875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.6328125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="20.6328125" style="3" customWidth="1"/>
+    <col min="6" max="7" width="15.6328125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="45.81640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="0" style="3" hidden="1"/>
+    <col min="10" max="16384" width="8.7265625" style="3" hidden="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="23" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="23" t="s">
+        <v>201</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>491</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>493</v>
+      </c>
+      <c r="F1" s="23" t="s">
+        <v>495</v>
+      </c>
+      <c r="G1" s="23" t="s">
+        <v>496</v>
+      </c>
+      <c r="H1" s="23" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF58675A-C2E2-4804-A061-74EF114D288F}">
   <dimension ref="A1:J11"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
@@ -3432,7 +3785,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B73385E-A93D-4809-A6CB-D5FDE97D6171}">
   <dimension ref="A1:H50"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
@@ -4129,20 +4482,30 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="B26" s="15">
-        <v>0</v>
-      </c>
-      <c r="C26" s="17" t="str">
+        <v>1</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>464</v>
+      </c>
+      <c r="C26" s="17">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="16"/>
+        <v>1500</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>197</v>
+      </c>
+      <c r="G26" s="16" t="s">
+        <v>465</v>
+      </c>
+      <c r="H26" s="16" t="s">
+        <v>466</v>
+      </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="18" t="b">
@@ -4565,7 +4928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B072A382-E462-4BE1-97F8-C914956E97E2}">
   <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
@@ -4727,7 +5090,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A64E22B-8706-4C7D-8FD7-8DB91A3B148C}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.35"/>
@@ -4850,7 +5213,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BC8A8BC-C561-4B6F-BC57-3A027560508C}">
   <dimension ref="A1:J11"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.35"/>
@@ -4958,194 +5321,6 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E9ACF1C-C12B-4B5A-BD57-0454748C5027}">
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="18.1796875" customWidth="1"/>
-    <col min="2" max="2" width="16.26953125" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" customWidth="1"/>
-    <col min="4" max="4" width="16.26953125" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" customWidth="1"/>
-    <col min="6" max="7" width="18.54296875" customWidth="1"/>
-    <col min="8" max="8" width="54.90625" customWidth="1"/>
-    <col min="9" max="16384" width="8.7265625" hidden="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>201</v>
-      </c>
-      <c r="B1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C1" t="s">
-        <v>228</v>
-      </c>
-      <c r="D1" t="s">
-        <v>230</v>
-      </c>
-      <c r="E1" t="s">
-        <v>89</v>
-      </c>
-      <c r="F1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C2" t="s">
-        <v>234</v>
-      </c>
-      <c r="D2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E2" t="s">
-        <v>90</v>
-      </c>
-      <c r="F2" t="s">
-        <v>93</v>
-      </c>
-      <c r="G2" t="s">
-        <v>91</v>
-      </c>
-      <c r="H2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>147</v>
-      </c>
-      <c r="C3" t="s">
-        <v>229</v>
-      </c>
-      <c r="D3" t="s">
-        <v>233</v>
-      </c>
-      <c r="E3" t="s">
-        <v>150</v>
-      </c>
-      <c r="F3" t="s">
-        <v>148</v>
-      </c>
-      <c r="G3" t="s">
-        <v>149</v>
-      </c>
-      <c r="H3" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C4" t="s">
-        <v>369</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>370</v>
-      </c>
-      <c r="E4" t="s">
-        <v>371</v>
-      </c>
-      <c r="F4" t="s">
-        <v>123</v>
-      </c>
-      <c r="G4" t="s">
-        <v>372</v>
-      </c>
-      <c r="H4" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>88</v>
-      </c>
-      <c r="C5" t="s">
-        <v>369</v>
-      </c>
-      <c r="D5" t="s">
-        <v>378</v>
-      </c>
-      <c r="E5" t="s">
-        <v>377</v>
-      </c>
-      <c r="F5" t="s">
-        <v>175</v>
-      </c>
-      <c r="G5" t="s">
-        <v>379</v>
-      </c>
-      <c r="H5" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5697,7 +5872,31 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B19" t="s">
+        <v>462</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" t="s">
+        <v>110</v>
+      </c>
+      <c r="E19" s="5">
+        <v>0.05</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="H19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
@@ -5740,6 +5939,194 @@
   <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E9ACF1C-C12B-4B5A-BD57-0454748C5027}">
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.1796875" customWidth="1"/>
+    <col min="2" max="2" width="16.26953125" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" customWidth="1"/>
+    <col min="4" max="4" width="16.26953125" customWidth="1"/>
+    <col min="5" max="5" width="15.26953125" customWidth="1"/>
+    <col min="6" max="7" width="18.54296875" customWidth="1"/>
+    <col min="8" max="8" width="54.90625" customWidth="1"/>
+    <col min="9" max="16384" width="8.7265625" hidden="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" t="s">
+        <v>228</v>
+      </c>
+      <c r="D1" t="s">
+        <v>230</v>
+      </c>
+      <c r="E1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" t="s">
+        <v>234</v>
+      </c>
+      <c r="D2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D3" t="s">
+        <v>233</v>
+      </c>
+      <c r="E3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G3" t="s">
+        <v>149</v>
+      </c>
+      <c r="H3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" t="s">
+        <v>369</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="E4" t="s">
+        <v>371</v>
+      </c>
+      <c r="F4" t="s">
+        <v>123</v>
+      </c>
+      <c r="G4" t="s">
+        <v>372</v>
+      </c>
+      <c r="H4" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" t="s">
+        <v>369</v>
+      </c>
+      <c r="D5" t="s">
+        <v>378</v>
+      </c>
+      <c r="E5" t="s">
+        <v>377</v>
+      </c>
+      <c r="F5" t="s">
+        <v>175</v>
+      </c>
+      <c r="G5" t="s">
+        <v>379</v>
+      </c>
+      <c r="H5" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6400,7 +6787,7 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>449</v>
@@ -6426,7 +6813,7 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>449</v>
@@ -6452,33 +6839,115 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C36" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="C36" s="12">
+        <v>20</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>467</v>
+      </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C37" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="C37" s="12">
+        <v>20</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>469</v>
+      </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C38" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="C38" s="12">
+        <v>30</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>485</v>
+      </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C39" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="C39" s="12">
+        <v>30</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>484</v>
+      </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C40" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="C40" s="12">
+        <v>5</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>488</v>
+      </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="b">
@@ -6791,12 +7260,48 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E4" t="s">
+        <v>470</v>
+      </c>
+      <c r="F4" t="s">
+        <v>471</v>
+      </c>
+      <c r="G4" t="s">
+        <v>472</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>473</v>
+      </c>
+      <c r="C5" t="s">
+        <v>474</v>
+      </c>
+      <c r="D5" t="s">
+        <v>475</v>
+      </c>
+      <c r="E5" t="s">
+        <v>476</v>
+      </c>
+      <c r="F5" t="s">
+        <v>477</v>
+      </c>
+      <c r="G5" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -7612,7 +8117,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>479</v>
+      </c>
+      <c r="D11" t="s">
+        <v>480</v>
+      </c>
+      <c r="E11" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Added more parts back
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA597E36-0E70-4D13-9861-BA1C34C11D36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B24E037-9FFD-4AB0-8D05-13182DA3B83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="8" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="8" activeTab="8" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="550">
   <si>
     <t>Capacitance</t>
   </si>
@@ -1643,6 +1643,72 @@
   </si>
   <si>
     <t>OR Controller N+1 ORing Controller N-Channel 1:1 12-WSON (3x3)</t>
+  </si>
+  <si>
+    <t>TVS</t>
+  </si>
+  <si>
+    <t>33V</t>
+  </si>
+  <si>
+    <t>N/A, rated for 600W</t>
+  </si>
+  <si>
+    <t>SMBJ33CA</t>
+  </si>
+  <si>
+    <t>53.3V Clamp 11.3A Ipp Tvs Diode Surface Mount DO-214AA (SMBJ)</t>
+  </si>
+  <si>
+    <t>90.9k</t>
+  </si>
+  <si>
+    <t>CR0603-FX-9092ELF</t>
+  </si>
+  <si>
+    <t>90.9 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Moisture Resistant Thick Film</t>
+  </si>
+  <si>
+    <t>9.09k</t>
+  </si>
+  <si>
+    <t>RMCF0603FT9K09</t>
+  </si>
+  <si>
+    <t>9.09 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
+    <t>3.48k</t>
+  </si>
+  <si>
+    <t>RMCF0603FT3K48</t>
+  </si>
+  <si>
+    <t>3.48 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
+    <t>SPI-CAN Bridge</t>
+  </si>
+  <si>
+    <t>MCP2518FDT-E/SL</t>
+  </si>
+  <si>
+    <t>Uses single-ended CAN</t>
+  </si>
+  <si>
+    <t>CAN Controller CAN 2.0 SPI Interface 14-SOIC</t>
+  </si>
+  <si>
+    <t>CAN Frontend Transceiver</t>
+  </si>
+  <si>
+    <t>Single-ended CAN to CAN FD</t>
+  </si>
+  <si>
+    <t>ATA6561-GAQW-N</t>
+  </si>
+  <si>
+    <t>1/1 Transceiver CANbus 8-SO</t>
   </si>
 </sst>
 </file>
@@ -2085,32 +2151,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
@@ -2141,6 +2181,32 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2186,13 +2252,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I26" totalsRowShown="0">
   <autoFilter ref="A1:I26" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="75"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="74"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="65"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="73"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="72"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -2381,20 +2447,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="77">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="71">
   <autoFilter ref="A1:H50" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H31">
     <sortCondition ref="B1:B31"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="76"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="72"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="71"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="70"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="69"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="70"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="68"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2417,10 +2483,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G7" totalsRowShown="0" headerRowDxfId="64">
-  <autoFilter ref="A1:G7" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G20" totalsRowShown="0" headerRowDxfId="77">
+  <autoFilter ref="A1:G20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="76"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -3914,31 +3980,31 @@
         <v>1</v>
       </c>
       <c r="B2" s="15">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="C2" s="17">
-        <f t="shared" ref="C2:C33" si="0">IF(ISNUMBER(B2),
+        <f>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
 IF(RIGHT(B2,1)="k",1000,
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</f>
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>53</v>
+        <v>139</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>8</v>
+        <v>128</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>196</v>
+        <v>264</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>56</v>
+        <v>428</v>
       </c>
       <c r="H2" s="16" t="s">
-        <v>57</v>
+        <v>429</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -3946,26 +4012,31 @@
         <v>1</v>
       </c>
       <c r="B3" s="15">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C3" s="17">
-        <f t="shared" si="0"/>
-        <v>33</v>
+        <f>IF(ISNUMBER(B3),
+IF(B3=0,"",B3),
+VALUE(LEFT(B3,LEN(B3)-1))*
+IF(RIGHT(B3,1)="k",1000,
+IF(RIGHT(B3,1)="M",1000000,
+IF(RIGHT(B3,1)="m",0.001,1))))</f>
+        <v>27</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="E3" s="16" t="s">
         <v>8</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>66</v>
+        <v>196</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -3973,26 +4044,31 @@
         <v>1</v>
       </c>
       <c r="B4" s="15">
-        <v>100</v>
+        <v>33</v>
       </c>
       <c r="C4" s="17">
-        <f t="shared" si="0"/>
-        <v>100</v>
+        <f>IF(ISNUMBER(B4),
+IF(B4=0,"",B4),
+VALUE(LEFT(B4,LEN(B4)-1))*
+IF(RIGHT(B4,1)="k",1000,
+IF(RIGHT(B4,1)="M",1000000,
+IF(RIGHT(B4,1)="m",0.001,1))))</f>
+        <v>33</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="E4" s="16" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>196</v>
+        <v>66</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>238</v>
+        <v>63</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>239</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -4000,11 +4076,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="15">
-        <v>220</v>
+        <v>100</v>
       </c>
       <c r="C5" s="17">
-        <f t="shared" si="0"/>
-        <v>220</v>
+        <f>IF(ISNUMBER(B5),
+IF(B5=0,"",B5),
+VALUE(LEFT(B5,LEN(B5)-1))*
+IF(RIGHT(B5,1)="k",1000,
+IF(RIGHT(B5,1)="M",1000000,
+IF(RIGHT(B5,1)="m",0.001,1))))</f>
+        <v>100</v>
       </c>
       <c r="D5" s="16" t="s">
         <v>53</v>
@@ -4016,10 +4097,10 @@
         <v>196</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>62</v>
+        <v>238</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>61</v>
+        <v>239</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -4030,23 +4111,28 @@
         <v>220</v>
       </c>
       <c r="C6" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B6),
+IF(B6=0,"",B6),
+VALUE(LEFT(B6,LEN(B6)-1))*
+IF(RIGHT(B6,1)="k",1000,
+IF(RIGHT(B6,1)="M",1000000,
+IF(RIGHT(B6,1)="m",0.001,1))))</f>
         <v>220</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>53</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>140</v>
+        <v>196</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>167</v>
+        <v>62</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>166</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -4057,77 +4143,92 @@
         <v>220</v>
       </c>
       <c r="C7" s="17">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B7),
+IF(B7=0,"",B7),
+VALUE(LEFT(B7,LEN(B7)-1))*
+IF(RIGHT(B7,1)="k",1000,
+IF(RIGHT(B7,1)="M",1000000,
+IF(RIGHT(B7,1)="m",0.001,1))))</f>
         <v>220</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>139</v>
+        <v>53</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>128</v>
+        <v>24</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>264</v>
+        <v>140</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>358</v>
+        <v>167</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>359</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>60</v>
+      <c r="B8" s="15">
+        <v>220</v>
       </c>
       <c r="C8" s="17">
-        <f t="shared" si="0"/>
-        <v>1000</v>
+        <f>IF(ISNUMBER(B8),
+IF(B8=0,"",B8),
+VALUE(LEFT(B8,LEN(B8)-1))*
+IF(RIGHT(B8,1)="k",1000,
+IF(RIGHT(B8,1)="M",1000000,
+IF(RIGHT(B8,1)="m",0.001,1))))</f>
+        <v>220</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>53</v>
+        <v>139</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>8</v>
+        <v>128</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>196</v>
+        <v>264</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>58</v>
+        <v>358</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>59</v>
+        <v>359</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="B9" s="15" t="s">
-        <v>60</v>
+      <c r="B9" s="15">
+        <v>680</v>
       </c>
       <c r="C9" s="17">
-        <f t="shared" si="0"/>
-        <v>1000</v>
+        <f>IF(ISNUMBER(B9),
+IF(B9=0,"",B9),
+VALUE(LEFT(B9,LEN(B9)-1))*
+IF(RIGHT(B9,1)="k",1000,
+IF(RIGHT(B9,1)="M",1000000,
+IF(RIGHT(B9,1)="m",0.001,1))))</f>
+        <v>680</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>196</v>
+        <v>140</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>133</v>
+        <v>443</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>134</v>
+        <v>444</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -4135,14 +4236,19 @@
         <v>1</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="C10" s="17">
-        <f t="shared" si="0"/>
-        <v>2000</v>
+        <f>IF(ISNUMBER(B10),
+IF(B10=0,"",B10),
+VALUE(LEFT(B10,LEN(B10)-1))*
+IF(RIGHT(B10,1)="k",1000,
+IF(RIGHT(B10,1)="M",1000000,
+IF(RIGHT(B10,1)="m",0.001,1))))</f>
+        <v>1000</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="E10" s="16" t="s">
         <v>8</v>
@@ -4151,10 +4257,10 @@
         <v>196</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
@@ -4162,26 +4268,31 @@
         <v>1</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>371</v>
+        <v>60</v>
       </c>
       <c r="C11" s="17">
-        <f t="shared" si="0"/>
-        <v>3300</v>
+        <f>IF(ISNUMBER(B11),
+IF(B11=0,"",B11),
+VALUE(LEFT(B11,LEN(B11)-1))*
+IF(RIGHT(B11,1)="k",1000,
+IF(RIGHT(B11,1)="M",1000000,
+IF(RIGHT(B11,1)="m",0.001,1))))</f>
+        <v>1000</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F11" s="16" t="s">
         <v>196</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>372</v>
+        <v>133</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>373</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -4189,11 +4300,16 @@
         <v>1</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>52</v>
+        <v>461</v>
       </c>
       <c r="C12" s="17">
-        <f t="shared" si="0"/>
-        <v>5100</v>
+        <f>IF(ISNUMBER(B12),
+IF(B12=0,"",B12),
+VALUE(LEFT(B12,LEN(B12)-1))*
+IF(RIGHT(B12,1)="k",1000,
+IF(RIGHT(B12,1)="M",1000000,
+IF(RIGHT(B12,1)="m",0.001,1))))</f>
+        <v>1500</v>
       </c>
       <c r="D12" s="16" t="s">
         <v>53</v>
@@ -4205,10 +4321,10 @@
         <v>196</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>54</v>
+        <v>462</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>55</v>
+        <v>463</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -4216,26 +4332,31 @@
         <v>1</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="C13" s="17">
-        <f t="shared" si="0"/>
-        <v>10000</v>
+        <f>IF(ISNUMBER(B13),
+IF(B13=0,"",B13),
+VALUE(LEFT(B13,LEN(B13)-1))*
+IF(RIGHT(B13,1)="k",1000,
+IF(RIGHT(B13,1)="M",1000000,
+IF(RIGHT(B13,1)="m",0.001,1))))</f>
+        <v>2000</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>139</v>
+        <v>70</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>140</v>
+        <v>196</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>141</v>
+        <v>67</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>142</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
@@ -4243,11 +4364,16 @@
         <v>1</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>138</v>
+        <v>371</v>
       </c>
       <c r="C14" s="17">
-        <f t="shared" si="0"/>
-        <v>10000</v>
+        <f>IF(ISNUMBER(B14),
+IF(B14=0,"",B14),
+VALUE(LEFT(B14,LEN(B14)-1))*
+IF(RIGHT(B14,1)="k",1000,
+IF(RIGHT(B14,1)="M",1000000,
+IF(RIGHT(B14,1)="m",0.001,1))))</f>
+        <v>3300</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>53</v>
@@ -4259,10 +4385,10 @@
         <v>196</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>391</v>
+        <v>372</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>392</v>
+        <v>373</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -4270,11 +4396,16 @@
         <v>1</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>329</v>
+        <v>539</v>
       </c>
       <c r="C15" s="17">
-        <f t="shared" si="0"/>
-        <v>47000</v>
+        <f>IF(ISNUMBER(B15),
+IF(B15=0,"",B15),
+VALUE(LEFT(B15,LEN(B15)-1))*
+IF(RIGHT(B15,1)="k",1000,
+IF(RIGHT(B15,1)="M",1000000,
+IF(RIGHT(B15,1)="m",0.001,1))))</f>
+        <v>3480</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>53</v>
@@ -4286,10 +4417,10 @@
         <v>196</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>330</v>
+        <v>540</v>
       </c>
       <c r="H15" s="16" t="s">
-        <v>331</v>
+        <v>541</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -4297,26 +4428,31 @@
         <v>1</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>143</v>
+        <v>52</v>
       </c>
       <c r="C16" s="17">
-        <f t="shared" si="0"/>
-        <v>52300</v>
+        <f>IF(ISNUMBER(B16),
+IF(B16=0,"",B16),
+VALUE(LEFT(B16,LEN(B16)-1))*
+IF(RIGHT(B16,1)="k",1000,
+IF(RIGHT(B16,1)="M",1000000,
+IF(RIGHT(B16,1)="m",0.001,1))))</f>
+        <v>5100</v>
       </c>
       <c r="D16" s="16" t="s">
         <v>53</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>140</v>
+        <v>196</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>144</v>
+        <v>54</v>
       </c>
       <c r="H16" s="16" t="s">
-        <v>145</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -4324,26 +4460,31 @@
         <v>1</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>267</v>
+        <v>536</v>
       </c>
       <c r="C17" s="17">
-        <f t="shared" si="0"/>
-        <v>100000</v>
+        <f>IF(ISNUMBER(B17),
+IF(B17=0,"",B17),
+VALUE(LEFT(B17,LEN(B17)-1))*
+IF(RIGHT(B17,1)="k",1000,
+IF(RIGHT(B17,1)="M",1000000,
+IF(RIGHT(B17,1)="m",0.001,1))))</f>
+        <v>9090</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>53</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>128</v>
+        <v>8</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>264</v>
+        <v>196</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>265</v>
+        <v>537</v>
       </c>
       <c r="H17" s="16" t="s">
-        <v>266</v>
+        <v>538</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
@@ -4351,26 +4492,31 @@
         <v>1</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>291</v>
+        <v>138</v>
       </c>
       <c r="C18" s="17">
-        <f t="shared" si="0"/>
-        <v>680000</v>
+        <f>IF(ISNUMBER(B18),
+IF(B18=0,"",B18),
+VALUE(LEFT(B18,LEN(B18)-1))*
+IF(RIGHT(B18,1)="k",1000,
+IF(RIGHT(B18,1)="M",1000000,
+IF(RIGHT(B18,1)="m",0.001,1))))</f>
+        <v>10000</v>
       </c>
       <c r="D18" s="16" t="s">
         <v>139</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>128</v>
+        <v>24</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>289</v>
+        <v>140</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>292</v>
+        <v>141</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>294</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
@@ -4378,26 +4524,31 @@
         <v>1</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>288</v>
+        <v>138</v>
       </c>
       <c r="C19" s="17">
-        <f t="shared" si="0"/>
-        <v>1000000</v>
+        <f>IF(ISNUMBER(B19),
+IF(B19=0,"",B19),
+VALUE(LEFT(B19,LEN(B19)-1))*
+IF(RIGHT(B19,1)="k",1000,
+IF(RIGHT(B19,1)="M",1000000,
+IF(RIGHT(B19,1)="m",0.001,1))))</f>
+        <v>10000</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>139</v>
+        <v>53</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>128</v>
+        <v>8</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>289</v>
+        <v>196</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>290</v>
+        <v>391</v>
       </c>
       <c r="H19" s="16" t="s">
-        <v>293</v>
+        <v>392</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
@@ -4405,11 +4556,16 @@
         <v>1</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>288</v>
+        <v>440</v>
       </c>
       <c r="C20" s="17">
-        <f t="shared" si="0"/>
-        <v>1000000</v>
+        <f>IF(ISNUMBER(B20),
+IF(B20=0,"",B20),
+VALUE(LEFT(B20,LEN(B20)-1))*
+IF(RIGHT(B20,1)="k",1000,
+IF(RIGHT(B20,1)="M",1000000,
+IF(RIGHT(B20,1)="m",0.001,1))))</f>
+        <v>15000</v>
       </c>
       <c r="D20" s="16" t="s">
         <v>53</v>
@@ -4418,13 +4574,13 @@
         <v>8</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>196</v>
+        <v>140</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>323</v>
+        <v>441</v>
       </c>
       <c r="H20" s="16" t="s">
-        <v>324</v>
+        <v>442</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
@@ -4432,14 +4588,19 @@
         <v>1</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>385</v>
+        <v>329</v>
       </c>
       <c r="C21" s="17">
-        <f t="shared" si="0"/>
-        <v>200000</v>
+        <f>IF(ISNUMBER(B21),
+IF(B21=0,"",B21),
+VALUE(LEFT(B21,LEN(B21)-1))*
+IF(RIGHT(B21,1)="k",1000,
+IF(RIGHT(B21,1)="M",1000000,
+IF(RIGHT(B21,1)="m",0.001,1))))</f>
+        <v>47000</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>139</v>
+        <v>53</v>
       </c>
       <c r="E21" s="16" t="s">
         <v>8</v>
@@ -4448,10 +4609,10 @@
         <v>196</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>386</v>
+        <v>330</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>387</v>
+        <v>331</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
@@ -4459,53 +4620,63 @@
         <v>1</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>388</v>
+        <v>143</v>
       </c>
       <c r="C22" s="17">
-        <f t="shared" si="0"/>
-        <v>300000</v>
+        <f>IF(ISNUMBER(B22),
+IF(B22=0,"",B22),
+VALUE(LEFT(B22,LEN(B22)-1))*
+IF(RIGHT(B22,1)="k",1000,
+IF(RIGHT(B22,1)="M",1000000,
+IF(RIGHT(B22,1)="m",0.001,1))))</f>
+        <v>52300</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>53</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F22" s="16" t="s">
         <v>140</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>389</v>
+        <v>144</v>
       </c>
       <c r="H22" s="16" t="s">
-        <v>390</v>
+        <v>145</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="B23" s="15">
-        <v>10</v>
+      <c r="B23" s="15" t="s">
+        <v>533</v>
       </c>
       <c r="C23" s="17">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>IF(ISNUMBER(B23),
+IF(B23=0,"",B23),
+VALUE(LEFT(B23,LEN(B23)-1))*
+IF(RIGHT(B23,1)="k",1000,
+IF(RIGHT(B23,1)="M",1000000,
+IF(RIGHT(B23,1)="m",0.001,1))))</f>
+        <v>90900</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>139</v>
+        <v>53</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>128</v>
+        <v>8</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>264</v>
+        <v>196</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>428</v>
+        <v>534</v>
       </c>
       <c r="H23" s="16" t="s">
-        <v>429</v>
+        <v>535</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
@@ -4513,53 +4684,63 @@
         <v>1</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>440</v>
+        <v>267</v>
       </c>
       <c r="C24" s="17">
-        <f t="shared" si="0"/>
-        <v>15000</v>
+        <f>IF(ISNUMBER(B24),
+IF(B24=0,"",B24),
+VALUE(LEFT(B24,LEN(B24)-1))*
+IF(RIGHT(B24,1)="k",1000,
+IF(RIGHT(B24,1)="M",1000000,
+IF(RIGHT(B24,1)="m",0.001,1))))</f>
+        <v>100000</v>
       </c>
       <c r="D24" s="16" t="s">
         <v>53</v>
       </c>
       <c r="E24" s="16" t="s">
-        <v>8</v>
+        <v>128</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>140</v>
+        <v>264</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>441</v>
+        <v>265</v>
       </c>
       <c r="H24" s="16" t="s">
-        <v>442</v>
+        <v>266</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="B25" s="15">
-        <v>680</v>
+      <c r="B25" s="15" t="s">
+        <v>385</v>
       </c>
       <c r="C25" s="17">
-        <f t="shared" si="0"/>
-        <v>680</v>
+        <f>IF(ISNUMBER(B25),
+IF(B25=0,"",B25),
+VALUE(LEFT(B25,LEN(B25)-1))*
+IF(RIGHT(B25,1)="k",1000,
+IF(RIGHT(B25,1)="M",1000000,
+IF(RIGHT(B25,1)="m",0.001,1))))</f>
+        <v>200000</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>53</v>
+        <v>139</v>
       </c>
       <c r="E25" s="16" t="s">
         <v>8</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>140</v>
+        <v>196</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>443</v>
+        <v>386</v>
       </c>
       <c r="H25" s="16" t="s">
-        <v>444</v>
+        <v>387</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
@@ -4567,11 +4748,16 @@
         <v>1</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>461</v>
+        <v>388</v>
       </c>
       <c r="C26" s="17">
-        <f t="shared" si="0"/>
-        <v>1500</v>
+        <f>IF(ISNUMBER(B26),
+IF(B26=0,"",B26),
+VALUE(LEFT(B26,LEN(B26)-1))*
+IF(RIGHT(B26,1)="k",1000,
+IF(RIGHT(B26,1)="M",1000000,
+IF(RIGHT(B26,1)="m",0.001,1))))</f>
+        <v>300000</v>
       </c>
       <c r="D26" s="16" t="s">
         <v>53</v>
@@ -4580,65 +4766,110 @@
         <v>8</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>196</v>
+        <v>140</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>462</v>
+        <v>389</v>
       </c>
       <c r="H26" s="16" t="s">
-        <v>463</v>
+        <v>390</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="B27" s="15">
-        <v>0</v>
-      </c>
-      <c r="C27" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
-      <c r="H27" s="16"/>
+        <v>1</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>291</v>
+      </c>
+      <c r="C27" s="17">
+        <f>IF(ISNUMBER(B27),
+IF(B27=0,"",B27),
+VALUE(LEFT(B27,LEN(B27)-1))*
+IF(RIGHT(B27,1)="k",1000,
+IF(RIGHT(B27,1)="M",1000000,
+IF(RIGHT(B27,1)="m",0.001,1))))</f>
+        <v>680000</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="E27" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="F27" s="16" t="s">
+        <v>289</v>
+      </c>
+      <c r="G27" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="H27" s="16" t="s">
+        <v>294</v>
+      </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="B28" s="15">
-        <v>0</v>
-      </c>
-      <c r="C28" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
+        <v>1</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="C28" s="17">
+        <f>IF(ISNUMBER(B28),
+IF(B28=0,"",B28),
+VALUE(LEFT(B28,LEN(B28)-1))*
+IF(RIGHT(B28,1)="k",1000,
+IF(RIGHT(B28,1)="M",1000000,
+IF(RIGHT(B28,1)="m",0.001,1))))</f>
+        <v>1000000</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="F28" s="16" t="s">
+        <v>289</v>
+      </c>
+      <c r="G28" s="16" t="s">
+        <v>290</v>
+      </c>
+      <c r="H28" s="16" t="s">
+        <v>293</v>
+      </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="B29" s="15">
-        <v>0</v>
-      </c>
-      <c r="C29" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
+        <v>1</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="C29" s="17">
+        <f>IF(ISNUMBER(B29),
+IF(B29=0,"",B29),
+VALUE(LEFT(B29,LEN(B29)-1))*
+IF(RIGHT(B29,1)="k",1000,
+IF(RIGHT(B29,1)="M",1000000,
+IF(RIGHT(B29,1)="m",0.001,1))))</f>
+        <v>1000000</v>
+      </c>
+      <c r="D29" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="E29" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="G29" s="16" t="s">
+        <v>323</v>
+      </c>
+      <c r="H29" s="16" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="18" t="b">
@@ -4648,7 +4879,12 @@
         <v>0</v>
       </c>
       <c r="C30" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B30),
+IF(B30=0,"",B30),
+VALUE(LEFT(B30,LEN(B30)-1))*
+IF(RIGHT(B30,1)="k",1000,
+IF(RIGHT(B30,1)="M",1000000,
+IF(RIGHT(B30,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D30" s="16"/>
@@ -4665,7 +4901,12 @@
         <v>0</v>
       </c>
       <c r="C31" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B31),
+IF(B31=0,"",B31),
+VALUE(LEFT(B31,LEN(B31)-1))*
+IF(RIGHT(B31,1)="k",1000,
+IF(RIGHT(B31,1)="M",1000000,
+IF(RIGHT(B31,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D31" s="16"/>
@@ -4682,7 +4923,12 @@
         <v>0</v>
       </c>
       <c r="C32" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B32),
+IF(B32=0,"",B32),
+VALUE(LEFT(B32,LEN(B32)-1))*
+IF(RIGHT(B32,1)="k",1000,
+IF(RIGHT(B32,1)="M",1000000,
+IF(RIGHT(B32,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D32" s="16"/>
@@ -4699,7 +4945,12 @@
         <v>0</v>
       </c>
       <c r="C33" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(ISNUMBER(B33),
+IF(B33=0,"",B33),
+VALUE(LEFT(B33,LEN(B33)-1))*
+IF(RIGHT(B33,1)="k",1000,
+IF(RIGHT(B33,1)="M",1000000,
+IF(RIGHT(B33,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D33" s="16"/>
@@ -4716,7 +4967,7 @@
         <v>0</v>
       </c>
       <c r="C34" s="17" t="str">
-        <f t="shared" ref="C34:C50" si="1">IF(ISNUMBER(B34),
+        <f>IF(ISNUMBER(B34),
 IF(B34=0,"",B34),
 VALUE(LEFT(B34,LEN(B34)-1))*
 IF(RIGHT(B34,1)="k",1000,
@@ -4738,7 +4989,12 @@
         <v>0</v>
       </c>
       <c r="C35" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B35),
+IF(B35=0,"",B35),
+VALUE(LEFT(B35,LEN(B35)-1))*
+IF(RIGHT(B35,1)="k",1000,
+IF(RIGHT(B35,1)="M",1000000,
+IF(RIGHT(B35,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D35" s="16"/>
@@ -4755,7 +5011,12 @@
         <v>0</v>
       </c>
       <c r="C36" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B36),
+IF(B36=0,"",B36),
+VALUE(LEFT(B36,LEN(B36)-1))*
+IF(RIGHT(B36,1)="k",1000,
+IF(RIGHT(B36,1)="M",1000000,
+IF(RIGHT(B36,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D36" s="16"/>
@@ -4772,7 +5033,12 @@
         <v>0</v>
       </c>
       <c r="C37" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B37),
+IF(B37=0,"",B37),
+VALUE(LEFT(B37,LEN(B37)-1))*
+IF(RIGHT(B37,1)="k",1000,
+IF(RIGHT(B37,1)="M",1000000,
+IF(RIGHT(B37,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D37" s="16"/>
@@ -4789,7 +5055,12 @@
         <v>0</v>
       </c>
       <c r="C38" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B38),
+IF(B38=0,"",B38),
+VALUE(LEFT(B38,LEN(B38)-1))*
+IF(RIGHT(B38,1)="k",1000,
+IF(RIGHT(B38,1)="M",1000000,
+IF(RIGHT(B38,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D38" s="16"/>
@@ -4806,7 +5077,12 @@
         <v>0</v>
       </c>
       <c r="C39" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B39),
+IF(B39=0,"",B39),
+VALUE(LEFT(B39,LEN(B39)-1))*
+IF(RIGHT(B39,1)="k",1000,
+IF(RIGHT(B39,1)="M",1000000,
+IF(RIGHT(B39,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D39" s="16"/>
@@ -4823,7 +5099,12 @@
         <v>0</v>
       </c>
       <c r="C40" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B40),
+IF(B40=0,"",B40),
+VALUE(LEFT(B40,LEN(B40)-1))*
+IF(RIGHT(B40,1)="k",1000,
+IF(RIGHT(B40,1)="M",1000000,
+IF(RIGHT(B40,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D40" s="16"/>
@@ -4840,7 +5121,12 @@
         <v>0</v>
       </c>
       <c r="C41" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B41),
+IF(B41=0,"",B41),
+VALUE(LEFT(B41,LEN(B41)-1))*
+IF(RIGHT(B41,1)="k",1000,
+IF(RIGHT(B41,1)="M",1000000,
+IF(RIGHT(B41,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D41" s="16"/>
@@ -4857,7 +5143,12 @@
         <v>0</v>
       </c>
       <c r="C42" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B42),
+IF(B42=0,"",B42),
+VALUE(LEFT(B42,LEN(B42)-1))*
+IF(RIGHT(B42,1)="k",1000,
+IF(RIGHT(B42,1)="M",1000000,
+IF(RIGHT(B42,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D42" s="16"/>
@@ -4874,7 +5165,12 @@
         <v>0</v>
       </c>
       <c r="C43" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B43),
+IF(B43=0,"",B43),
+VALUE(LEFT(B43,LEN(B43)-1))*
+IF(RIGHT(B43,1)="k",1000,
+IF(RIGHT(B43,1)="M",1000000,
+IF(RIGHT(B43,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D43" s="16"/>
@@ -4891,7 +5187,12 @@
         <v>0</v>
       </c>
       <c r="C44" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B44),
+IF(B44=0,"",B44),
+VALUE(LEFT(B44,LEN(B44)-1))*
+IF(RIGHT(B44,1)="k",1000,
+IF(RIGHT(B44,1)="M",1000000,
+IF(RIGHT(B44,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D44" s="16"/>
@@ -4908,7 +5209,12 @@
         <v>0</v>
       </c>
       <c r="C45" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B45),
+IF(B45=0,"",B45),
+VALUE(LEFT(B45,LEN(B45)-1))*
+IF(RIGHT(B45,1)="k",1000,
+IF(RIGHT(B45,1)="M",1000000,
+IF(RIGHT(B45,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D45" s="16"/>
@@ -4925,7 +5231,12 @@
         <v>0</v>
       </c>
       <c r="C46" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B46),
+IF(B46=0,"",B46),
+VALUE(LEFT(B46,LEN(B46)-1))*
+IF(RIGHT(B46,1)="k",1000,
+IF(RIGHT(B46,1)="M",1000000,
+IF(RIGHT(B46,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D46" s="16"/>
@@ -4942,7 +5253,12 @@
         <v>0</v>
       </c>
       <c r="C47" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B47),
+IF(B47=0,"",B47),
+VALUE(LEFT(B47,LEN(B47)-1))*
+IF(RIGHT(B47,1)="k",1000,
+IF(RIGHT(B47,1)="M",1000000,
+IF(RIGHT(B47,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D47" s="16"/>
@@ -4959,7 +5275,12 @@
         <v>0</v>
       </c>
       <c r="C48" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B48),
+IF(B48=0,"",B48),
+VALUE(LEFT(B48,LEN(B48)-1))*
+IF(RIGHT(B48,1)="k",1000,
+IF(RIGHT(B48,1)="M",1000000,
+IF(RIGHT(B48,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D48" s="16"/>
@@ -4976,7 +5297,12 @@
         <v>0</v>
       </c>
       <c r="C49" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B49),
+IF(B49=0,"",B49),
+VALUE(LEFT(B49,LEN(B49)-1))*
+IF(RIGHT(B49,1)="k",1000,
+IF(RIGHT(B49,1)="M",1000000,
+IF(RIGHT(B49,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D49" s="16"/>
@@ -4993,7 +5319,12 @@
         <v>0</v>
       </c>
       <c r="C50" s="17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(B50),
+IF(B50=0,"",B50),
+VALUE(LEFT(B50,LEN(B50)-1))*
+IF(RIGHT(B50,1)="k",1000,
+IF(RIGHT(B50,1)="M",1000000,
+IF(RIGHT(B50,1)="m",0.001,1))))</f>
         <v/>
       </c>
       <c r="D50" s="16"/>
@@ -7402,7 +7733,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B0A492-FDE3-4289-9C55-9A97FFD78944}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.08984375" customWidth="1"/>
@@ -7529,11 +7860,94 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>528</v>
+      </c>
+      <c r="C6" t="s">
+        <v>529</v>
+      </c>
+      <c r="D6" t="s">
+        <v>530</v>
+      </c>
+      <c r="E6" t="s">
+        <v>175</v>
+      </c>
+      <c r="F6" t="s">
+        <v>531</v>
+      </c>
+      <c r="G6" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8388,12 +8802,36 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B14" t="s">
+        <v>542</v>
+      </c>
+      <c r="C14" t="s">
+        <v>544</v>
+      </c>
+      <c r="D14" t="s">
+        <v>543</v>
+      </c>
+      <c r="E14" t="s">
+        <v>545</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B15" t="s">
+        <v>546</v>
+      </c>
+      <c r="C15" t="s">
+        <v>547</v>
+      </c>
+      <c r="D15" t="s">
+        <v>548</v>
+      </c>
+      <c r="E15" t="s">
+        <v>549</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
5/19 Connections for NP board added
Will submit pull request when the board is done
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA597E36-0E70-4D13-9861-BA1C34C11D36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02B72D8D-4C6A-47B0-9459-D34D5ED59831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="8" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9420" firstSheet="1" activeTab="2" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="531">
   <si>
     <t>Capacitance</t>
   </si>
@@ -1643,6 +1643,15 @@
   </si>
   <si>
     <t>OR Controller N+1 ORing Controller N-Channel 1:1 12-WSON (3x3)</t>
+  </si>
+  <si>
+    <t>1778777</t>
+  </si>
+  <si>
+    <t>1778845</t>
+  </si>
+  <si>
+    <t>3 Position Terminal Block Header, Male Pins, Shrouded (4 Side) 0.098" (2.50mm) 90°, Right Angle Surface Mount</t>
   </si>
 </sst>
 </file>
@@ -2023,20 +2032,6 @@
       </extLst>
     </dxf>
     <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -2104,22 +2099,6 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
@@ -2141,6 +2120,36 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2186,13 +2195,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I26" totalsRowShown="0">
   <autoFilter ref="A1:I26" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="75"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="74"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="65"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="73"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="72"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -2381,20 +2390,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="77">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="71">
   <autoFilter ref="A1:H50" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H31">
     <sortCondition ref="B1:B31"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="76"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="72"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="71"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="70"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="69"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="70"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="68"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2417,10 +2426,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G7" totalsRowShown="0" headerRowDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G7" totalsRowShown="0" headerRowDxfId="62">
   <autoFilter ref="A1:G7" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="61"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -2433,11 +2442,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="60">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="61"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="60"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="59"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="58"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -2448,25 +2457,25 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="59">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="57">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="58"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="56"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="55"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="56"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="54"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="53">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="51">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="52"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="49"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -2486,8 +2495,8 @@
     <sortCondition ref="B1:B10"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="77"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="76"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -2831,19 +2840,19 @@
     <tabColor rgb="FF00B050"/>
   </sheetPr>
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>191</v>
       </c>
@@ -2851,12 +2860,12 @@
         <v>198</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>181</v>
       </c>
@@ -2864,52 +2873,52 @@
         <v>199</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>186</v>
       </c>
@@ -2922,17 +2931,17 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B0DCFA9-0ACD-44E9-B5AC-404F4D59A007}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.54296875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="21.1796875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="22.1796875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="15.5546875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="21.21875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="22.21875" style="3" customWidth="1"/>
     <col min="4" max="4" width="32" style="3" customWidth="1"/>
-    <col min="5" max="5" width="45.81640625" style="3" customWidth="1"/>
-    <col min="6" max="16384" width="8.7265625" style="3" hidden="1"/>
+    <col min="5" max="5" width="45.77734375" style="3" customWidth="1"/>
+    <col min="6" max="16384" width="8.77734375" style="3" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>200</v>
       </c>
@@ -2949,7 +2958,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="b">
         <v>1</v>
       </c>
@@ -2966,7 +2975,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="b">
         <v>1</v>
       </c>
@@ -2983,7 +2992,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="b">
         <v>1</v>
       </c>
@@ -3000,37 +3009,37 @@
         <v>308</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="b">
         <v>0</v>
       </c>
@@ -3046,19 +3055,19 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9362198B-44BD-4E55-B62E-439143EC0CFE}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="8.7265625" customWidth="1"/>
-    <col min="4" max="4" width="16.36328125" customWidth="1"/>
-    <col min="5" max="5" width="14.36328125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="17.453125" customWidth="1"/>
-    <col min="7" max="7" width="31.81640625" customWidth="1"/>
-    <col min="8" max="8" width="43.26953125" customWidth="1"/>
-    <col min="9" max="16384" width="8.7265625" hidden="1"/>
+    <col min="3" max="3" width="8.77734375" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" customWidth="1"/>
+    <col min="7" max="7" width="31.77734375" customWidth="1"/>
+    <col min="8" max="8" width="43.21875" customWidth="1"/>
+    <col min="9" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>200</v>
       </c>
@@ -3084,7 +3093,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -3107,7 +3116,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -3130,7 +3139,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
@@ -3153,7 +3162,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>1</v>
       </c>
@@ -3176,7 +3185,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>1</v>
       </c>
@@ -3199,7 +3208,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>1</v>
       </c>
@@ -3225,7 +3234,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>1</v>
       </c>
@@ -3248,7 +3257,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>1</v>
       </c>
@@ -3271,7 +3280,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>1</v>
       </c>
@@ -3306,15 +3315,15 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9F1A110-D627-46EF-8744-E79E320771F1}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="6" width="20.6328125" customWidth="1"/>
-    <col min="7" max="7" width="55.36328125" customWidth="1"/>
-    <col min="8" max="16384" width="8.7265625" hidden="1"/>
+    <col min="2" max="6" width="20.6640625" customWidth="1"/>
+    <col min="7" max="7" width="55.33203125" customWidth="1"/>
+    <col min="8" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
         <v>200</v>
       </c>
@@ -3337,7 +3346,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -3360,7 +3369,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -3383,37 +3392,37 @@
         <v>458</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>0</v>
       </c>
@@ -3430,16 +3439,16 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95B4EE80-6917-43D6-8B0A-D27EC0A92AF4}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="17.7265625" customWidth="1"/>
+    <col min="2" max="2" width="17.77734375" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="37.08984375" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" hidden="1"/>
+    <col min="4" max="4" width="37.109375" customWidth="1"/>
+    <col min="5" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>200</v>
       </c>
@@ -3453,7 +3462,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -3467,7 +3476,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -3481,7 +3490,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
@@ -3495,7 +3504,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>1</v>
       </c>
@@ -3509,7 +3518,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>1</v>
       </c>
@@ -3523,7 +3532,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>1</v>
       </c>
@@ -3537,32 +3546,32 @@
         <v>506</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="b">
         <v>0</v>
       </c>
@@ -3578,19 +3587,19 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22B86CF3-50F4-4B19-99AD-AF8E53CE9DBA}">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.55" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="15.54296875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="21.1796875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.6328125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="20.6328125" style="3" customWidth="1"/>
-    <col min="6" max="7" width="15.6328125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="45.81640625" style="3" customWidth="1"/>
+    <col min="1" max="2" width="15.5546875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="21.21875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" style="3" customWidth="1"/>
+    <col min="6" max="7" width="15.6640625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="45.77734375" style="3" customWidth="1"/>
     <col min="9" max="9" width="0" style="3" hidden="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.7265625" style="3" hidden="1"/>
+    <col min="10" max="16384" width="8.77734375" style="3" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="23" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="23" t="s">
         <v>200</v>
       </c>
@@ -3616,7 +3625,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="b">
         <v>1</v>
       </c>
@@ -3642,7 +3651,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="b">
         <v>1</v>
       </c>
@@ -3668,42 +3677,42 @@
         <v>497</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="b">
         <v>0</v>
       </c>
@@ -3719,17 +3728,17 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF58675A-C2E2-4804-A061-74EF114D288F}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.90625" style="14" customWidth="1"/>
-    <col min="2" max="2" width="18.6328125" style="14" customWidth="1"/>
-    <col min="3" max="8" width="11.7265625" style="14" customWidth="1"/>
-    <col min="9" max="9" width="20.26953125" style="14" customWidth="1"/>
-    <col min="10" max="10" width="34.36328125" style="14" customWidth="1"/>
-    <col min="11" max="16384" width="8.7265625" style="14" hidden="1"/>
+    <col min="1" max="1" width="17.88671875" style="14" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" style="14" customWidth="1"/>
+    <col min="3" max="8" width="11.77734375" style="14" customWidth="1"/>
+    <col min="9" max="9" width="20.21875" style="14" customWidth="1"/>
+    <col min="10" max="10" width="34.33203125" style="14" customWidth="1"/>
+    <col min="11" max="16384" width="8.77734375" style="14" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>200</v>
       </c>
@@ -3761,7 +3770,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="b">
         <v>1</v>
       </c>
@@ -3790,7 +3799,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="b">
         <v>1</v>
       </c>
@@ -3819,42 +3828,42 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="b">
         <v>0</v>
       </c>
@@ -3870,20 +3879,20 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B73385E-A93D-4809-A6CB-D5FDE97D6171}">
   <dimension ref="A1:H50"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.1796875" style="19" customWidth="1"/>
-    <col min="2" max="2" width="14.6328125" customWidth="1"/>
-    <col min="3" max="3" width="9.7265625" customWidth="1"/>
-    <col min="4" max="4" width="11.1796875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="17.21875" style="19" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="9.77734375" customWidth="1"/>
+    <col min="4" max="4" width="11.21875" style="3" customWidth="1"/>
     <col min="5" max="5" width="10" style="3" customWidth="1"/>
-    <col min="6" max="6" width="9.7265625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="24.453125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="31.26953125" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="8.7265625" style="3" hidden="1"/>
+    <col min="6" max="6" width="9.77734375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="24.44140625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="31.21875" style="3" customWidth="1"/>
+    <col min="9" max="16384" width="8.77734375" style="3" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>200</v>
       </c>
@@ -3909,7 +3918,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="b">
         <v>1</v>
       </c>
@@ -3941,7 +3950,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="b">
         <v>1</v>
       </c>
@@ -3968,7 +3977,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="b">
         <v>1</v>
       </c>
@@ -3995,7 +4004,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="b">
         <v>1</v>
       </c>
@@ -4022,7 +4031,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="b">
         <v>1</v>
       </c>
@@ -4049,7 +4058,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="b">
         <v>1</v>
       </c>
@@ -4076,7 +4085,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="18" t="b">
         <v>1</v>
       </c>
@@ -4103,7 +4112,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="18" t="b">
         <v>1</v>
       </c>
@@ -4130,7 +4139,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="18" t="b">
         <v>1</v>
       </c>
@@ -4157,7 +4166,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="18" t="b">
         <v>1</v>
       </c>
@@ -4184,7 +4193,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="18" t="b">
         <v>1</v>
       </c>
@@ -4211,7 +4220,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="18" t="b">
         <v>1</v>
       </c>
@@ -4238,7 +4247,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="18" t="b">
         <v>1</v>
       </c>
@@ -4265,7 +4274,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="18" t="b">
         <v>1</v>
       </c>
@@ -4292,7 +4301,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="18" t="b">
         <v>1</v>
       </c>
@@ -4319,7 +4328,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="18" t="b">
         <v>1</v>
       </c>
@@ -4346,7 +4355,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="18" t="b">
         <v>1</v>
       </c>
@@ -4373,7 +4382,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="18" t="b">
         <v>1</v>
       </c>
@@ -4400,7 +4409,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="18" t="b">
         <v>1</v>
       </c>
@@ -4427,7 +4436,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="18" t="b">
         <v>1</v>
       </c>
@@ -4454,7 +4463,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="18" t="b">
         <v>1</v>
       </c>
@@ -4481,7 +4490,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="18" t="b">
         <v>1</v>
       </c>
@@ -4508,7 +4517,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="b">
         <v>1</v>
       </c>
@@ -4535,7 +4544,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="18" t="b">
         <v>1</v>
       </c>
@@ -4562,7 +4571,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="18" t="b">
         <v>1</v>
       </c>
@@ -4589,7 +4598,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="18" t="b">
         <v>0</v>
       </c>
@@ -4606,7 +4615,7 @@
       <c r="G27" s="16"/>
       <c r="H27" s="16"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="18" t="b">
         <v>0</v>
       </c>
@@ -4623,7 +4632,7 @@
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="18" t="b">
         <v>0</v>
       </c>
@@ -4640,7 +4649,7 @@
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="18" t="b">
         <v>0</v>
       </c>
@@ -4657,7 +4666,7 @@
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="18" t="b">
         <v>0</v>
       </c>
@@ -4674,7 +4683,7 @@
       <c r="G31" s="16"/>
       <c r="H31" s="16"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="18" t="b">
         <v>0</v>
       </c>
@@ -4691,7 +4700,7 @@
       <c r="G32" s="16"/>
       <c r="H32" s="16"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="18" t="b">
         <v>0</v>
       </c>
@@ -4708,7 +4717,7 @@
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="18" t="b">
         <v>0</v>
       </c>
@@ -4730,7 +4739,7 @@
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="18" t="b">
         <v>0</v>
       </c>
@@ -4747,7 +4756,7 @@
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="18" t="b">
         <v>0</v>
       </c>
@@ -4764,7 +4773,7 @@
       <c r="G36" s="16"/>
       <c r="H36" s="16"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="18" t="b">
         <v>0</v>
       </c>
@@ -4781,7 +4790,7 @@
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="18" t="b">
         <v>0</v>
       </c>
@@ -4798,7 +4807,7 @@
       <c r="G38" s="16"/>
       <c r="H38" s="16"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="18" t="b">
         <v>0</v>
       </c>
@@ -4815,7 +4824,7 @@
       <c r="G39" s="16"/>
       <c r="H39" s="16"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="18" t="b">
         <v>0</v>
       </c>
@@ -4832,7 +4841,7 @@
       <c r="G40" s="16"/>
       <c r="H40" s="16"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="18" t="b">
         <v>0</v>
       </c>
@@ -4849,7 +4858,7 @@
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="18" t="b">
         <v>0</v>
       </c>
@@ -4866,7 +4875,7 @@
       <c r="G42" s="16"/>
       <c r="H42" s="16"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="18" t="b">
         <v>0</v>
       </c>
@@ -4883,7 +4892,7 @@
       <c r="G43" s="16"/>
       <c r="H43" s="16"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="18" t="b">
         <v>0</v>
       </c>
@@ -4900,7 +4909,7 @@
       <c r="G44" s="16"/>
       <c r="H44" s="16"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="18" t="b">
         <v>0</v>
       </c>
@@ -4917,7 +4926,7 @@
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="18" t="b">
         <v>0</v>
       </c>
@@ -4934,7 +4943,7 @@
       <c r="G46" s="16"/>
       <c r="H46" s="16"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="18" t="b">
         <v>0</v>
       </c>
@@ -4951,7 +4960,7 @@
       <c r="G47" s="16"/>
       <c r="H47" s="16"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="18" t="b">
         <v>0</v>
       </c>
@@ -4968,7 +4977,7 @@
       <c r="G48" s="16"/>
       <c r="H48" s="16"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="18" t="b">
         <v>0</v>
       </c>
@@ -4985,7 +4994,7 @@
       <c r="G49" s="16"/>
       <c r="H49" s="16"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="18" t="b">
         <v>0</v>
       </c>
@@ -5013,19 +5022,19 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B072A382-E462-4BE1-97F8-C914956E97E2}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.90625" customWidth="1"/>
-    <col min="2" max="2" width="22.26953125" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" customWidth="1"/>
-    <col min="4" max="4" width="19.26953125" customWidth="1"/>
-    <col min="5" max="5" width="14.90625" customWidth="1"/>
-    <col min="6" max="6" width="20.90625" customWidth="1"/>
-    <col min="7" max="7" width="41.81640625" customWidth="1"/>
-    <col min="8" max="16384" width="8.7265625" hidden="1"/>
+    <col min="1" max="1" width="16.88671875" customWidth="1"/>
+    <col min="2" max="2" width="22.21875" customWidth="1"/>
+    <col min="3" max="3" width="13.77734375" customWidth="1"/>
+    <col min="4" max="4" width="19.21875" customWidth="1"/>
+    <col min="5" max="5" width="14.88671875" customWidth="1"/>
+    <col min="6" max="6" width="20.88671875" customWidth="1"/>
+    <col min="7" max="7" width="41.77734375" customWidth="1"/>
+    <col min="8" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>200</v>
       </c>
@@ -5048,7 +5057,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -5071,7 +5080,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -5094,7 +5103,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
@@ -5117,7 +5126,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>1</v>
       </c>
@@ -5134,32 +5143,32 @@
         <v>416</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="b">
         <v>0</v>
       </c>
@@ -5175,19 +5184,19 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A64E22B-8706-4C7D-8FD7-8DB91A3B148C}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.55" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.90625" customWidth="1"/>
-    <col min="2" max="2" width="22.26953125" customWidth="1"/>
-    <col min="3" max="3" width="17.6328125" customWidth="1"/>
-    <col min="4" max="4" width="13.81640625" customWidth="1"/>
-    <col min="5" max="5" width="19.26953125" customWidth="1"/>
-    <col min="6" max="6" width="41.81640625" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" customWidth="1"/>
+    <col min="2" max="2" width="22.21875" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="5" max="5" width="19.21875" customWidth="1"/>
+    <col min="6" max="6" width="41.77734375" customWidth="1"/>
     <col min="7" max="8" width="0" hidden="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.7265625" hidden="1"/>
+    <col min="9" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="22" t="s">
         <v>200</v>
       </c>
@@ -5207,7 +5216,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -5227,7 +5236,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -5247,42 +5256,42 @@
         <v>344</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="b">
         <v>0</v>
       </c>
@@ -5298,18 +5307,18 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BC8A8BC-C561-4B6F-BC57-3A027560508C}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.55" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.90625" customWidth="1"/>
-    <col min="2" max="2" width="12.6328125" customWidth="1"/>
-    <col min="3" max="6" width="13.81640625" customWidth="1"/>
-    <col min="7" max="7" width="19.26953125" customWidth="1"/>
-    <col min="8" max="8" width="41.81640625" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="6" width="13.77734375" customWidth="1"/>
+    <col min="7" max="7" width="19.21875" customWidth="1"/>
+    <col min="8" max="8" width="41.77734375" customWidth="1"/>
     <col min="9" max="10" width="0" hidden="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.7265625" hidden="1"/>
+    <col min="11" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
         <v>200</v>
       </c>
@@ -5335,7 +5344,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -5361,47 +5370,47 @@
         <v>304</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="b">
         <v>0</v>
       </c>
@@ -5417,20 +5426,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{084DDF4D-1E9D-4C12-BB94-6E06CEFC760F}">
   <dimension ref="A1:I26"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.26953125" customWidth="1"/>
-    <col min="2" max="2" width="14.36328125" customWidth="1"/>
-    <col min="3" max="3" width="14.36328125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.08984375" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" customWidth="1"/>
+    <col min="1" max="1" width="17.21875" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" customWidth="1"/>
     <col min="6" max="7" width="15" style="3" customWidth="1"/>
-    <col min="8" max="8" width="9.81640625" customWidth="1"/>
-    <col min="9" max="9" width="26.90625" customWidth="1"/>
-    <col min="10" max="16384" width="8.7265625" hidden="1"/>
+    <col min="8" max="8" width="9.77734375" customWidth="1"/>
+    <col min="9" max="9" width="26.88671875" customWidth="1"/>
+    <col min="10" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>200</v>
       </c>
@@ -5459,7 +5468,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -5488,7 +5497,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -5517,7 +5526,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
@@ -5546,7 +5555,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>1</v>
       </c>
@@ -5575,7 +5584,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>1</v>
       </c>
@@ -5604,7 +5613,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>1</v>
       </c>
@@ -5633,7 +5642,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>1</v>
       </c>
@@ -5662,7 +5671,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>1</v>
       </c>
@@ -5691,7 +5700,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>1</v>
       </c>
@@ -5720,7 +5729,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="b">
         <v>1</v>
       </c>
@@ -5749,7 +5758,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="b">
         <v>1</v>
       </c>
@@ -5778,7 +5787,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="b">
         <v>1</v>
       </c>
@@ -5807,7 +5816,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="b">
         <v>1</v>
       </c>
@@ -5836,7 +5845,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="b">
         <v>1</v>
       </c>
@@ -5865,7 +5874,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="b">
         <v>1</v>
       </c>
@@ -5894,7 +5903,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="b">
         <v>1</v>
       </c>
@@ -5923,7 +5932,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="b">
         <v>1</v>
       </c>
@@ -5952,7 +5961,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="b">
         <v>1</v>
       </c>
@@ -5981,7 +5990,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="b">
         <v>1</v>
       </c>
@@ -6010,7 +6019,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="b">
         <v>1</v>
       </c>
@@ -6039,7 +6048,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="b">
         <v>1</v>
       </c>
@@ -6068,7 +6077,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="b">
         <v>1</v>
       </c>
@@ -6097,17 +6106,17 @@
         <v>520</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="b">
         <v>0</v>
       </c>
@@ -6124,19 +6133,19 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E9ACF1C-C12B-4B5A-BD57-0454748C5027}">
   <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.1796875" customWidth="1"/>
-    <col min="2" max="2" width="16.26953125" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" customWidth="1"/>
-    <col min="4" max="4" width="16.26953125" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" customWidth="1"/>
-    <col min="6" max="7" width="18.54296875" customWidth="1"/>
-    <col min="8" max="8" width="54.90625" customWidth="1"/>
-    <col min="9" max="16384" width="8.7265625" hidden="1"/>
+    <col min="1" max="1" width="18.21875" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" customWidth="1"/>
+    <col min="4" max="4" width="16.21875" customWidth="1"/>
+    <col min="5" max="5" width="15.21875" customWidth="1"/>
+    <col min="6" max="7" width="18.5546875" customWidth="1"/>
+    <col min="8" max="8" width="54.88671875" customWidth="1"/>
+    <col min="9" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>200</v>
       </c>
@@ -6162,7 +6171,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -6188,7 +6197,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -6214,7 +6223,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
@@ -6240,7 +6249,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>1</v>
       </c>
@@ -6266,37 +6275,37 @@
         <v>377</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="b">
         <v>0</v>
       </c>
@@ -6312,24 +6321,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31311A32-7C4D-4571-8105-957397FF3475}">
   <dimension ref="A1:XDX50"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.1796875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="8.453125" style="11" customWidth="1"/>
+    <col min="1" max="1" width="16.21875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="8.44140625" style="11" customWidth="1"/>
     <col min="4" max="4" width="18" style="3" customWidth="1"/>
-    <col min="5" max="5" width="16.54296875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" style="3" customWidth="1"/>
     <col min="6" max="6" width="17" style="3" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="37.54296875" style="3" customWidth="1"/>
-    <col min="9" max="16340" width="8.7265625" style="3" hidden="1"/>
+    <col min="7" max="7" width="12.44140625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="37.5546875" style="3" customWidth="1"/>
+    <col min="9" max="16340" width="8.77734375" style="3" hidden="1"/>
     <col min="16341" max="16341" width="0" style="3" hidden="1"/>
-    <col min="16342" max="16350" width="8.7265625" style="3" hidden="1"/>
+    <col min="16342" max="16350" width="8.77734375" style="3" hidden="1"/>
     <col min="16351" max="16352" width="0" style="3" hidden="1"/>
-    <col min="16353" max="16384" width="8.7265625" style="3" hidden="1"/>
+    <col min="16353" max="16384" width="8.77734375" style="3" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>200</v>
       </c>
@@ -6355,7 +6364,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="b">
         <v>1</v>
       </c>
@@ -6375,7 +6384,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="b">
         <v>1</v>
       </c>
@@ -6398,7 +6407,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="b">
         <v>1</v>
       </c>
@@ -6412,7 +6421,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="b">
         <v>1</v>
       </c>
@@ -6426,7 +6435,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="b">
         <v>1</v>
       </c>
@@ -6440,7 +6449,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="b">
         <v>1</v>
       </c>
@@ -6454,7 +6463,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="b">
         <v>1</v>
       </c>
@@ -6468,7 +6477,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="b">
         <v>1</v>
       </c>
@@ -6482,7 +6491,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="b">
         <v>1</v>
       </c>
@@ -6496,7 +6505,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="b">
         <v>1</v>
       </c>
@@ -6510,7 +6519,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="b">
         <v>1</v>
       </c>
@@ -6524,7 +6533,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="b">
         <v>1</v>
       </c>
@@ -6547,7 +6556,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="b">
         <v>1</v>
       </c>
@@ -6570,7 +6579,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="b">
         <v>1</v>
       </c>
@@ -6590,7 +6599,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="b">
         <v>1</v>
       </c>
@@ -6610,7 +6619,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="b">
         <v>1</v>
       </c>
@@ -6630,7 +6639,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="b">
         <v>1</v>
       </c>
@@ -6653,7 +6662,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="b">
         <v>1</v>
       </c>
@@ -6667,7 +6676,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="b">
         <v>1</v>
       </c>
@@ -6687,7 +6696,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="b">
         <v>1</v>
       </c>
@@ -6707,7 +6716,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="b">
         <v>1</v>
       </c>
@@ -6727,7 +6736,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="b">
         <v>1</v>
       </c>
@@ -6747,7 +6756,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="10" t="b">
         <v>1</v>
       </c>
@@ -6767,7 +6776,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="10" t="b">
         <v>1</v>
       </c>
@@ -6787,7 +6796,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="b">
         <v>1</v>
       </c>
@@ -6810,7 +6819,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="10" t="b">
         <v>1</v>
       </c>
@@ -6831,7 +6840,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="b">
         <v>1</v>
       </c>
@@ -6854,7 +6863,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="10" t="b">
         <v>1</v>
       </c>
@@ -6877,7 +6886,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="b">
         <v>1</v>
       </c>
@@ -6900,7 +6909,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="b">
         <v>1</v>
       </c>
@@ -6923,7 +6932,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="10" t="b">
         <v>1</v>
       </c>
@@ -6946,7 +6955,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="10" t="b">
         <v>1</v>
       </c>
@@ -6963,7 +6972,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="10" t="b">
         <v>1</v>
       </c>
@@ -6989,7 +6998,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="b">
         <v>1</v>
       </c>
@@ -7015,7 +7024,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="b">
         <v>1</v>
       </c>
@@ -7035,7 +7044,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="10" t="b">
         <v>1</v>
       </c>
@@ -7058,7 +7067,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="10" t="b">
         <v>1</v>
       </c>
@@ -7081,7 +7090,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="10" t="b">
         <v>1</v>
       </c>
@@ -7107,7 +7116,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="10" t="b">
         <v>1</v>
       </c>
@@ -7127,7 +7136,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="b">
         <v>1</v>
       </c>
@@ -7147,7 +7156,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="10" t="b">
         <v>1</v>
       </c>
@@ -7167,7 +7176,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="10" t="b">
         <v>1</v>
       </c>
@@ -7190,43 +7199,60 @@
         <v>517</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C44" s="12"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="C44" s="12">
+        <v>3</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C45" s="12"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C46" s="12"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C47" s="12"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C48" s="12"/>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C49" s="12"/>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="10" t="b">
         <v>0</v>
       </c>
@@ -7244,20 +7270,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15EC580B-30DF-4B7B-9130-28D1AB04F48B}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.08984375" customWidth="1"/>
-    <col min="2" max="2" width="17.1796875" customWidth="1"/>
-    <col min="3" max="3" width="14.6328125" customWidth="1"/>
-    <col min="4" max="4" width="17.90625" customWidth="1"/>
-    <col min="5" max="5" width="10.81640625" customWidth="1"/>
-    <col min="6" max="6" width="30.36328125" customWidth="1"/>
-    <col min="7" max="7" width="46.54296875" customWidth="1"/>
+    <col min="1" max="1" width="19.109375" customWidth="1"/>
+    <col min="2" max="2" width="17.21875" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.88671875" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" customWidth="1"/>
+    <col min="6" max="6" width="30.33203125" customWidth="1"/>
+    <col min="7" max="7" width="46.5546875" customWidth="1"/>
     <col min="8" max="8" width="0" hidden="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.7265625" hidden="1"/>
+    <col min="9" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>200</v>
       </c>
@@ -7280,7 +7306,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -7303,7 +7329,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -7326,67 +7352,67 @@
         <v>163</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="b">
         <v>0</v>
       </c>
@@ -7403,19 +7429,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B0A492-FDE3-4289-9C55-9A97FFD78944}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.08984375" customWidth="1"/>
-    <col min="2" max="2" width="15.7265625" customWidth="1"/>
-    <col min="3" max="3" width="18.7265625" customWidth="1"/>
-    <col min="4" max="4" width="20.1796875" customWidth="1"/>
-    <col min="5" max="5" width="14.6328125" customWidth="1"/>
-    <col min="6" max="6" width="19.54296875" customWidth="1"/>
-    <col min="7" max="7" width="31.54296875" customWidth="1"/>
-    <col min="8" max="16384" width="8.7265625" hidden="1"/>
+    <col min="1" max="1" width="17.109375" customWidth="1"/>
+    <col min="2" max="2" width="15.77734375" customWidth="1"/>
+    <col min="3" max="3" width="18.77734375" customWidth="1"/>
+    <col min="4" max="4" width="20.21875" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="6" max="6" width="19.5546875" customWidth="1"/>
+    <col min="7" max="7" width="31.5546875" customWidth="1"/>
+    <col min="8" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>200</v>
       </c>
@@ -7438,7 +7464,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -7458,7 +7484,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -7481,7 +7507,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
@@ -7504,7 +7530,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>1</v>
       </c>
@@ -7527,12 +7553,12 @@
         <v>475</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>0</v>
       </c>
@@ -7548,18 +7574,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA81E30-EE7D-41F0-A52A-2E2ED23F3E7D}">
   <dimension ref="A1:I50"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.55" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="3" width="17.08984375" customWidth="1"/>
-    <col min="4" max="4" width="15.7265625" customWidth="1"/>
-    <col min="5" max="5" width="19.54296875" customWidth="1"/>
-    <col min="6" max="6" width="31.54296875" customWidth="1"/>
-    <col min="7" max="8" width="8.7265625" hidden="1" customWidth="1"/>
+    <col min="1" max="3" width="17.109375" customWidth="1"/>
+    <col min="4" max="4" width="15.77734375" customWidth="1"/>
+    <col min="5" max="5" width="19.5546875" customWidth="1"/>
+    <col min="6" max="6" width="31.5546875" customWidth="1"/>
+    <col min="7" max="8" width="8.77734375" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="0" hidden="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.7265625" hidden="1"/>
+    <col min="10" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" s="6" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>200</v>
       </c>
@@ -7579,7 +7605,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -7596,7 +7622,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -7616,7 +7642,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
@@ -7633,7 +7659,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>1</v>
       </c>
@@ -7650,7 +7676,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>1</v>
       </c>
@@ -7667,7 +7693,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>0</v>
       </c>
@@ -7684,217 +7710,217 @@
         <v>439</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:1" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="9" t="b">
         <v>0</v>
       </c>
@@ -7910,17 +7936,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D615741A-82C1-4BD2-8BEF-3B31C5127744}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.453125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="21.7265625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="14.453125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="54.36328125" style="3" customWidth="1"/>
-    <col min="6" max="16384" width="8.7265625" style="3" hidden="1"/>
+    <col min="1" max="1" width="18.44140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="21.77734375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="54.33203125" style="3" customWidth="1"/>
+    <col min="6" max="16384" width="8.77734375" style="3" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>200</v>
       </c>
@@ -7937,7 +7963,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="b">
         <v>1</v>
       </c>
@@ -7954,47 +7980,47 @@
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="b">
         <v>0</v>
       </c>
@@ -8010,19 +8036,19 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{518482E7-D1DD-4AAD-BE98-FD2EBFF08ED8}">
   <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="17" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="16.90625" customWidth="1"/>
-    <col min="9" max="9" width="26.7265625" customWidth="1"/>
+    <col min="8" max="8" width="16.88671875" customWidth="1"/>
+    <col min="9" max="9" width="26.77734375" customWidth="1"/>
     <col min="10" max="10" width="0" hidden="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.7265625" hidden="1"/>
+    <col min="11" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>200</v>
       </c>
@@ -8051,7 +8077,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -8077,7 +8103,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -8097,7 +8123,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
@@ -8123,32 +8149,32 @@
         <v>287</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>0</v>
       </c>
@@ -8164,17 +8190,17 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{713F692B-7F28-45B7-9D1E-A5B0F0D04085}">
   <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="3" width="27.7265625" customWidth="1"/>
-    <col min="4" max="4" width="24.90625" customWidth="1"/>
-    <col min="5" max="5" width="55.36328125" customWidth="1"/>
+    <col min="2" max="3" width="27.77734375" customWidth="1"/>
+    <col min="4" max="4" width="24.88671875" customWidth="1"/>
+    <col min="5" max="5" width="55.33203125" customWidth="1"/>
     <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" hidden="1"/>
+    <col min="7" max="16384" width="8.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>200</v>
       </c>
@@ -8191,7 +8217,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -8205,7 +8231,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -8219,7 +8245,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
@@ -8236,7 +8262,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="b">
         <v>1</v>
       </c>
@@ -8253,7 +8279,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="b">
         <v>1</v>
       </c>
@@ -8270,7 +8296,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="b">
         <v>1</v>
       </c>
@@ -8287,7 +8313,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="b">
         <v>1</v>
       </c>
@@ -8304,7 +8330,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="b">
         <v>1</v>
       </c>
@@ -8321,7 +8347,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="b">
         <v>1</v>
       </c>
@@ -8338,7 +8364,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="b">
         <v>1</v>
       </c>
@@ -8352,7 +8378,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="b">
         <v>1</v>
       </c>
@@ -8369,7 +8395,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="b">
         <v>1</v>
       </c>
@@ -8386,87 +8412,87 @@
         <v>527</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
assigned correct part number to 1000uF cap
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE14C2BD-F928-40A3-9114-355E754769CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03AC511D-29E4-4A88-802F-A62F90A02D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="12" activeTab="18" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="1" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -39,7 +39,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Welcome!'!$A$1:$A$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -60,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="594">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="603">
   <si>
     <t>Capacitance</t>
   </si>
@@ -1625,9 +1624,6 @@
     <t>C0603C103K5RACTU</t>
   </si>
   <si>
-    <t>GCM155R71H104KE02J</t>
-  </si>
-  <si>
     <t>CL10B472KB8WPNC</t>
   </si>
   <si>
@@ -1842,6 +1838,36 @@
   </si>
   <si>
     <t>N-Channel 40 V 175A (Tj) 179W (Tc) Surface Mount PG-TDSON-8-43</t>
+  </si>
+  <si>
+    <t>CEM-1212S</t>
+  </si>
+  <si>
+    <t>Buzzers Transducer, Externally Driven Magnetic 12 V 40mA 2.4kHz 85dB @ 12V, 10cm Through Hole PC Pins</t>
+  </si>
+  <si>
+    <t>SOT-323</t>
+  </si>
+  <si>
+    <t>1.4A</t>
+  </si>
+  <si>
+    <t>160mOhm</t>
+  </si>
+  <si>
+    <t>BSS816NWH6327XTSA1</t>
+  </si>
+  <si>
+    <t>N-Channel 20 V 1.4A (Ta) 500mW (Ta) Surface Mount PG-SOT323</t>
+  </si>
+  <si>
+    <t>CT08E-16S400-2</t>
+  </si>
+  <si>
+    <t>Buzzers Transducer, Externally Driven Magnetic 12 V 80mA 4kHz 100dB @ 12V, 10cm Surface Mount Solder Pads</t>
+  </si>
+  <si>
+    <t>CL10B104KB8NNNC</t>
   </si>
 </sst>
 </file>
@@ -2158,13 +2184,6 @@
       </extLst>
     </dxf>
     <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -2341,6 +2360,13 @@
         </ext>
       </extLst>
     </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2385,13 +2411,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="77"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="76"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="75"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="75"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="74"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="74"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="73"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -2403,11 +2429,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H10" totalsRowShown="0">
   <autoFilter ref="A1:H10" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="42"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="41"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="40"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="39"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -2417,10 +2443,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="38">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="37"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -2439,7 +2465,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="77"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -2584,20 +2610,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="73">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="72">
   <autoFilter ref="A1:H50" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="72"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="71"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="70"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="69"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="68"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="67"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="66"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="65"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="71"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="70"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="69"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="65"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="64"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2620,10 +2646,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G20" totalsRowShown="0" headerRowDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G20" totalsRowShown="0" headerRowDxfId="63">
   <autoFilter ref="A1:G20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="62"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -2636,11 +2662,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="61">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="61"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="60"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="60"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="59"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -2651,25 +2677,25 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="59">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="58">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="58"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="56"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="55"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="53">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="52">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="52"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="50"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -2689,8 +2715,8 @@
     <sortCondition ref="B1:B10"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="48"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -2700,14 +2726,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="47">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="47"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3742,12 +3768,30 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>235</v>
+      </c>
+      <c r="C8" t="s">
+        <v>593</v>
+      </c>
+      <c r="D8" t="s">
+        <v>594</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>235</v>
+      </c>
+      <c r="C9" t="s">
+        <v>600</v>
+      </c>
+      <c r="D9" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -4246,10 +4290,10 @@
         <v>196</v>
       </c>
       <c r="G6" s="16" t="s">
+        <v>549</v>
+      </c>
+      <c r="H6" s="16" t="s">
         <v>550</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>551</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -4500,7 +4544,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C16" s="17">
         <f t="shared" si="0"/>
@@ -4516,10 +4560,10 @@
         <v>196</v>
       </c>
       <c r="G16" s="16" t="s">
+        <v>539</v>
+      </c>
+      <c r="H16" s="16" t="s">
         <v>540</v>
-      </c>
-      <c r="H16" s="16" t="s">
-        <v>541</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -4554,7 +4598,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="C18" s="17">
         <f t="shared" si="0"/>
@@ -4570,10 +4614,10 @@
         <v>196</v>
       </c>
       <c r="G18" s="16" t="s">
+        <v>536</v>
+      </c>
+      <c r="H18" s="16" t="s">
         <v>537</v>
-      </c>
-      <c r="H18" s="16" t="s">
-        <v>538</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
@@ -4716,7 +4760,7 @@
         <v>1</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="C24" s="17">
         <f t="shared" si="0"/>
@@ -4732,10 +4776,10 @@
         <v>196</v>
       </c>
       <c r="G24" s="16" t="s">
+        <v>533</v>
+      </c>
+      <c r="H24" s="16" t="s">
         <v>534</v>
-      </c>
-      <c r="H24" s="16" t="s">
-        <v>535</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
@@ -4905,7 +4949,7 @@
         <v>1</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C31" s="17">
         <f t="shared" si="0"/>
@@ -4921,10 +4965,10 @@
         <v>196</v>
       </c>
       <c r="G31" s="16" t="s">
+        <v>574</v>
+      </c>
+      <c r="H31" s="16" t="s">
         <v>575</v>
-      </c>
-      <c r="H31" s="16" t="s">
-        <v>576</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
@@ -4948,10 +4992,10 @@
         <v>196</v>
       </c>
       <c r="G32" s="16" t="s">
+        <v>576</v>
+      </c>
+      <c r="H32" s="16" t="s">
         <v>577</v>
-      </c>
-      <c r="H32" s="16" t="s">
-        <v>578</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
@@ -4975,10 +5019,10 @@
         <v>196</v>
       </c>
       <c r="G33" s="16" t="s">
+        <v>578</v>
+      </c>
+      <c r="H33" s="16" t="s">
         <v>579</v>
-      </c>
-      <c r="H33" s="16" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
@@ -4986,7 +5030,7 @@
         <v>1</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="C34" s="17">
         <f t="shared" ref="C34:C50" si="1">IF(ISNUMBER(B34),
@@ -5007,10 +5051,10 @@
         <v>196</v>
       </c>
       <c r="G34" s="16" t="s">
+        <v>584</v>
+      </c>
+      <c r="H34" s="16" t="s">
         <v>585</v>
-      </c>
-      <c r="H34" s="16" t="s">
-        <v>586</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
@@ -5609,7 +5653,7 @@
         <v>283</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="G1" s="21" t="s">
         <v>300</v>
@@ -5661,24 +5705,48 @@
         <v>40</v>
       </c>
       <c r="E3" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="F3" t="s">
+        <v>589</v>
+      </c>
+      <c r="G3" t="s">
         <v>590</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>591</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>592</v>
-      </c>
-      <c r="I3" t="s">
-        <v>593</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>299</v>
+      </c>
+      <c r="C4" t="s">
+        <v>301</v>
+      </c>
+      <c r="D4">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>596</v>
+      </c>
+      <c r="F4" t="s">
+        <v>597</v>
+      </c>
+      <c r="G4" t="s">
+        <v>595</v>
+      </c>
+      <c r="H4" t="s">
+        <v>598</v>
+      </c>
+      <c r="I4" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -5795,7 +5863,7 @@
         <v>9</v>
       </c>
       <c r="I2" t="s">
-        <v>521</v>
+        <v>602</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -6375,7 +6443,7 @@
         <v>9</v>
       </c>
       <c r="I22" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
@@ -6415,7 +6483,7 @@
         <v>112</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="D24" t="s">
         <v>346</v>
@@ -6433,7 +6501,7 @@
         <v>115</v>
       </c>
       <c r="I24" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
@@ -6441,7 +6509,7 @@
         <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>24</v>
@@ -6462,7 +6530,7 @@
         <v>9</v>
       </c>
       <c r="I25" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
@@ -6491,7 +6559,7 @@
         <v>9</v>
       </c>
       <c r="I26" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
@@ -6779,19 +6847,19 @@
         <v>227</v>
       </c>
       <c r="D6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="E6" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F6" t="s">
         <v>395</v>
       </c>
       <c r="G6" t="s">
+        <v>558</v>
+      </c>
+      <c r="H6" t="s">
         <v>559</v>
-      </c>
-      <c r="H6" t="s">
-        <v>560</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -7594,13 +7662,13 @@
         <v>334</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>413</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
@@ -7750,7 +7818,7 @@
         <v>334</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
@@ -7767,13 +7835,13 @@
         <v>334</v>
       </c>
       <c r="E46" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="G46" s="3" t="s">
         <v>581</v>
       </c>
-      <c r="G46" s="3" t="s">
+      <c r="H46" s="3" t="s">
         <v>582</v>
-      </c>
-      <c r="H46" s="3" t="s">
-        <v>583</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
@@ -7899,22 +7967,22 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C4" t="s">
         <v>102</v>
       </c>
       <c r="D4" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="E4" t="s">
         <v>106</v>
       </c>
       <c r="F4" t="s">
+        <v>551</v>
+      </c>
+      <c r="G4" t="s">
         <v>552</v>
-      </c>
-      <c r="G4" t="s">
-        <v>553</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -8118,22 +8186,22 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
+        <v>527</v>
+      </c>
+      <c r="C6" t="s">
         <v>528</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>529</v>
-      </c>
-      <c r="D6" t="s">
-        <v>530</v>
       </c>
       <c r="E6" t="s">
         <v>175</v>
       </c>
       <c r="F6" t="s">
+        <v>530</v>
+      </c>
+      <c r="G6" t="s">
         <v>531</v>
-      </c>
-      <c r="G6" t="s">
-        <v>532</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -8913,7 +8981,7 @@
         <v>213</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="D5" t="s">
         <v>93</v>
@@ -8930,7 +8998,7 @@
         <v>339</v>
       </c>
       <c r="C6" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="D6" t="s">
         <v>340</v>
@@ -9046,13 +9114,13 @@
         <v>339</v>
       </c>
       <c r="C13" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D13" t="s">
+        <v>525</v>
+      </c>
+      <c r="E13" t="s">
         <v>526</v>
-      </c>
-      <c r="E13" t="s">
-        <v>527</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -9060,16 +9128,16 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
+        <v>541</v>
+      </c>
+      <c r="C14" t="s">
+        <v>543</v>
+      </c>
+      <c r="D14" t="s">
         <v>542</v>
       </c>
-      <c r="C14" t="s">
+      <c r="E14" t="s">
         <v>544</v>
-      </c>
-      <c r="D14" t="s">
-        <v>543</v>
-      </c>
-      <c r="E14" t="s">
-        <v>545</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -9077,16 +9145,16 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
+        <v>545</v>
+      </c>
+      <c r="C15" t="s">
         <v>546</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>547</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>548</v>
-      </c>
-      <c r="E15" t="s">
-        <v>549</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -9094,13 +9162,13 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
+        <v>564</v>
+      </c>
+      <c r="D16" t="s">
         <v>565</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>566</v>
-      </c>
-      <c r="E16" t="s">
-        <v>567</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -9108,16 +9176,16 @@
         <v>0</v>
       </c>
       <c r="B17" t="s">
+        <v>567</v>
+      </c>
+      <c r="C17" t="s">
         <v>568</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>569</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>570</v>
-      </c>
-      <c r="E17" t="s">
-        <v>571</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
added rgb led, updated rp2350a ref design
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03AC511D-29E4-4A88-802F-A62F90A02D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0FBE42-2508-46A5-AE2C-4068FBA541A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="1" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="10" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1058" uniqueCount="607">
   <si>
     <t>Capacitance</t>
   </si>
@@ -1868,6 +1868,18 @@
   </si>
   <si>
     <t>CL10B104KB8NNNC</t>
+  </si>
+  <si>
+    <t>RGB LED</t>
+  </si>
+  <si>
+    <t>1.55x1.55mm</t>
+  </si>
+  <si>
+    <t>LTST-E143EGBW-P1</t>
+  </si>
+  <si>
+    <t>Red, Green, Blue (RGB) 623nm Red, 528nm Green, 471nm Blue LED Indication - Discrete 1.85V Red, 2.9V Green, 2.9V Blue 4-SMD, No Lead</t>
   </si>
 </sst>
 </file>
@@ -2184,6 +2196,13 @@
       </extLst>
     </dxf>
     <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -2360,13 +2379,6 @@
         </ext>
       </extLst>
     </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2411,13 +2423,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="76"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="77"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="76"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="74"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="73"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="75"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="74"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -2426,14 +2438,14 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H10" totalsRowShown="0">
-  <autoFilter ref="A1:H10" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H20" totalsRowShown="0">
+  <autoFilter ref="A1:H20" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="41"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="42"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="41"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="40"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -2443,10 +2455,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="39">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="38"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -2465,7 +2477,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="77"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="37"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -2610,20 +2622,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="72">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="73">
   <autoFilter ref="A1:H50" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="71"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="69"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="68"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="65"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="64"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="72"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="69"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="67"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="66"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2646,10 +2658,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G20" totalsRowShown="0" headerRowDxfId="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G20" totalsRowShown="0" headerRowDxfId="64">
   <autoFilter ref="A1:G20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="63"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -2662,11 +2674,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="62">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="60"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="60"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -2677,25 +2689,25 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="59">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="57"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="54"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="58"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="57"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="56"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="55"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="53">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="51"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="52"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="51"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -2715,8 +2727,8 @@
     <sortCondition ref="B1:B10"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="49"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -2726,14 +2738,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="48">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="46"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3274,7 +3286,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9362198B-44BD-4E55-B62E-439143EC0CFE}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -3521,6 +3533,77 @@
       </c>
       <c r="G10" t="s">
         <v>435</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>603</v>
+      </c>
+      <c r="C11" t="s">
+        <v>364</v>
+      </c>
+      <c r="D11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="F11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11" t="s">
+        <v>605</v>
+      </c>
+      <c r="H11" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="9" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed old zener footprint, added new SOT-123 Zener part
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC2702C8-D98E-401F-9BA1-E377C190AE91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA2AB7D-BF26-44AF-A4B2-0E63D9DF32E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="10" activeTab="15" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="2" activeTab="4" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="611">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="614">
   <si>
     <t>Capacitance</t>
   </si>
@@ -1892,6 +1892,15 @@
   </si>
   <si>
     <t>220 Ohms ±5% 0.125W, 1/8W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
+    <t>N/A, rated for 1/2W</t>
+  </si>
+  <si>
+    <t>CMHZ5232B TR PBFREE</t>
+  </si>
+  <si>
+    <t>Zener Diode 5.6 V 500 mW ±5% Surface Mount SOD-123</t>
   </si>
 </sst>
 </file>
@@ -2069,55 +2078,11 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2385,11 +2350,55 @@
       </extLst>
     </dxf>
     <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2435,13 +2444,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="76"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="67"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="66"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="74"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="73"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="64"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -2453,11 +2462,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H20" totalsRowShown="0">
   <autoFilter ref="A1:H20" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="41"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="31"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="30"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -2467,10 +2476,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="29">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="28"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -2489,7 +2498,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="27"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -2499,54 +2508,54 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="26">
   <autoFilter ref="A1:H11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="8">
-    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="33"/>
-    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="30"/>
-    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="24"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="22"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="21"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="20"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="19"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="18"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="10"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
   <autoFilter ref="A1:H50" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="C1:C50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="12"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="10">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="75"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="74"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="73">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -2554,11 +2563,11 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="72"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="71"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="70"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="69"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2568,7 +2577,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}" name="Switches" displayName="Switches" ref="A1:G11" totalsRowShown="0">
   <autoFilter ref="A1:G11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="77"/>
+    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="5"/>
     <tableColumn id="1" xr3:uid="{C868B851-3D2D-4863-96B3-5412E9A862E1}" name="Function"/>
     <tableColumn id="6" xr3:uid="{D6EA3AC7-CEF9-4E2A-800B-297C8C002273}" name="Circuit"/>
     <tableColumn id="2" xr3:uid="{5048C5E7-258E-4EC2-B0BD-C338C4D84C91}" name="Part Number"/>
@@ -2634,20 +2643,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="72">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="63">
   <autoFilter ref="A1:H50" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="71"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="69"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="68"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="65"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="64"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="62"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="61"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="60"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="59"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="57"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2670,10 +2679,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G20" totalsRowShown="0" headerRowDxfId="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G20" totalsRowShown="0" headerRowDxfId="54">
   <autoFilter ref="A1:G20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="53"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -2686,11 +2695,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="52">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="60"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="50"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -2701,25 +2710,25 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="49">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="57"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="54"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="48"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="47"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="45"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="43">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="51"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="42"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="41"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -2739,8 +2748,8 @@
     <sortCondition ref="B1:B10"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="39"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -2750,14 +2759,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="38">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="46"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8319,7 +8328,25 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>468</v>
+      </c>
+      <c r="C7" t="s">
+        <v>469</v>
+      </c>
+      <c r="D7" t="s">
+        <v>611</v>
+      </c>
+      <c r="E7" t="s">
+        <v>465</v>
+      </c>
+      <c r="F7" t="s">
+        <v>612</v>
+      </c>
+      <c r="G7" t="s">
+        <v>613</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
added new 12V reg, several new Zener diodes, several new TVS diodes
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA2AB7D-BF26-44AF-A4B2-0E63D9DF32E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32CC1E38-6C10-4D10-90CA-351392E151BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="2" activeTab="4" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="4" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1172" uniqueCount="638">
   <si>
     <t>Capacitance</t>
   </si>
@@ -1471,9 +1471,6 @@
     <t>5.6V</t>
   </si>
   <si>
-    <t>N/A, rated for 1W</t>
-  </si>
-  <si>
     <t>DO-214AC</t>
   </si>
   <si>
@@ -1642,9 +1639,6 @@
     <t>33V</t>
   </si>
   <si>
-    <t>N/A, rated for 600W</t>
-  </si>
-  <si>
     <t>SMBJ33CA</t>
   </si>
   <si>
@@ -1894,13 +1888,91 @@
     <t>220 Ohms ±5% 0.125W, 1/8W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
   </si>
   <si>
-    <t>N/A, rated for 1/2W</t>
-  </si>
-  <si>
     <t>CMHZ5232B TR PBFREE</t>
   </si>
   <si>
     <t>Zener Diode 5.6 V 500 mW ±5% Surface Mount SOD-123</t>
+  </si>
+  <si>
+    <t>Barometric Pressure Sensor</t>
+  </si>
+  <si>
+    <t>Pressure Sensor 4.35PSI ~ 18.13PSI (30kPa ~ 125kPa) Absolute 10-WFLGA</t>
+  </si>
+  <si>
+    <t>BMP581</t>
+  </si>
+  <si>
+    <t>3.5V</t>
+  </si>
+  <si>
+    <t>SOD-123F</t>
+  </si>
+  <si>
+    <t>KDZVTR3.3B</t>
+  </si>
+  <si>
+    <t>Zener Diode 3.5 V 1 W ±6.06% Surface Mount PMDU</t>
+  </si>
+  <si>
+    <t>1W</t>
+  </si>
+  <si>
+    <t>600W</t>
+  </si>
+  <si>
+    <t>Max Power</t>
+  </si>
+  <si>
+    <t>1206</t>
+  </si>
+  <si>
+    <t>HRG3216P-1000-D-T1</t>
+  </si>
+  <si>
+    <t>100 Ohms ±0.5% 1W Chip Resistor 1206 (3216 Metric) Anti-Sulfur, Automotive AEC-Q200, Moisture Resistant Thin Film</t>
+  </si>
+  <si>
+    <t>14-35V</t>
+  </si>
+  <si>
+    <t>0.1A</t>
+  </si>
+  <si>
+    <t>L78L12ACUTR</t>
+  </si>
+  <si>
+    <t>Linear Voltage Regulator IC Positive Fixed 1 Output 100mA SOT-89-3</t>
+  </si>
+  <si>
+    <t>0.33uF</t>
+  </si>
+  <si>
+    <t>CGA3E3X7R1H334K080AB</t>
+  </si>
+  <si>
+    <t>12.75V</t>
+  </si>
+  <si>
+    <t>KDZVTR12B</t>
+  </si>
+  <si>
+    <t>Zener Diode 12.75 V 1 W Surface Mount PMDU</t>
+  </si>
+  <si>
+    <t>4V</t>
+  </si>
+  <si>
+    <t>CDSOD323-T03C</t>
+  </si>
+  <si>
+    <t>SOD-323</t>
+  </si>
+  <si>
+    <t>19V (Typ) Clamp 20A (8/20µs) Ipp Tvs Diode Surface Mount SOD-323</t>
+  </si>
+  <si>
+    <t>350W</t>
   </si>
 </sst>
 </file>
@@ -2083,6 +2155,57 @@
           <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2292,16 +2415,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
@@ -2350,55 +2463,14 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2444,13 +2516,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="75"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="66"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="74"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="65"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="73"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="72"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -2462,11 +2534,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H20" totalsRowShown="0">
   <autoFilter ref="A1:H20" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="42"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="41"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="40"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -2476,10 +2548,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="39">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="38"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -2498,7 +2570,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="37"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -2508,54 +2580,54 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="36">
   <autoFilter ref="A1:H11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="8">
-    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="24"/>
-    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="15"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="19"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:H50" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="C1:C50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="75"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="74"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="73">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="11">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -2563,11 +2635,11 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="72"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="71"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="70"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="69"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2643,20 +2715,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="71">
   <autoFilter ref="A1:H50" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="62"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="57"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="56"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="55"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="70"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="68"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2679,13 +2751,14 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:G20" totalsRowShown="0" headerRowDxfId="54">
-  <autoFilter ref="A1:G20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
-  <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="53"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="77">
+  <autoFilter ref="A1:H20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
+  <tableColumns count="8">
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="76"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
+    <tableColumn id="8" xr3:uid="{66B2EB52-5AE2-4548-B193-8FF8FA377575}" name="Max Power"/>
     <tableColumn id="4" xr3:uid="{F22F5C42-5634-4AAD-A267-60DD814F054A}" name="Mount"/>
     <tableColumn id="5" xr3:uid="{181DC390-2120-46F7-9ECA-AEE686154CC2}" name="Part Number"/>
     <tableColumn id="6" xr3:uid="{C0E57478-74C4-4270-9ACE-76D0D4BB0DB3}" name="Description"/>
@@ -2695,11 +2768,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="62">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="51"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="60"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -2710,25 +2783,25 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="59">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="48"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="46"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="44"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="58"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="57"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="56"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="55"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="53">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="42"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="52"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="51"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -2748,8 +2821,8 @@
     <sortCondition ref="B1:B10"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="49"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -2759,14 +2832,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="48">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="37"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3561,7 +3634,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="C11" t="s">
         <v>362</v>
@@ -3570,16 +3643,16 @@
         <v>104</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="F11" t="s">
         <v>22</v>
       </c>
       <c r="G11" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="H11" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -3861,13 +3934,13 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
+        <v>501</v>
+      </c>
+      <c r="C7" t="s">
         <v>502</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>503</v>
-      </c>
-      <c r="D7" t="s">
-        <v>504</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -3878,10 +3951,10 @@
         <v>233</v>
       </c>
       <c r="C8" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="D8" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -3892,10 +3965,10 @@
         <v>233</v>
       </c>
       <c r="C9" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="D9" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -3952,16 +4025,16 @@
         <v>81</v>
       </c>
       <c r="D1" s="23" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F1" s="23" t="s">
+        <v>489</v>
+      </c>
+      <c r="G1" s="23" t="s">
         <v>490</v>
-      </c>
-      <c r="G1" s="23" t="s">
-        <v>491</v>
       </c>
       <c r="H1" s="23" t="s">
         <v>32</v>
@@ -3978,19 +4051,19 @@
         <v>259</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -3998,25 +4071,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>484</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>485</v>
-      </c>
       <c r="D3" s="3" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>493</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>494</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>494</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -4394,10 +4467,10 @@
         <v>194</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -4421,10 +4494,10 @@
         <v>138</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -4648,7 +4721,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="C16" s="17">
         <f t="shared" si="0"/>
@@ -4664,10 +4737,10 @@
         <v>194</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="H16" s="16" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -4702,7 +4775,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="C18" s="17">
         <f t="shared" si="0"/>
@@ -4718,10 +4791,10 @@
         <v>194</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
@@ -4864,7 +4937,7 @@
         <v>1</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="C24" s="17">
         <f t="shared" si="0"/>
@@ -4880,10 +4953,10 @@
         <v>194</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="H24" s="16" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
@@ -5053,7 +5126,7 @@
         <v>1</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="C31" s="17">
         <f t="shared" si="0"/>
@@ -5069,10 +5142,10 @@
         <v>194</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="H31" s="16" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
@@ -5096,10 +5169,10 @@
         <v>194</v>
       </c>
       <c r="G32" s="16" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="H32" s="16" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
@@ -5123,10 +5196,10 @@
         <v>194</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="H33" s="16" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
@@ -5134,7 +5207,7 @@
         <v>1</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C34" s="17">
         <f t="shared" ref="C34:C50" si="1">IF(ISNUMBER(B34),
@@ -5155,28 +5228,38 @@
         <v>194</v>
       </c>
       <c r="G34" s="16" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="H34" s="16" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B35" s="15">
-        <v>0</v>
-      </c>
-      <c r="C35" s="17" t="str">
+        <v>100</v>
+      </c>
+      <c r="C35" s="17">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="16"/>
-      <c r="H35" s="16"/>
+        <v>100</v>
+      </c>
+      <c r="D35" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E35" s="16" t="s">
+        <v>621</v>
+      </c>
+      <c r="F35" s="16" t="s">
+        <v>618</v>
+      </c>
+      <c r="G35" s="16" t="s">
+        <v>622</v>
+      </c>
+      <c r="H35" s="16" t="s">
+        <v>623</v>
+      </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="18" t="b">
@@ -5570,22 +5653,22 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="C6" t="s">
         <v>73</v>
       </c>
       <c r="D6" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="E6" t="s">
         <v>75</v>
       </c>
       <c r="F6" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="G6" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -5775,7 +5858,7 @@
         <v>281</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="G1" s="21" t="s">
         <v>298</v>
@@ -5827,19 +5910,19 @@
         <v>40</v>
       </c>
       <c r="E3" t="s">
+        <v>583</v>
+      </c>
+      <c r="F3" t="s">
         <v>585</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>586</v>
+      </c>
+      <c r="H3" t="s">
         <v>587</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>588</v>
-      </c>
-      <c r="H3" t="s">
-        <v>589</v>
-      </c>
-      <c r="I3" t="s">
-        <v>590</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -5856,19 +5939,19 @@
         <v>20</v>
       </c>
       <c r="E4" t="s">
+        <v>592</v>
+      </c>
+      <c r="F4" t="s">
+        <v>593</v>
+      </c>
+      <c r="G4" t="s">
+        <v>591</v>
+      </c>
+      <c r="H4" t="s">
         <v>594</v>
       </c>
-      <c r="F4" t="s">
+      <c r="I4" t="s">
         <v>595</v>
-      </c>
-      <c r="G4" t="s">
-        <v>593</v>
-      </c>
-      <c r="H4" t="s">
-        <v>596</v>
-      </c>
-      <c r="I4" t="s">
-        <v>597</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -5985,7 +6068,7 @@
         <v>9</v>
       </c>
       <c r="I2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -6507,7 +6590,7 @@
         <v>9</v>
       </c>
       <c r="I20" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
@@ -6515,7 +6598,7 @@
         <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>8</v>
@@ -6536,7 +6619,7 @@
         <v>9</v>
       </c>
       <c r="I21" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
@@ -6544,7 +6627,7 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>8</v>
@@ -6565,7 +6648,7 @@
         <v>9</v>
       </c>
       <c r="I22" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
@@ -6573,7 +6656,7 @@
         <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>8</v>
@@ -6594,7 +6677,7 @@
         <v>9</v>
       </c>
       <c r="I23" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
@@ -6605,7 +6688,7 @@
         <v>110</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="D24" t="s">
         <v>344</v>
@@ -6623,7 +6706,7 @@
         <v>113</v>
       </c>
       <c r="I24" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
@@ -6631,7 +6714,7 @@
         <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>24</v>
@@ -6652,7 +6735,7 @@
         <v>9</v>
       </c>
       <c r="I25" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
@@ -6681,12 +6764,36 @@
         <v>9</v>
       </c>
       <c r="I26" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B27" t="s">
+        <v>628</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" t="s">
+        <v>107</v>
+      </c>
+      <c r="E27" s="5">
+        <v>0.1</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="H27" t="s">
+        <v>9</v>
+      </c>
+      <c r="I27" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
@@ -6969,24 +7076,45 @@
         <v>225</v>
       </c>
       <c r="D6" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="E6" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="F6" t="s">
         <v>393</v>
       </c>
       <c r="G6" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="H6" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7" t="s">
+        <v>364</v>
+      </c>
+      <c r="D7" t="s">
+        <v>624</v>
+      </c>
+      <c r="E7" t="s">
+        <v>605</v>
+      </c>
+      <c r="F7" t="s">
+        <v>625</v>
+      </c>
+      <c r="G7" t="s">
+        <v>626</v>
+      </c>
+      <c r="H7" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -7265,7 +7393,7 @@
         <v>1</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C14" s="12">
         <v>3</v>
@@ -7274,13 +7402,13 @@
         <v>332</v>
       </c>
       <c r="E14" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>514</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>516</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -7288,7 +7416,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C15" s="12">
         <v>1</v>
@@ -7297,10 +7425,10 @@
         <v>203</v>
       </c>
       <c r="E15" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="H15" s="3" t="s">
         <v>498</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -7308,7 +7436,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C16" s="12">
         <v>1</v>
@@ -7317,10 +7445,10 @@
         <v>203</v>
       </c>
       <c r="E16" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>500</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -7432,13 +7560,13 @@
         <v>332</v>
       </c>
       <c r="E21" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>477</v>
       </c>
-      <c r="F21" s="3" t="s">
-        <v>478</v>
-      </c>
       <c r="H21" s="3" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
@@ -7455,16 +7583,16 @@
         <v>331</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>464</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
@@ -7784,13 +7912,13 @@
         <v>332</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>411</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
@@ -7890,7 +8018,7 @@
         <v>1</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C43" s="12">
         <v>5</v>
@@ -7899,10 +8027,10 @@
         <v>332</v>
       </c>
       <c r="E43" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="H43" s="3" t="s">
         <v>482</v>
-      </c>
-      <c r="H43" s="3" t="s">
-        <v>483</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
@@ -7931,7 +8059,7 @@
         <v>1</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C45" s="12">
         <v>5</v>
@@ -7940,7 +8068,7 @@
         <v>332</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
@@ -7957,13 +8085,13 @@
         <v>332</v>
       </c>
       <c r="E46" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="H46" s="3" t="s">
         <v>578</v>
-      </c>
-      <c r="G46" s="3" t="s">
-        <v>579</v>
-      </c>
-      <c r="H46" s="3" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
@@ -8089,22 +8217,22 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="C4" t="s">
         <v>100</v>
       </c>
       <c r="D4" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="E4" t="s">
         <v>104</v>
       </c>
       <c r="F4" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="G4" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -8178,20 +8306,21 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B0A492-FDE3-4289-9C55-9A97FFD78944}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.08984375" customWidth="1"/>
     <col min="2" max="2" width="15.7265625" customWidth="1"/>
     <col min="3" max="3" width="18.7265625" customWidth="1"/>
     <col min="4" max="4" width="20.1796875" customWidth="1"/>
-    <col min="5" max="5" width="14.6328125" customWidth="1"/>
-    <col min="6" max="6" width="19.54296875" customWidth="1"/>
-    <col min="7" max="7" width="31.54296875" customWidth="1"/>
-    <col min="8" max="16384" width="8.7265625" hidden="1"/>
+    <col min="5" max="5" width="10.6328125" customWidth="1"/>
+    <col min="6" max="6" width="14.6328125" customWidth="1"/>
+    <col min="7" max="7" width="19.54296875" customWidth="1"/>
+    <col min="8" max="8" width="31.54296875" customWidth="1"/>
+    <col min="9" max="16384" width="8.7265625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>198</v>
       </c>
@@ -8205,16 +8334,19 @@
         <v>115</v>
       </c>
       <c r="E1" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -8227,14 +8359,14 @@
       <c r="D2" t="s">
         <v>120</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>121</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -8247,17 +8379,17 @@
       <c r="D3" t="s">
         <v>172</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>173</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>174</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
@@ -8270,17 +8402,17 @@
       <c r="D4" t="s">
         <v>172</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>465</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>466</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="b">
         <v>1</v>
       </c>
@@ -8290,43 +8422,43 @@
       <c r="C5" t="s">
         <v>469</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>618</v>
+      </c>
+      <c r="F5" t="s">
         <v>470</v>
       </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>471</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>472</v>
       </c>
-      <c r="G5" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B6" t="s">
+        <v>524</v>
+      </c>
+      <c r="C6" t="s">
         <v>525</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
+        <v>619</v>
+      </c>
+      <c r="F6" t="s">
+        <v>173</v>
+      </c>
+      <c r="G6" t="s">
         <v>526</v>
       </c>
-      <c r="D6" t="s">
+      <c r="H6" t="s">
         <v>527</v>
       </c>
-      <c r="E6" t="s">
-        <v>173</v>
-      </c>
-      <c r="F6" t="s">
-        <v>528</v>
-      </c>
-      <c r="G6" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="b">
         <v>1</v>
       </c>
@@ -8336,60 +8468,114 @@
       <c r="C7" t="s">
         <v>469</v>
       </c>
-      <c r="D7" t="s">
-        <v>611</v>
-      </c>
       <c r="E7" t="s">
+        <v>287</v>
+      </c>
+      <c r="F7" t="s">
         <v>465</v>
       </c>
-      <c r="F7" t="s">
-        <v>612</v>
-      </c>
       <c r="G7" t="s">
-        <v>613</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+        <v>609</v>
+      </c>
+      <c r="H7" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>468</v>
+      </c>
+      <c r="C8" t="s">
+        <v>614</v>
+      </c>
+      <c r="E8" t="s">
+        <v>618</v>
+      </c>
+      <c r="F8" t="s">
+        <v>615</v>
+      </c>
+      <c r="G8" t="s">
+        <v>616</v>
+      </c>
+      <c r="H8" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>468</v>
+      </c>
+      <c r="C9" t="s">
+        <v>630</v>
+      </c>
+      <c r="E9" t="s">
+        <v>618</v>
+      </c>
+      <c r="F9" t="s">
+        <v>615</v>
+      </c>
+      <c r="G9" t="s">
+        <v>631</v>
+      </c>
+      <c r="H9" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>524</v>
+      </c>
+      <c r="C10" t="s">
+        <v>633</v>
+      </c>
+      <c r="E10" t="s">
+        <v>637</v>
+      </c>
+      <c r="F10" t="s">
+        <v>635</v>
+      </c>
+      <c r="G10" t="s">
+        <v>634</v>
+      </c>
+      <c r="H10" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="b">
         <v>0</v>
       </c>
@@ -9121,7 +9307,7 @@
         <v>211</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D5" t="s">
         <v>91</v>
@@ -9138,7 +9324,7 @@
         <v>337</v>
       </c>
       <c r="C6" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="D6" t="s">
         <v>338</v>
@@ -9220,13 +9406,13 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
+        <v>473</v>
+      </c>
+      <c r="D11" t="s">
         <v>474</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>475</v>
-      </c>
-      <c r="E11" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -9234,16 +9420,16 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
+        <v>508</v>
+      </c>
+      <c r="C12" t="s">
         <v>509</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>510</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>511</v>
-      </c>
-      <c r="E12" t="s">
-        <v>512</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -9254,13 +9440,13 @@
         <v>337</v>
       </c>
       <c r="C13" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="D13" t="s">
+        <v>522</v>
+      </c>
+      <c r="E13" t="s">
         <v>523</v>
-      </c>
-      <c r="E13" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -9268,16 +9454,16 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
+        <v>537</v>
+      </c>
+      <c r="C14" t="s">
         <v>539</v>
       </c>
-      <c r="C14" t="s">
-        <v>541</v>
-      </c>
       <c r="D14" t="s">
+        <v>538</v>
+      </c>
+      <c r="E14" t="s">
         <v>540</v>
-      </c>
-      <c r="E14" t="s">
-        <v>542</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -9285,16 +9471,16 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
+        <v>541</v>
+      </c>
+      <c r="C15" t="s">
+        <v>542</v>
+      </c>
+      <c r="D15" t="s">
         <v>543</v>
       </c>
-      <c r="C15" t="s">
+      <c r="E15" t="s">
         <v>544</v>
-      </c>
-      <c r="D15" t="s">
-        <v>545</v>
-      </c>
-      <c r="E15" t="s">
-        <v>546</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -9302,35 +9488,44 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
+        <v>560</v>
+      </c>
+      <c r="D16" t="s">
+        <v>561</v>
+      </c>
+      <c r="E16" t="s">
         <v>562</v>
-      </c>
-      <c r="D16" t="s">
-        <v>563</v>
-      </c>
-      <c r="E16" t="s">
-        <v>564</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="s">
+        <v>563</v>
+      </c>
+      <c r="C17" t="s">
+        <v>564</v>
+      </c>
+      <c r="D17" t="s">
         <v>565</v>
       </c>
-      <c r="C17" t="s">
+      <c r="E17" t="s">
         <v>566</v>
-      </c>
-      <c r="D17" t="s">
-        <v>567</v>
-      </c>
-      <c r="E17" t="s">
-        <v>568</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B18" t="s">
+        <v>611</v>
+      </c>
+      <c r="D18" t="s">
+        <v>613</v>
+      </c>
+      <c r="E18" t="s">
+        <v>612</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
added new 12bit single-ended ADC
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC5DB1E5-4DE5-4B02-A0F2-2FEA76FF2314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79ABEEC2-C59E-4644-8F95-E43D27D06BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="15" activeTab="16" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="8" activeTab="8" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1121" uniqueCount="647">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="650">
   <si>
     <t>Capacitance</t>
   </si>
@@ -1978,9 +1978,6 @@
     <t>ADC</t>
   </si>
   <si>
-    <t>18bit resolution, ~2.7-5.5V</t>
-  </si>
-  <si>
     <t>MCP3421A3T-E/CH</t>
   </si>
   <si>
@@ -2000,6 +1997,18 @@
   </si>
   <si>
     <t>3 Position Terminal Block Header, Male Pins, Shrouded (4 Side) 0.098" (2.50mm) 90°, Right Angle Surface Mount</t>
+  </si>
+  <si>
+    <t>12bit resolution, single-ended, ~2.7-5.5V</t>
+  </si>
+  <si>
+    <t>18bit resolution, differential, ~2.7-5.5V</t>
+  </si>
+  <si>
+    <t>MCP3221A0T-E/OT</t>
+  </si>
+  <si>
+    <t>12 Bit Analog to Digital Converter 1 Input 1 SAR SOT-23-5</t>
   </si>
 </sst>
 </file>
@@ -2175,13 +2184,6 @@
           <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -2461,22 +2463,6 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
@@ -2498,6 +2484,29 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2543,13 +2552,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="76"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="75"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="65"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="74"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="73"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -2561,11 +2570,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H20" totalsRowShown="0">
   <autoFilter ref="A1:H20" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="42"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="41"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="40"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="39"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -2575,10 +2584,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="38">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="37"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -2597,7 +2606,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="36"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -2607,54 +2616,54 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="35">
   <autoFilter ref="A1:H11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="8">
-    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="34"/>
-    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="31"/>
-    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="25"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="20"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="19"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="22"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="20"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="19"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="18"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
   <autoFilter ref="A1:H50" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="C1:C50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="13"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="11">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="10">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -2662,11 +2671,11 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2676,7 +2685,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}" name="Switches" displayName="Switches" ref="A1:G11" totalsRowShown="0">
   <autoFilter ref="A1:G11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="77"/>
     <tableColumn id="1" xr3:uid="{C868B851-3D2D-4863-96B3-5412E9A862E1}" name="Function"/>
     <tableColumn id="6" xr3:uid="{D6EA3AC7-CEF9-4E2A-800B-297C8C002273}" name="Circuit"/>
     <tableColumn id="2" xr3:uid="{5048C5E7-258E-4EC2-B0BD-C338C4D84C91}" name="Part Number"/>
@@ -2742,20 +2751,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="77">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="72">
   <autoFilter ref="A1:H50" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="76"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="72"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="71"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="70"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="69"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="71"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="70"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="69"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="65"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="64"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2778,10 +2787,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="63">
   <autoFilter ref="A1:H20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="62"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -2795,11 +2804,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="61">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="61"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="60"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="60"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="59"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -2810,25 +2819,25 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="59">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="58">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="58"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="56"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="55"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="53">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="52">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="52"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="50"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -2848,8 +2857,8 @@
     <sortCondition ref="B1:B10"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="48"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -2859,14 +2868,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="47">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="47"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8126,7 +8135,7 @@
         <v>1</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="C47" s="12">
         <v>3</v>
@@ -8135,16 +8144,16 @@
         <v>332</v>
       </c>
       <c r="E47" s="3" t="s">
+        <v>642</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>644</v>
+      </c>
+      <c r="G47" s="3" t="s">
         <v>643</v>
       </c>
-      <c r="F47" s="3" t="s">
+      <c r="H47" s="3" t="s">
         <v>645</v>
-      </c>
-      <c r="G47" s="3" t="s">
-        <v>644</v>
-      </c>
-      <c r="H47" s="3" t="s">
-        <v>646</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
@@ -9583,18 +9592,30 @@
         <v>638</v>
       </c>
       <c r="C19" t="s">
+        <v>647</v>
+      </c>
+      <c r="D19" t="s">
         <v>639</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>640</v>
-      </c>
-      <c r="E19" t="s">
-        <v>641</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B20" t="s">
+        <v>638</v>
+      </c>
+      <c r="C20" t="s">
+        <v>646</v>
+      </c>
+      <c r="D20" t="s">
+        <v>648</v>
+      </c>
+      <c r="E20" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
created new parts for modem board stack
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79ABEEC2-C59E-4644-8F95-E43D27D06BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672E2545-7E40-45BC-BFF7-E5DBDDCD145F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="8" activeTab="8" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="41805" yWindow="30" windowWidth="19110" windowHeight="11175" firstSheet="3" activeTab="6" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -19,9 +19,9 @@
     <sheet name="Crystals &amp; Oscillators" sheetId="7" r:id="rId4"/>
     <sheet name="Diodes" sheetId="13" r:id="rId5"/>
     <sheet name="Devices" sheetId="16" r:id="rId6"/>
-    <sheet name="Ferrite Beads" sheetId="10" r:id="rId7"/>
-    <sheet name="Fuses" sheetId="8" r:id="rId8"/>
-    <sheet name="ICs" sheetId="12" r:id="rId9"/>
+    <sheet name="ICs" sheetId="12" r:id="rId7"/>
+    <sheet name="Ferrite Beads" sheetId="10" r:id="rId8"/>
+    <sheet name="Fuses" sheetId="8" r:id="rId9"/>
     <sheet name="Inductors" sheetId="3" r:id="rId10"/>
     <sheet name="LEDs" sheetId="5" r:id="rId11"/>
     <sheet name="Memory" sheetId="17" r:id="rId12"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="650">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="678">
   <si>
     <t>Capacitance</t>
   </si>
@@ -2009,6 +2009,90 @@
   </si>
   <si>
     <t>12 Bit Analog to Digital Converter 1 Input 1 SAR SOT-23-5</t>
+  </si>
+  <si>
+    <t>1778764</t>
+  </si>
+  <si>
+    <t>1778832</t>
+  </si>
+  <si>
+    <t>2 Position Terminal Block Header, Male Pins, Shrouded (4 Side) 0.098" (2.50mm) 90°, Right Angle Surface Mount</t>
+  </si>
+  <si>
+    <t>280389-2</t>
+  </si>
+  <si>
+    <t>280365</t>
+  </si>
+  <si>
+    <t>2.54mm pitch</t>
+  </si>
+  <si>
+    <t>Connector Header Through Hole, Right Angle 8 position 0.100" (2.54mm)</t>
+  </si>
+  <si>
+    <t>Rectangular</t>
+  </si>
+  <si>
+    <t>15-40V</t>
+  </si>
+  <si>
+    <t>XL1509-12-EV</t>
+  </si>
+  <si>
+    <t>Buck Switching Regulator IC Positive Fixed 12V 1 Output 3A 8-SOIC (0.154", 3.90mm Width)</t>
+  </si>
+  <si>
+    <t>100uF</t>
+  </si>
+  <si>
+    <t>EEE-FT1V101AP</t>
+  </si>
+  <si>
+    <t>68uH</t>
+  </si>
+  <si>
+    <t>SMD 10.85 x 10.2mm</t>
+  </si>
+  <si>
+    <t>VSHB1060T-680MC</t>
+  </si>
+  <si>
+    <t>68 µH Shielded Wirewound Inductor 3.7 A 115mOhm Max 2-SMD Low DCR, Low Loss, Soft Saturation</t>
+  </si>
+  <si>
+    <t>60V</t>
+  </si>
+  <si>
+    <t>SK36A-LTP</t>
+  </si>
+  <si>
+    <t>Diode 60 V 3A Surface Mount DO-214AC (SMA)</t>
+  </si>
+  <si>
+    <t>180W</t>
+  </si>
+  <si>
+    <t>120W</t>
+  </si>
+  <si>
+    <t>1000W</t>
+  </si>
+  <si>
+    <t>40W</t>
+  </si>
+  <si>
+    <t>Bridge (UART-RS232)</t>
+  </si>
+  <si>
+    <t>MAX3232ECDR</t>
+  </si>
+  <si>
+    <t>2/2 Transceiver Full RS232 16-SOIC</t>
+  </si>
+  <si>
+    <t>2 channels</t>
   </si>
 </sst>
 </file>
@@ -2184,6 +2268,13 @@
           <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -2382,20 +2473,6 @@
       </extLst>
     </dxf>
     <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -2508,6 +2585,13 @@
         </ext>
       </extLst>
     </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2552,13 +2636,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="76"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="75"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="74"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="74"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="73"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="73"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="72"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -2570,11 +2654,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H20" totalsRowShown="0">
   <autoFilter ref="A1:H20" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="41"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="42"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="41"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="40"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -2584,10 +2668,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="39">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="38"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -2606,7 +2690,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="37"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -2616,54 +2700,54 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="36">
   <autoFilter ref="A1:H11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="8">
-    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="33"/>
-    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="30"/>
-    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="24"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="22"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="21"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="20"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="19"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="18"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="19"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:H50" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="C1:C50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="12"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="10">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="11">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -2671,11 +2755,11 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2685,7 +2769,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}" name="Switches" displayName="Switches" ref="A1:G11" totalsRowShown="0">
   <autoFilter ref="A1:G11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="77"/>
+    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="5"/>
     <tableColumn id="1" xr3:uid="{C868B851-3D2D-4863-96B3-5412E9A862E1}" name="Function"/>
     <tableColumn id="6" xr3:uid="{D6EA3AC7-CEF9-4E2A-800B-297C8C002273}" name="Circuit"/>
     <tableColumn id="2" xr3:uid="{5048C5E7-258E-4EC2-B0BD-C338C4D84C91}" name="Part Number"/>
@@ -2751,20 +2835,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="72">
-  <autoFilter ref="A1:H50" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="71">
+  <autoFilter ref="A1:H100" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="71"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="69"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="68"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="65"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="64"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="70"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="68"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2787,10 +2871,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="62">
   <autoFilter ref="A1:H20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H20">
+    <sortCondition ref="B1:B20"/>
+  </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="61"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -2804,11 +2891,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="60">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="60"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="59"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="58"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -2819,25 +2906,42 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}" name="ICs" displayName="ICs" ref="A1:E30" totalsRowShown="0">
+  <autoFilter ref="A1:E30" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E10">
+    <sortCondition ref="B1:B10"/>
+  </sortState>
+  <tableColumns count="5">
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="77"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="76"/>
+    <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
+    <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="57">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="57"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="54"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="56"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="54"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="52">
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="51">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="51"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="49"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -2850,32 +2954,15 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}" name="ICs" displayName="ICs" ref="A1:E30" totalsRowShown="0">
-  <autoFilter ref="A1:E30" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E10">
-    <sortCondition ref="B1:B10"/>
-  </sortState>
-  <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="48"/>
-    <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
-    <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
-    <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="48">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="46"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3373,7 +3460,19 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>663</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>665</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>666</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -6834,7 +6933,31 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B28" t="s">
+        <v>661</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="D28" t="s">
+        <v>344</v>
+      </c>
+      <c r="E28" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="H28" t="s">
+        <v>113</v>
+      </c>
+      <c r="I28" t="s">
+        <v>662</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
@@ -7155,7 +7278,28 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>144</v>
+      </c>
+      <c r="C8" t="s">
+        <v>225</v>
+      </c>
+      <c r="D8" t="s">
+        <v>658</v>
+      </c>
+      <c r="E8" t="s">
+        <v>605</v>
+      </c>
+      <c r="F8" t="s">
+        <v>120</v>
+      </c>
+      <c r="G8" t="s">
+        <v>659</v>
+      </c>
+      <c r="H8" t="s">
+        <v>660</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -7188,7 +7332,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31311A32-7C4D-4571-8105-957397FF3475}">
-  <dimension ref="A1:XDX50"/>
+  <dimension ref="A1:XDX100"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.1796875" style="3" customWidth="1"/>
@@ -7722,7 +7866,7 @@
         <v>1</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>206</v>
+        <v>657</v>
       </c>
       <c r="C27" s="12">
         <v>10</v>
@@ -7765,7 +7909,7 @@
         <v>1</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>206</v>
+        <v>657</v>
       </c>
       <c r="C29" s="12">
         <v>16</v>
@@ -8158,21 +8302,361 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C48" s="12"/>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="C48" s="12">
+        <v>2</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>651</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>643</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="C49" s="12"/>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B49" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="C49" s="12">
+        <v>8</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C50" s="12"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A51" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C51" s="12"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A52" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C52" s="12"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A53" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C53" s="12"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A54" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C54" s="12"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A55" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C55" s="12"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A56" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C56" s="12"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A57" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C57" s="12"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A58" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C58" s="12"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A59" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C59" s="12"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A60" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C60" s="12"/>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A61" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C61" s="12"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A62" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C62" s="12"/>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A63" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C63" s="12"/>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A64" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C64" s="12"/>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C65" s="12"/>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C66" s="12"/>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C67" s="12"/>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C68" s="12"/>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C69" s="12"/>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A70" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C70" s="12"/>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A71" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C71" s="12"/>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A72" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C72" s="12"/>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A73" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C73" s="12"/>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A74" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C74" s="12"/>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A75" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C75" s="12"/>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A76" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C76" s="12"/>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A77" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C77" s="12"/>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A78" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C78" s="12"/>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A79" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C79" s="12"/>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A80" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C80" s="12"/>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A81" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C81" s="12"/>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A82" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C82" s="12"/>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A83" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C83" s="12"/>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A84" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C84" s="12"/>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A85" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C85" s="12"/>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A86" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C86" s="12"/>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A87" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C87" s="12"/>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A88" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C88" s="12"/>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A89" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C89" s="12"/>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A90" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C90" s="12"/>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A91" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C91" s="12"/>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A92" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C92" s="12"/>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A93" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C93" s="12"/>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A94" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C94" s="12"/>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A95" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C95" s="12"/>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A96" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C96" s="12"/>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A97" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C97" s="12"/>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A98" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C98" s="12"/>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A99" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C99" s="12"/>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A100" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="C100" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8407,19 +8891,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>170</v>
       </c>
       <c r="C2" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="D2" t="s">
-        <v>120</v>
+        <v>172</v>
+      </c>
+      <c r="E2" t="s">
+        <v>672</v>
       </c>
       <c r="F2" t="s">
-        <v>121</v>
+        <v>173</v>
       </c>
       <c r="G2" t="s">
-        <v>122</v>
+        <v>174</v>
+      </c>
+      <c r="H2" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -8427,22 +8917,22 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>170</v>
+        <v>117</v>
       </c>
       <c r="C3" t="s">
-        <v>171</v>
+        <v>118</v>
       </c>
       <c r="D3" t="s">
-        <v>172</v>
+        <v>120</v>
+      </c>
+      <c r="E3" t="s">
+        <v>671</v>
       </c>
       <c r="F3" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="G3" t="s">
-        <v>174</v>
-      </c>
-      <c r="H3" t="s">
-        <v>175</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -8458,6 +8948,9 @@
       <c r="D4" t="s">
         <v>172</v>
       </c>
+      <c r="E4" t="s">
+        <v>673</v>
+      </c>
       <c r="F4" t="s">
         <v>465</v>
       </c>
@@ -8473,22 +8966,25 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>468</v>
+        <v>117</v>
       </c>
       <c r="C5" t="s">
-        <v>469</v>
+        <v>667</v>
+      </c>
+      <c r="D5" t="s">
+        <v>120</v>
       </c>
       <c r="E5" t="s">
-        <v>618</v>
+        <v>670</v>
       </c>
       <c r="F5" t="s">
         <v>470</v>
       </c>
       <c r="G5" t="s">
-        <v>471</v>
+        <v>668</v>
       </c>
       <c r="H5" t="s">
-        <v>472</v>
+        <v>669</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -8519,22 +9015,22 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>468</v>
+        <v>524</v>
       </c>
       <c r="C7" t="s">
-        <v>469</v>
+        <v>633</v>
       </c>
       <c r="E7" t="s">
-        <v>287</v>
+        <v>637</v>
       </c>
       <c r="F7" t="s">
-        <v>465</v>
+        <v>635</v>
       </c>
       <c r="G7" t="s">
-        <v>609</v>
+        <v>634</v>
       </c>
       <c r="H7" t="s">
-        <v>610</v>
+        <v>636</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -8545,19 +9041,19 @@
         <v>468</v>
       </c>
       <c r="C8" t="s">
-        <v>614</v>
+        <v>469</v>
       </c>
       <c r="E8" t="s">
         <v>618</v>
       </c>
       <c r="F8" t="s">
-        <v>615</v>
+        <v>470</v>
       </c>
       <c r="G8" t="s">
-        <v>616</v>
+        <v>471</v>
       </c>
       <c r="H8" t="s">
-        <v>617</v>
+        <v>472</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -8568,19 +9064,19 @@
         <v>468</v>
       </c>
       <c r="C9" t="s">
-        <v>630</v>
+        <v>469</v>
       </c>
       <c r="E9" t="s">
-        <v>618</v>
+        <v>287</v>
       </c>
       <c r="F9" t="s">
-        <v>615</v>
+        <v>465</v>
       </c>
       <c r="G9" t="s">
-        <v>631</v>
+        <v>609</v>
       </c>
       <c r="H9" t="s">
-        <v>632</v>
+        <v>610</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -8588,27 +9084,45 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>524</v>
+        <v>468</v>
       </c>
       <c r="C10" t="s">
-        <v>633</v>
+        <v>614</v>
       </c>
       <c r="E10" t="s">
-        <v>637</v>
+        <v>618</v>
       </c>
       <c r="F10" t="s">
-        <v>635</v>
+        <v>615</v>
       </c>
       <c r="G10" t="s">
-        <v>634</v>
+        <v>616</v>
       </c>
       <c r="H10" t="s">
-        <v>636</v>
+        <v>617</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>468</v>
+      </c>
+      <c r="C11" t="s">
+        <v>630</v>
+      </c>
+      <c r="E11" t="s">
+        <v>618</v>
+      </c>
+      <c r="F11" t="s">
+        <v>615</v>
+      </c>
+      <c r="G11" t="s">
+        <v>631</v>
+      </c>
+      <c r="H11" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -9027,6 +9541,414 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{713F692B-7F28-45B7-9D1E-A5B0F0D04085}">
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="3" width="27.7265625" customWidth="1"/>
+    <col min="4" max="4" width="24.90625" customWidth="1"/>
+    <col min="5" max="5" width="55.36328125" customWidth="1"/>
+    <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.7265625" hidden="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" t="s">
+        <v>209</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>212</v>
+      </c>
+      <c r="D2" t="s">
+        <v>168</v>
+      </c>
+      <c r="E2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>308</v>
+      </c>
+      <c r="D3" t="s">
+        <v>307</v>
+      </c>
+      <c r="E3" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" t="s">
+        <v>210</v>
+      </c>
+      <c r="D4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="D5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C6" t="s">
+        <v>520</v>
+      </c>
+      <c r="D6" t="s">
+        <v>338</v>
+      </c>
+      <c r="E6" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>315</v>
+      </c>
+      <c r="C7" t="s">
+        <v>316</v>
+      </c>
+      <c r="D7" t="s">
+        <v>317</v>
+      </c>
+      <c r="E7" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>323</v>
+      </c>
+      <c r="C8" t="s">
+        <v>324</v>
+      </c>
+      <c r="D8" t="s">
+        <v>325</v>
+      </c>
+      <c r="E8" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" t="s">
+        <v>380</v>
+      </c>
+      <c r="D9" t="s">
+        <v>381</v>
+      </c>
+      <c r="E9" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>420</v>
+      </c>
+      <c r="C10" t="s">
+        <v>423</v>
+      </c>
+      <c r="D10" t="s">
+        <v>421</v>
+      </c>
+      <c r="E10" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>473</v>
+      </c>
+      <c r="D11" t="s">
+        <v>474</v>
+      </c>
+      <c r="E11" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" t="s">
+        <v>508</v>
+      </c>
+      <c r="C12" t="s">
+        <v>509</v>
+      </c>
+      <c r="D12" t="s">
+        <v>510</v>
+      </c>
+      <c r="E12" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
+        <v>337</v>
+      </c>
+      <c r="C13" t="s">
+        <v>519</v>
+      </c>
+      <c r="D13" t="s">
+        <v>522</v>
+      </c>
+      <c r="E13" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B14" t="s">
+        <v>537</v>
+      </c>
+      <c r="C14" t="s">
+        <v>539</v>
+      </c>
+      <c r="D14" t="s">
+        <v>538</v>
+      </c>
+      <c r="E14" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" t="s">
+        <v>541</v>
+      </c>
+      <c r="C15" t="s">
+        <v>542</v>
+      </c>
+      <c r="D15" t="s">
+        <v>543</v>
+      </c>
+      <c r="E15" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" t="s">
+        <v>560</v>
+      </c>
+      <c r="D16" t="s">
+        <v>561</v>
+      </c>
+      <c r="E16" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" t="s">
+        <v>563</v>
+      </c>
+      <c r="C17" t="s">
+        <v>564</v>
+      </c>
+      <c r="D17" t="s">
+        <v>565</v>
+      </c>
+      <c r="E17" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" t="s">
+        <v>611</v>
+      </c>
+      <c r="D18" t="s">
+        <v>613</v>
+      </c>
+      <c r="E18" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" t="s">
+        <v>638</v>
+      </c>
+      <c r="C19" t="s">
+        <v>647</v>
+      </c>
+      <c r="D19" t="s">
+        <v>639</v>
+      </c>
+      <c r="E19" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" t="s">
+        <v>638</v>
+      </c>
+      <c r="C20" t="s">
+        <v>646</v>
+      </c>
+      <c r="D20" t="s">
+        <v>648</v>
+      </c>
+      <c r="E20" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B21" t="s">
+        <v>674</v>
+      </c>
+      <c r="C21" t="s">
+        <v>677</v>
+      </c>
+      <c r="D21" t="s">
+        <v>675</v>
+      </c>
+      <c r="E21" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D615741A-82C1-4BD2-8BEF-3B31C5127744}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
@@ -9126,7 +10048,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{518482E7-D1DD-4AAD-BE98-FD2EBFF08ED8}">
   <dimension ref="A1:J10"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
@@ -9278,400 +10200,4 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{713F692B-7F28-45B7-9D1E-A5B0F0D04085}">
-  <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="3" width="27.7265625" customWidth="1"/>
-    <col min="4" max="4" width="24.90625" customWidth="1"/>
-    <col min="5" max="5" width="55.36328125" customWidth="1"/>
-    <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" hidden="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>198</v>
-      </c>
-      <c r="B1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C1" t="s">
-        <v>209</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>212</v>
-      </c>
-      <c r="D2" t="s">
-        <v>168</v>
-      </c>
-      <c r="E2" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>308</v>
-      </c>
-      <c r="D3" t="s">
-        <v>307</v>
-      </c>
-      <c r="E3" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" t="s">
-        <v>210</v>
-      </c>
-      <c r="D4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>521</v>
-      </c>
-      <c r="D5" t="s">
-        <v>91</v>
-      </c>
-      <c r="E5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B6" t="s">
-        <v>337</v>
-      </c>
-      <c r="C6" t="s">
-        <v>520</v>
-      </c>
-      <c r="D6" t="s">
-        <v>338</v>
-      </c>
-      <c r="E6" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B7" t="s">
-        <v>315</v>
-      </c>
-      <c r="C7" t="s">
-        <v>316</v>
-      </c>
-      <c r="D7" t="s">
-        <v>317</v>
-      </c>
-      <c r="E7" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B8" t="s">
-        <v>323</v>
-      </c>
-      <c r="C8" t="s">
-        <v>324</v>
-      </c>
-      <c r="D8" t="s">
-        <v>325</v>
-      </c>
-      <c r="E8" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B9" t="s">
-        <v>80</v>
-      </c>
-      <c r="C9" t="s">
-        <v>380</v>
-      </c>
-      <c r="D9" t="s">
-        <v>381</v>
-      </c>
-      <c r="E9" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" t="s">
-        <v>420</v>
-      </c>
-      <c r="C10" t="s">
-        <v>423</v>
-      </c>
-      <c r="D10" t="s">
-        <v>421</v>
-      </c>
-      <c r="E10" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B11" t="s">
-        <v>473</v>
-      </c>
-      <c r="D11" t="s">
-        <v>474</v>
-      </c>
-      <c r="E11" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B12" t="s">
-        <v>508</v>
-      </c>
-      <c r="C12" t="s">
-        <v>509</v>
-      </c>
-      <c r="D12" t="s">
-        <v>510</v>
-      </c>
-      <c r="E12" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B13" t="s">
-        <v>337</v>
-      </c>
-      <c r="C13" t="s">
-        <v>519</v>
-      </c>
-      <c r="D13" t="s">
-        <v>522</v>
-      </c>
-      <c r="E13" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B14" t="s">
-        <v>537</v>
-      </c>
-      <c r="C14" t="s">
-        <v>539</v>
-      </c>
-      <c r="D14" t="s">
-        <v>538</v>
-      </c>
-      <c r="E14" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B15" t="s">
-        <v>541</v>
-      </c>
-      <c r="C15" t="s">
-        <v>542</v>
-      </c>
-      <c r="D15" t="s">
-        <v>543</v>
-      </c>
-      <c r="E15" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B16" t="s">
-        <v>560</v>
-      </c>
-      <c r="D16" t="s">
-        <v>561</v>
-      </c>
-      <c r="E16" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B17" t="s">
-        <v>563</v>
-      </c>
-      <c r="C17" t="s">
-        <v>564</v>
-      </c>
-      <c r="D17" t="s">
-        <v>565</v>
-      </c>
-      <c r="E17" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B18" t="s">
-        <v>611</v>
-      </c>
-      <c r="D18" t="s">
-        <v>613</v>
-      </c>
-      <c r="E18" t="s">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B19" t="s">
-        <v>638</v>
-      </c>
-      <c r="C19" t="s">
-        <v>647</v>
-      </c>
-      <c r="D19" t="s">
-        <v>639</v>
-      </c>
-      <c r="E19" t="s">
-        <v>640</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B20" t="s">
-        <v>638</v>
-      </c>
-      <c r="C20" t="s">
-        <v>646</v>
-      </c>
-      <c r="D20" t="s">
-        <v>648</v>
-      </c>
-      <c r="E20" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
New parts, created spreadsheet for parts storage JSON data
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672E2545-7E40-45BC-BFF7-E5DBDDCD145F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E36CDF2-540D-4CF0-B628-1D5C8CF94C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41805" yWindow="30" windowWidth="19110" windowHeight="11175" firstSheet="3" activeTab="6" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="6" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1180" uniqueCount="684">
   <si>
     <t>Capacitance</t>
   </si>
@@ -2093,6 +2093,24 @@
   </si>
   <si>
     <t>2 channels</t>
+  </si>
+  <si>
+    <t>0.47uF</t>
+  </si>
+  <si>
+    <t>TMK107B7474KA-TR</t>
+  </si>
+  <si>
+    <t>GNSS</t>
+  </si>
+  <si>
+    <t>Triple-band, RTK, PPP-RTK</t>
+  </si>
+  <si>
+    <t>ZED-F20P-00B</t>
+  </si>
+  <si>
+    <t>- RF Receiver BeiDou, Galileo, GNSS, GPS, QZSS, SBAS -167dBm 8Mbps Not Included 54-LGA (22x17)</t>
   </si>
 </sst>
 </file>
@@ -2506,6 +2524,20 @@
     <dxf>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
@@ -2578,20 +2610,6 @@
         </ext>
       </extLst>
     </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2636,13 +2654,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="75"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="77"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="74"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="76"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="73"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="72"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="75"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="74"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -2835,20 +2853,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="73">
   <autoFilter ref="A1:H100" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="70"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="69"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="68"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="67"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="66"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="65"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="72"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="69"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="67"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="66"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2871,13 +2889,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="64">
   <autoFilter ref="A1:H20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H20">
     <sortCondition ref="B1:B20"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="61"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="63"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -2891,11 +2909,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="60">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="62">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="59"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="58"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="60"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -2912,8 +2930,8 @@
     <sortCondition ref="B1:B10"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="77"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="76"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="59"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="58"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -6962,7 +6980,31 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B29" t="s">
+        <v>678</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" t="s">
+        <v>18</v>
+      </c>
+      <c r="E29" s="5">
+        <v>0.1</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="H29" t="s">
+        <v>9</v>
+      </c>
+      <c r="I29" t="s">
+        <v>679</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
@@ -9897,7 +9939,19 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B22" t="s">
+        <v>680</v>
+      </c>
+      <c r="C22" t="s">
+        <v>681</v>
+      </c>
+      <c r="D22" t="s">
+        <v>682</v>
+      </c>
+      <c r="E22" t="s">
+        <v>683</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
updates to parts storage, new parts
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46FA153-7A13-48E9-8A27-861D10DEABF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E03495-11E2-430C-B94A-28BEA21669A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="2" activeTab="2" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="2" activeTab="5" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1223" uniqueCount="716">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1243" uniqueCount="730">
   <si>
     <t>Capacitance</t>
   </si>
@@ -2207,6 +2207,48 @@
   </si>
   <si>
     <t>SMA Connector Jack, Female Socket 50 Ohms Through Hole, Right Angle Solder</t>
+  </si>
+  <si>
+    <t>Illumination LED</t>
+  </si>
+  <si>
+    <t>1414</t>
+  </si>
+  <si>
+    <t>XPEBWT-H1-0000-00CZ5</t>
+  </si>
+  <si>
+    <t>LED Lighting XLamp® XP-E2 White, Neutral 4000K 2.9V 350mA 110° 1414 (3535 Metric)</t>
+  </si>
+  <si>
+    <t>IMU</t>
+  </si>
+  <si>
+    <t>6-axis, accelerometer &amp; gyroscope</t>
+  </si>
+  <si>
+    <t>ISM330DLCTR</t>
+  </si>
+  <si>
+    <t>Accelerometer, Gyroscope, Temperature, 6 Axis Sensor I2C, SPI Output</t>
+  </si>
+  <si>
+    <t>PH2RA-04-UA</t>
+  </si>
+  <si>
+    <t>Connector Header Through Hole, Right Angle 4 position 0.100" (2.54mm)</t>
+  </si>
+  <si>
+    <t>IMU  / Accelerometer</t>
+  </si>
+  <si>
+    <t>3-axis Piezoelectric Accelerometer</t>
+  </si>
+  <si>
+    <t>830M1-0025</t>
+  </si>
+  <si>
+    <t>Accelerometer X, Y, Z Axis ±25g 2Hz ~ 15kHz 12-LCC</t>
   </si>
 </sst>
 </file>
@@ -2389,6 +2431,57 @@
           <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2617,6 +2710,22 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
@@ -2638,73 +2747,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2750,13 +2792,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="68"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="66"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="67"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="65"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="65"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -2768,11 +2810,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H20" totalsRowShown="0">
   <autoFilter ref="A1:H20" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="42"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="41"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="40"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -2782,10 +2824,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="39">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="38"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -2804,7 +2846,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="37"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -2814,54 +2856,54 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="36">
   <autoFilter ref="A1:H11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="8">
-    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="24"/>
-    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="15"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="19"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H50" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:H50" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="C1:C50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="75"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="74"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="73">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="11">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -2869,11 +2911,11 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="72"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="71"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="70"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="69"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2949,20 +2991,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="77">
   <autoFilter ref="A1:H100" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H100">
     <sortCondition ref="B1:B100"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="62"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="57"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="56"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="55"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="76"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="73"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="72"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="71"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="70"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="69"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2985,13 +3027,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="64">
   <autoFilter ref="A1:H20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H20">
     <sortCondition ref="B1:B20"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="53"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="63"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -3011,8 +3053,8 @@
     <sortCondition ref="B1:B30"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="52"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="62"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="61"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -3022,11 +3064,11 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="60">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="49"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="48"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="59"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="58"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -3037,25 +3079,25 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="57">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="46"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="56"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="54"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="51">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="40"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="49"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -3069,14 +3111,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="48">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="37"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3918,7 +3960,28 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B12" t="s">
+        <v>716</v>
+      </c>
+      <c r="C12" t="s">
+        <v>416</v>
+      </c>
+      <c r="D12" t="s">
+        <v>104</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>717</v>
+      </c>
+      <c r="F12" t="s">
+        <v>361</v>
+      </c>
+      <c r="G12" t="s">
+        <v>718</v>
+      </c>
+      <c r="H12" t="s">
+        <v>719</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -8610,9 +8673,26 @@
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C53" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="C53" s="12">
+        <v>4</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>724</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>725</v>
+      </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" s="10" t="b">
@@ -9841,12 +9921,36 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B26" t="s">
+        <v>720</v>
+      </c>
+      <c r="C26" t="s">
+        <v>721</v>
+      </c>
+      <c r="D26" t="s">
+        <v>722</v>
+      </c>
+      <c r="E26" t="s">
+        <v>723</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B27" t="s">
+        <v>726</v>
+      </c>
+      <c r="C27" t="s">
+        <v>727</v>
+      </c>
+      <c r="D27" t="s">
+        <v>728</v>
+      </c>
+      <c r="E27" t="s">
+        <v>729</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
@@ -9866,8 +9970,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
started adding some parts for air quality sensor board
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAEC1D9A-2DF8-4AA0-BC2E-39F976399A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00828F05-2324-40CC-B2C6-BBA72079403B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" firstSheet="3" activeTab="5" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="5" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1274" uniqueCount="749">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1285" uniqueCount="759">
   <si>
     <t>Capacitance</t>
   </si>
@@ -2306,6 +2306,36 @@
   </si>
   <si>
     <t>Bus Switch 8 x 1:1 20-TSSOP</t>
+  </si>
+  <si>
+    <t>SCD41-D-R2</t>
+  </si>
+  <si>
+    <t>CO2 Sensor</t>
+  </si>
+  <si>
+    <t>Carbon Dioxide (CO2), Humidity, Temperature Sensor I2C</t>
+  </si>
+  <si>
+    <t>BME688</t>
+  </si>
+  <si>
+    <t>Gas, Humidity, Pressure, Temp Sensor</t>
+  </si>
+  <si>
+    <t>I2C or SPI</t>
+  </si>
+  <si>
+    <t>ENS160-BGLM</t>
+  </si>
+  <si>
+    <t>VoC, AQI Sensor</t>
+  </si>
+  <si>
+    <t>Air Quality Sensor I2C, SPI</t>
+  </si>
+  <si>
+    <t>Gas, Humidity, Pressure, Temperature Sensor I2C, SPI Output</t>
   </si>
 </sst>
 </file>
@@ -3104,10 +3134,10 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}" name="ICs" displayName="ICs" ref="A1:E30" totalsRowShown="0">
-  <autoFilter ref="A1:E30" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E30">
-    <sortCondition ref="B1:B30"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}" name="ICs" displayName="ICs" ref="A1:E50" totalsRowShown="0">
+  <autoFilter ref="A1:E50" xr:uid="{CF6FA6FB-E17E-44DE-A790-4DB35B6C38E6}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E50">
+    <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="5">
     <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="77"/>
@@ -9621,7 +9651,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{713F692B-7F28-45B7-9D1E-A5B0F0D04085}">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -9767,16 +9797,16 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>541</v>
+        <v>708</v>
       </c>
       <c r="C9" t="s">
-        <v>542</v>
+        <v>709</v>
       </c>
       <c r="D9" t="s">
-        <v>543</v>
+        <v>710</v>
       </c>
       <c r="E9" t="s">
-        <v>544</v>
+        <v>711</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -9784,13 +9814,16 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>308</v>
+        <v>541</v>
+      </c>
+      <c r="C10" t="s">
+        <v>542</v>
       </c>
       <c r="D10" t="s">
-        <v>307</v>
+        <v>543</v>
       </c>
       <c r="E10" t="s">
-        <v>309</v>
+        <v>544</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -9798,16 +9831,13 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>563</v>
-      </c>
-      <c r="C11" t="s">
-        <v>564</v>
+        <v>308</v>
       </c>
       <c r="D11" t="s">
-        <v>565</v>
+        <v>307</v>
       </c>
       <c r="E11" t="s">
-        <v>566</v>
+        <v>309</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -9815,16 +9845,16 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>680</v>
+        <v>563</v>
       </c>
       <c r="C12" t="s">
-        <v>681</v>
+        <v>564</v>
       </c>
       <c r="D12" t="s">
-        <v>682</v>
+        <v>565</v>
       </c>
       <c r="E12" t="s">
-        <v>683</v>
+        <v>566</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -9835,13 +9865,13 @@
         <v>680</v>
       </c>
       <c r="C13" t="s">
-        <v>690</v>
+        <v>681</v>
       </c>
       <c r="D13" t="s">
-        <v>691</v>
+        <v>682</v>
       </c>
       <c r="E13" t="s">
-        <v>692</v>
+        <v>683</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -9849,13 +9879,16 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>560</v>
+        <v>680</v>
+      </c>
+      <c r="C14" t="s">
+        <v>690</v>
       </c>
       <c r="D14" t="s">
-        <v>561</v>
+        <v>691</v>
       </c>
       <c r="E14" t="s">
-        <v>562</v>
+        <v>692</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -9863,16 +9896,16 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>80</v>
+        <v>720</v>
       </c>
       <c r="C15" t="s">
-        <v>210</v>
+        <v>721</v>
       </c>
       <c r="D15" t="s">
-        <v>77</v>
+        <v>722</v>
       </c>
       <c r="E15" t="s">
-        <v>78</v>
+        <v>723</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -9880,16 +9913,16 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>80</v>
+        <v>726</v>
       </c>
       <c r="C16" t="s">
-        <v>380</v>
+        <v>727</v>
       </c>
       <c r="D16" t="s">
-        <v>381</v>
+        <v>728</v>
       </c>
       <c r="E16" t="s">
-        <v>382</v>
+        <v>729</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -9897,30 +9930,30 @@
         <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>473</v>
+        <v>560</v>
       </c>
       <c r="D17" t="s">
-        <v>474</v>
+        <v>561</v>
       </c>
       <c r="E17" t="s">
-        <v>475</v>
+        <v>562</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>521</v>
+      <c r="B18" t="s">
+        <v>745</v>
+      </c>
+      <c r="C18" t="s">
+        <v>747</v>
       </c>
       <c r="D18" t="s">
-        <v>91</v>
+        <v>746</v>
       </c>
       <c r="E18" t="s">
-        <v>92</v>
+        <v>748</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -9928,16 +9961,16 @@
         <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>337</v>
+        <v>80</v>
       </c>
       <c r="C19" t="s">
-        <v>520</v>
+        <v>210</v>
       </c>
       <c r="D19" t="s">
-        <v>338</v>
+        <v>77</v>
       </c>
       <c r="E19" t="s">
-        <v>339</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -9945,16 +9978,16 @@
         <v>1</v>
       </c>
       <c r="B20" t="s">
-        <v>337</v>
+        <v>80</v>
       </c>
       <c r="C20" t="s">
-        <v>519</v>
+        <v>380</v>
       </c>
       <c r="D20" t="s">
-        <v>522</v>
+        <v>381</v>
       </c>
       <c r="E20" t="s">
-        <v>523</v>
+        <v>382</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -9962,16 +9995,16 @@
         <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>537</v>
+        <v>704</v>
       </c>
       <c r="C21" t="s">
-        <v>539</v>
+        <v>705</v>
       </c>
       <c r="D21" t="s">
-        <v>538</v>
+        <v>707</v>
       </c>
       <c r="E21" t="s">
-        <v>540</v>
+        <v>706</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
@@ -9979,33 +10012,30 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>315</v>
-      </c>
-      <c r="C22" t="s">
-        <v>316</v>
+        <v>473</v>
       </c>
       <c r="D22" t="s">
-        <v>317</v>
+        <v>474</v>
       </c>
       <c r="E22" t="s">
-        <v>318</v>
+        <v>475</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="B23" t="s">
-        <v>323</v>
-      </c>
-      <c r="C23" t="s">
-        <v>324</v>
+      <c r="B23" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>521</v>
       </c>
       <c r="D23" t="s">
-        <v>325</v>
+        <v>91</v>
       </c>
       <c r="E23" t="s">
-        <v>326</v>
+        <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
@@ -10013,16 +10043,16 @@
         <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>704</v>
+        <v>337</v>
       </c>
       <c r="C24" t="s">
-        <v>705</v>
+        <v>520</v>
       </c>
       <c r="D24" t="s">
-        <v>707</v>
+        <v>338</v>
       </c>
       <c r="E24" t="s">
-        <v>706</v>
+        <v>339</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
@@ -10030,16 +10060,16 @@
         <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>708</v>
+        <v>337</v>
       </c>
       <c r="C25" t="s">
-        <v>709</v>
+        <v>519</v>
       </c>
       <c r="D25" t="s">
-        <v>710</v>
+        <v>522</v>
       </c>
       <c r="E25" t="s">
-        <v>711</v>
+        <v>523</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
@@ -10047,16 +10077,16 @@
         <v>1</v>
       </c>
       <c r="B26" t="s">
-        <v>720</v>
+        <v>537</v>
       </c>
       <c r="C26" t="s">
-        <v>721</v>
+        <v>539</v>
       </c>
       <c r="D26" t="s">
-        <v>722</v>
+        <v>538</v>
       </c>
       <c r="E26" t="s">
-        <v>723</v>
+        <v>540</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
@@ -10064,16 +10094,16 @@
         <v>1</v>
       </c>
       <c r="B27" t="s">
-        <v>726</v>
+        <v>315</v>
       </c>
       <c r="C27" t="s">
-        <v>727</v>
+        <v>316</v>
       </c>
       <c r="D27" t="s">
-        <v>728</v>
+        <v>317</v>
       </c>
       <c r="E27" t="s">
-        <v>729</v>
+        <v>318</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
@@ -10081,25 +10111,158 @@
         <v>1</v>
       </c>
       <c r="B28" t="s">
-        <v>745</v>
+        <v>323</v>
       </c>
       <c r="C28" t="s">
-        <v>747</v>
+        <v>324</v>
       </c>
       <c r="D28" t="s">
-        <v>746</v>
+        <v>325</v>
       </c>
       <c r="E28" t="s">
-        <v>748</v>
+        <v>326</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B29" t="s">
+        <v>750</v>
+      </c>
+      <c r="D29" t="s">
+        <v>749</v>
+      </c>
+      <c r="E29" t="s">
+        <v>751</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B30" t="s">
+        <v>753</v>
+      </c>
+      <c r="C30" t="s">
+        <v>754</v>
+      </c>
+      <c r="D30" t="s">
+        <v>752</v>
+      </c>
+      <c r="E30" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B31" t="s">
+        <v>756</v>
+      </c>
+      <c r="C31" t="s">
+        <v>754</v>
+      </c>
+      <c r="D31" t="s">
+        <v>755</v>
+      </c>
+      <c r="E31" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A35" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A36" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A38" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A39" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A40" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A41" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A42" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A43" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A44" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A45" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A46" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A47" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A48" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A49" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A50" s="9" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added parts for Erik
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B79FC3-1669-456E-A249-6FE403183254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1422983B-714F-4A9C-9DA7-07D49A2893BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="12" activeTab="15" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="10" activeTab="18" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1364" uniqueCount="802">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1418" uniqueCount="824">
   <si>
     <t>Capacitance</t>
   </si>
@@ -2395,9 +2395,6 @@
     <t>3Ohm</t>
   </si>
   <si>
-    <t>TO-236-3, SC-59, SOT-23-3</t>
-  </si>
-  <si>
     <t>BSS138</t>
   </si>
   <si>
@@ -2465,6 +2462,75 @@
   </si>
   <si>
     <t>499 kOhms ±1% 0.125W, 1/8W Chip Resistor 0603 (1608 Metric) Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
+    <t>4.87k</t>
+  </si>
+  <si>
+    <t>CR0603-FX-4871ELF</t>
+  </si>
+  <si>
+    <t>4.87 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Moisture Resistant Thick Film</t>
+  </si>
+  <si>
+    <t>8.25k</t>
+  </si>
+  <si>
+    <t>AF0603FR-078K25L</t>
+  </si>
+  <si>
+    <t>8.25 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Anti-Sulfur, Automotive AEC-Q200 Thick Film</t>
+  </si>
+  <si>
+    <t>RT0603FRE07681KL</t>
+  </si>
+  <si>
+    <t>681k</t>
+  </si>
+  <si>
+    <t>681 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Thin Film</t>
+  </si>
+  <si>
+    <t>MAX20410AFOA/VY+</t>
+  </si>
+  <si>
+    <t>10A</t>
+  </si>
+  <si>
+    <t>3.0-36V</t>
+  </si>
+  <si>
+    <t>0.8-10V</t>
+  </si>
+  <si>
+    <t>Buck Switching Regulator IC Positive Adjustable (Fixed) 0.8V (5V) 1 Output 10A 17-PowerWFQFN</t>
+  </si>
+  <si>
+    <t>TO-220-5</t>
+  </si>
+  <si>
+    <t>17-PowerWFQFN</t>
+  </si>
+  <si>
+    <t>SMCJ33CA</t>
+  </si>
+  <si>
+    <t>53.3V Clamp 28.2A Ipp Tvs Diode Surface Mount DO-214AB (SMCJ)</t>
+  </si>
+  <si>
+    <t>115mA</t>
+  </si>
+  <si>
+    <t>7.5Ohm</t>
+  </si>
+  <si>
+    <t>SOT-23-3</t>
+  </si>
+  <si>
+    <t>2N7002</t>
+  </si>
+  <si>
+    <t>N-Channel 60 V 115mA (Ta) 200mW (Ta) Surface Mount SOT-23-3</t>
   </si>
 </sst>
 </file>
@@ -2647,57 +2713,6 @@
           <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2900,6 +2915,20 @@
       </extLst>
     </dxf>
     <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2951,18 +2980,55 @@
       </extLst>
     </dxf>
     <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3008,13 +3074,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="75"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="67"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="74"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="66"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="73"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="72"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="64"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -3026,11 +3092,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H20" totalsRowShown="0">
   <autoFilter ref="A1:H20" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="42"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="31"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="30"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -3040,10 +3106,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="29">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="28"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -3062,7 +3128,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="27"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -3072,54 +3138,54 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="26">
   <autoFilter ref="A1:H11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="8">
-    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="34"/>
-    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="31"/>
-    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="25"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="20"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="19"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="10"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
   <autoFilter ref="A1:H100" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="C1:C50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="13"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="11">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="75"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="74"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="73">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -3127,11 +3193,11 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="72"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="71"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="70"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="69"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3187,18 +3253,20 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{82CFED5E-627B-4A23-9BFA-C489CEA32F25}" name="Voltage_Regulators" displayName="Voltage_Regulators" ref="A1:H12" totalsRowShown="0">
-  <autoFilter ref="A1:H12" xr:uid="{82CFED5E-627B-4A23-9BFA-C489CEA32F25}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{82CFED5E-627B-4A23-9BFA-C489CEA32F25}" name="Voltage_Regulators" displayName="Voltage_Regulators" ref="A1:J30" totalsRowShown="0">
+  <autoFilter ref="A1:J30" xr:uid="{82CFED5E-627B-4A23-9BFA-C489CEA32F25}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J12">
     <sortCondition ref="B1:B12"/>
   </sortState>
-  <tableColumns count="8">
+  <tableColumns count="10">
     <tableColumn id="3" xr3:uid="{DD7A1A9A-DE5A-4766-9947-A308E87BA7FD}" name="Added to Altium?" dataDxfId="0"/>
     <tableColumn id="1" xr3:uid="{7B7659A2-8D22-4954-B10E-C811D8D29B99}" name="Type"/>
     <tableColumn id="7" xr3:uid="{24DD5DAD-1853-4138-AB66-BA5667E60D26}" name="Operation"/>
     <tableColumn id="8" xr3:uid="{C0E1C407-BC33-4018-B09E-15A16329D7C6}" name="Input Voltage"/>
     <tableColumn id="2" xr3:uid="{1B401263-31AB-4380-A4FD-B256C750FA0B}" name="Output Voltage"/>
     <tableColumn id="4" xr3:uid="{5B3C6EDD-81A6-41AD-B149-C2BF3585E802}" name="Max output current"/>
+    <tableColumn id="10" xr3:uid="{6CD35AD7-D590-49B2-B0F8-29D64F621F32}" name="Mount Type"/>
+    <tableColumn id="9" xr3:uid="{3BAFA6E9-3767-49E8-A1C5-9C1E8B6EE0D4}" name="Package"/>
     <tableColumn id="6" xr3:uid="{B16EED48-4D3D-4D5C-88EC-B23C579A8E2D}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{58F36E9E-E2F2-4DE5-B2DC-96C9F966EEF9}" name="Description"/>
   </tableColumns>
@@ -3207,20 +3275,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="63">
   <autoFilter ref="A1:H100" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H100">
     <sortCondition ref="B1:B100"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="70"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="69"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="68"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="67"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="66"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="65"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="62"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="61"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="60"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="59"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="57"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3243,13 +3311,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="54">
   <autoFilter ref="A1:H20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H20">
     <sortCondition ref="B1:B20"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="61"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="53"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -3269,8 +3337,8 @@
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="77"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="76"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="52"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="51"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -3280,11 +3348,11 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="60">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="50">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="59"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="58"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="49"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="48"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -3295,25 +3363,25 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="57">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="47">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="56"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="54"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="53"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="52"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="51">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="41">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="50"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="39"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -3327,14 +3395,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="38">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="47"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5833,7 +5901,7 @@
         <v>1</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="C37" s="17">
         <f t="shared" si="1"/>
@@ -5849,10 +5917,10 @@
         <v>194</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="H37" s="16" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.35">
@@ -5860,7 +5928,7 @@
         <v>1</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C38" s="17">
         <f t="shared" si="1"/>
@@ -5876,10 +5944,10 @@
         <v>194</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="H38" s="16" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
@@ -5887,7 +5955,7 @@
         <v>1</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C39" s="17">
         <f t="shared" si="1"/>
@@ -5903,10 +5971,10 @@
         <v>194</v>
       </c>
       <c r="G39" s="16" t="s">
+        <v>787</v>
+      </c>
+      <c r="H39" s="16" t="s">
         <v>788</v>
-      </c>
-      <c r="H39" s="16" t="s">
-        <v>789</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.35">
@@ -5914,7 +5982,7 @@
         <v>1</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="C40" s="17">
         <f t="shared" si="1"/>
@@ -5930,10 +5998,10 @@
         <v>194</v>
       </c>
       <c r="G40" s="16" t="s">
+        <v>790</v>
+      </c>
+      <c r="H40" s="16" t="s">
         <v>791</v>
-      </c>
-      <c r="H40" s="16" t="s">
-        <v>792</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
@@ -5941,7 +6009,7 @@
         <v>1</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="C41" s="17">
         <f t="shared" si="1"/>
@@ -5957,10 +6025,10 @@
         <v>194</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="H41" s="16" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.35">
@@ -5968,7 +6036,7 @@
         <v>1</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="C42" s="17">
         <f t="shared" si="1"/>
@@ -5984,10 +6052,10 @@
         <v>194</v>
       </c>
       <c r="G42" s="16" t="s">
+        <v>796</v>
+      </c>
+      <c r="H42" s="16" t="s">
         <v>797</v>
-      </c>
-      <c r="H42" s="16" t="s">
-        <v>798</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
@@ -5995,7 +6063,7 @@
         <v>1</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="C43" s="17">
         <f t="shared" si="1"/>
@@ -6011,62 +6079,92 @@
         <v>138</v>
       </c>
       <c r="G43" s="16" t="s">
+        <v>799</v>
+      </c>
+      <c r="H43" s="16" t="s">
         <v>800</v>
-      </c>
-      <c r="H43" s="16" t="s">
-        <v>801</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="B44" s="15">
-        <v>0</v>
-      </c>
-      <c r="C44" s="17" t="str">
+        <v>1</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>801</v>
+      </c>
+      <c r="C44" s="17">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="D44" s="16"/>
-      <c r="E44" s="16"/>
-      <c r="F44" s="16"/>
-      <c r="G44" s="16"/>
-      <c r="H44" s="16"/>
+        <v>4870</v>
+      </c>
+      <c r="D44" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="E44" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F44" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="G44" s="16" t="s">
+        <v>802</v>
+      </c>
+      <c r="H44" s="16" t="s">
+        <v>803</v>
+      </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="B45" s="15">
-        <v>0</v>
-      </c>
-      <c r="C45" s="17" t="str">
+        <v>1</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>804</v>
+      </c>
+      <c r="C45" s="17">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16"/>
-      <c r="F45" s="16"/>
-      <c r="G45" s="16"/>
-      <c r="H45" s="16"/>
+        <v>8250</v>
+      </c>
+      <c r="D45" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="E45" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F45" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="G45" s="16" t="s">
+        <v>805</v>
+      </c>
+      <c r="H45" s="16" t="s">
+        <v>806</v>
+      </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="B46" s="15">
-        <v>0</v>
-      </c>
-      <c r="C46" s="17" t="str">
+        <v>1</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>808</v>
+      </c>
+      <c r="C46" s="17">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="D46" s="16"/>
-      <c r="E46" s="16"/>
-      <c r="F46" s="16"/>
-      <c r="G46" s="16"/>
-      <c r="H46" s="16"/>
+        <v>681000</v>
+      </c>
+      <c r="D46" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="E46" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F46" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="G46" s="16" t="s">
+        <v>807</v>
+      </c>
+      <c r="H46" s="16" t="s">
+        <v>809</v>
+      </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="18" t="b">
@@ -7536,18 +7634,42 @@
         <v>777</v>
       </c>
       <c r="G8" t="s">
+        <v>821</v>
+      </c>
+      <c r="H8" t="s">
         <v>778</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>779</v>
-      </c>
-      <c r="I8" t="s">
-        <v>780</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>297</v>
+      </c>
+      <c r="C9" t="s">
+        <v>299</v>
+      </c>
+      <c r="D9" t="s">
+        <v>667</v>
+      </c>
+      <c r="E9" t="s">
+        <v>819</v>
+      </c>
+      <c r="F9" t="s">
+        <v>820</v>
+      </c>
+      <c r="G9" t="s">
+        <v>821</v>
+      </c>
+      <c r="H9" t="s">
+        <v>822</v>
+      </c>
+      <c r="I9" t="s">
+        <v>823</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -8710,20 +8832,16 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E9ACF1C-C12B-4B5A-BD57-0454748C5027}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.1796875" customWidth="1"/>
-    <col min="2" max="2" width="16.26953125" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" customWidth="1"/>
-    <col min="4" max="4" width="16.26953125" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" customWidth="1"/>
-    <col min="6" max="7" width="18.54296875" customWidth="1"/>
-    <col min="8" max="8" width="54.90625" customWidth="1"/>
-    <col min="9" max="16384" width="8.7265625" hidden="1"/>
+    <col min="1" max="8" width="15.6328125" customWidth="1"/>
+    <col min="9" max="9" width="18.54296875" customWidth="1"/>
+    <col min="10" max="10" width="54.90625" customWidth="1"/>
+    <col min="11" max="16384" width="15.6328125" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>198</v>
       </c>
@@ -8743,13 +8861,19 @@
         <v>89</v>
       </c>
       <c r="G1" t="s">
+        <v>193</v>
+      </c>
+      <c r="H1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" t="s">
         <v>2</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="b">
         <v>1</v>
       </c>
@@ -8769,13 +8893,16 @@
         <v>90</v>
       </c>
       <c r="G2" t="s">
+        <v>104</v>
+      </c>
+      <c r="I2" t="s">
         <v>88</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="b">
         <v>1</v>
       </c>
@@ -8795,13 +8922,19 @@
         <v>120</v>
       </c>
       <c r="G3" t="s">
+        <v>126</v>
+      </c>
+      <c r="H3" t="s">
+        <v>815</v>
+      </c>
+      <c r="I3" t="s">
         <v>367</v>
       </c>
-      <c r="H3" t="s">
+      <c r="J3" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="b">
         <v>1</v>
       </c>
@@ -8821,65 +8954,74 @@
         <v>172</v>
       </c>
       <c r="G4" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" t="s">
         <v>374</v>
       </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>144</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>225</v>
+        <v>364</v>
       </c>
       <c r="D5" t="s">
-        <v>229</v>
+        <v>624</v>
       </c>
       <c r="E5" t="s">
-        <v>147</v>
+        <v>605</v>
       </c>
       <c r="F5" t="s">
-        <v>145</v>
+        <v>625</v>
       </c>
       <c r="G5" t="s">
-        <v>146</v>
-      </c>
-      <c r="H5" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+        <v>104</v>
+      </c>
+      <c r="I5" t="s">
+        <v>626</v>
+      </c>
+      <c r="J5" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="b">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>144</v>
+        <v>85</v>
       </c>
       <c r="C6" t="s">
-        <v>225</v>
+        <v>364</v>
       </c>
       <c r="D6" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="E6" t="s">
-        <v>553</v>
+        <v>87</v>
       </c>
       <c r="F6" t="s">
-        <v>393</v>
+        <v>730</v>
       </c>
       <c r="G6" t="s">
-        <v>554</v>
-      </c>
-      <c r="H6" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+        <v>104</v>
+      </c>
+      <c r="I6" t="s">
+        <v>731</v>
+      </c>
+      <c r="J6" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="b">
         <v>1</v>
       </c>
@@ -8890,22 +9032,25 @@
         <v>364</v>
       </c>
       <c r="D7" t="s">
-        <v>624</v>
+        <v>553</v>
       </c>
       <c r="E7" t="s">
-        <v>605</v>
+        <v>87</v>
       </c>
       <c r="F7" t="s">
-        <v>625</v>
+        <v>313</v>
       </c>
       <c r="G7" t="s">
-        <v>626</v>
-      </c>
-      <c r="H7" t="s">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+        <v>104</v>
+      </c>
+      <c r="I7" t="s">
+        <v>733</v>
+      </c>
+      <c r="J7" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="b">
         <v>1</v>
       </c>
@@ -8916,80 +9061,209 @@
         <v>225</v>
       </c>
       <c r="D8" t="s">
+        <v>229</v>
+      </c>
+      <c r="E8" t="s">
+        <v>147</v>
+      </c>
+      <c r="F8" t="s">
+        <v>145</v>
+      </c>
+      <c r="G8" t="s">
+        <v>104</v>
+      </c>
+      <c r="H8" t="s">
+        <v>816</v>
+      </c>
+      <c r="I8" t="s">
+        <v>146</v>
+      </c>
+      <c r="J8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C9" t="s">
+        <v>225</v>
+      </c>
+      <c r="D9" t="s">
+        <v>556</v>
+      </c>
+      <c r="E9" t="s">
+        <v>553</v>
+      </c>
+      <c r="F9" t="s">
+        <v>393</v>
+      </c>
+      <c r="G9" t="s">
+        <v>104</v>
+      </c>
+      <c r="I9" t="s">
+        <v>554</v>
+      </c>
+      <c r="J9" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>144</v>
+      </c>
+      <c r="C10" t="s">
+        <v>225</v>
+      </c>
+      <c r="D10" t="s">
         <v>658</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E10" t="s">
         <v>605</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F10" t="s">
         <v>120</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G10" t="s">
+        <v>104</v>
+      </c>
+      <c r="I10" t="s">
         <v>659</v>
       </c>
-      <c r="H8" t="s">
+      <c r="J10" t="s">
         <v>660</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B9" t="s">
-        <v>85</v>
-      </c>
-      <c r="C9" t="s">
-        <v>364</v>
-      </c>
-      <c r="D9" t="s">
-        <v>553</v>
-      </c>
-      <c r="E9" t="s">
-        <v>87</v>
-      </c>
-      <c r="F9" t="s">
-        <v>730</v>
-      </c>
-      <c r="G9" t="s">
-        <v>731</v>
-      </c>
-      <c r="H9" t="s">
-        <v>732</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" t="s">
-        <v>85</v>
-      </c>
-      <c r="C10" t="s">
-        <v>364</v>
-      </c>
-      <c r="D10" t="s">
-        <v>553</v>
-      </c>
-      <c r="E10" t="s">
-        <v>87</v>
-      </c>
-      <c r="F10" t="s">
-        <v>313</v>
-      </c>
-      <c r="G10" t="s">
-        <v>733</v>
-      </c>
-      <c r="H10" t="s">
-        <v>734</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" t="s">
+        <v>225</v>
+      </c>
+      <c r="D11" t="s">
+        <v>812</v>
+      </c>
+      <c r="E11" t="s">
+        <v>813</v>
+      </c>
+      <c r="F11" t="s">
+        <v>811</v>
+      </c>
+      <c r="G11" t="s">
+        <v>104</v>
+      </c>
+      <c r="H11" t="s">
+        <v>816</v>
+      </c>
+      <c r="I11" t="s">
+        <v>810</v>
+      </c>
+      <c r="J11" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30" s="9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10892,7 +11166,25 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
+        <v>524</v>
+      </c>
+      <c r="C13" t="s">
+        <v>525</v>
+      </c>
+      <c r="E13" t="s">
+        <v>766</v>
+      </c>
+      <c r="F13" t="s">
+        <v>767</v>
+      </c>
+      <c r="G13" t="s">
+        <v>817</v>
+      </c>
+      <c r="H13" t="s">
+        <v>818</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
added lora sx1276 rfm95 module
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1422983B-714F-4A9C-9DA7-07D49A2893BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F93B3C-326B-40A2-8B45-DFF4E426773E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="10" activeTab="18" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="6" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1418" uniqueCount="824">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1427" uniqueCount="831">
   <si>
     <t>Capacitance</t>
   </si>
@@ -2531,6 +2531,27 @@
   </si>
   <si>
     <t>N-Channel 60 V 115mA (Ta) 200mW (Ta) Surface Mount SOT-23-3</t>
+  </si>
+  <si>
+    <t>SX1276 LoRa Module 915MHz RFM95</t>
+  </si>
+  <si>
+    <t>LoRa Transceiver</t>
+  </si>
+  <si>
+    <t>SX1276 RFM95</t>
+  </si>
+  <si>
+    <t>Transceiver</t>
+  </si>
+  <si>
+    <t>NRPN081PAEN-RC</t>
+  </si>
+  <si>
+    <t>2.00mm pitch</t>
+  </si>
+  <si>
+    <t>Connector Header Through Hole 8 position 0.079" (2.00mm)</t>
   </si>
 </sst>
 </file>
@@ -2688,7 +2709,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FF7030A0"/>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2700,19 +2721,55 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FF92D050"/>
+          <bgColor rgb="FFC00000"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2980,53 +3037,17 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FFC00000"/>
+          <bgColor rgb="FF7030A0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3074,13 +3095,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="75"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="66"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="74"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="65"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="73"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="72"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -3092,11 +3113,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H20" totalsRowShown="0">
   <autoFilter ref="A1:H20" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="39"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="38"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -3106,10 +3127,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="37">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="36"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -3128,7 +3149,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="35"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -3138,54 +3159,54 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="34">
   <autoFilter ref="A1:H11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="8">
-    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="24"/>
-    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="32"/>
+    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="29"/>
+    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="15"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="18"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="17"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:H100" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="C1:C50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="75"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="74"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="73">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="9">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -3193,11 +3214,11 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="72"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="71"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="70"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="69"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3207,7 +3228,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}" name="Switches" displayName="Switches" ref="A1:G11" totalsRowShown="0">
   <autoFilter ref="A1:G11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="3"/>
     <tableColumn id="1" xr3:uid="{C868B851-3D2D-4863-96B3-5412E9A862E1}" name="Function"/>
     <tableColumn id="6" xr3:uid="{D6EA3AC7-CEF9-4E2A-800B-297C8C002273}" name="Circuit"/>
     <tableColumn id="2" xr3:uid="{5048C5E7-258E-4EC2-B0BD-C338C4D84C91}" name="Part Number"/>
@@ -3220,10 +3241,10 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{C800FF98-41EA-493F-A089-14FECFF39D7A}" name="Test_Points" displayName="Test_Points" ref="A1:F11" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{C800FF98-41EA-493F-A089-14FECFF39D7A}" name="Test_Points" displayName="Test_Points" ref="A1:F11" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:F11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{5FA1F5D0-B5EA-4DAB-B07A-643BF29E8565}" name="Added to Altium?" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{5FA1F5D0-B5EA-4DAB-B07A-643BF29E8565}" name="Added to Altium?" dataDxfId="1"/>
     <tableColumn id="1" xr3:uid="{CC1FCF46-8E52-4166-BC69-286FE8778BAA}" name="Mounting Type"/>
     <tableColumn id="3" xr3:uid="{25F97020-E67A-4F9F-99D3-71374E9FAEC5}" name="# of pads/points"/>
     <tableColumn id="6" xr3:uid="{6395E911-E7EB-4DC7-B232-C23AAD6F19AF}" name="Series"/>
@@ -3235,10 +3256,10 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{261C41B4-4EE2-4BF0-B2F3-2F2A51D3792A}" name="Transistors" displayName="Transistors" ref="A1:I40" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{261C41B4-4EE2-4BF0-B2F3-2F2A51D3792A}" name="Transistors" displayName="Transistors" ref="A1:I40" totalsRowShown="0" headerRowDxfId="77">
   <autoFilter ref="A1:I40" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{3A0D6614-B80A-4184-9ADE-5206B38A06E5}" name="Added to Altium?" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{3A0D6614-B80A-4184-9ADE-5206B38A06E5}" name="Added to Altium?" dataDxfId="76"/>
     <tableColumn id="1" xr3:uid="{05D09AC3-5445-495F-8B8E-1C98473F2758}" name="Technology"/>
     <tableColumn id="6" xr3:uid="{F919A207-76D0-435F-BB24-020D391F6DB9}" name="Configuration"/>
     <tableColumn id="8" xr3:uid="{4CC17C6A-1F84-408C-8AAD-69C3E5F234CA}" name="V_DS MAX"/>
@@ -3275,20 +3296,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="71">
   <autoFilter ref="A1:H100" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H100">
     <sortCondition ref="B1:B100"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="62"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="57"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="56"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="55"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="70"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="68"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3311,13 +3332,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="62">
   <autoFilter ref="A1:H20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H20">
     <sortCondition ref="B1:B20"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="53"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="61"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -3337,8 +3358,8 @@
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="52"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="60"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="59"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -3348,11 +3369,11 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="58">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="49"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="48"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="57"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="56"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -3363,25 +3384,25 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="55">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="46"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="49">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="40"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="47"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -3395,14 +3416,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="46">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="37"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="45"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -10394,9 +10415,26 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C54" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="C54" s="12">
+        <v>8</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>828</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>829</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>830</v>
+      </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" s="10" t="b">
@@ -12021,7 +12059,19 @@
     </row>
     <row r="8" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>825</v>
+      </c>
+      <c r="C8" t="s">
+        <v>826</v>
+      </c>
+      <c r="D8" t="s">
+        <v>827</v>
+      </c>
+      <c r="F8" t="s">
+        <v>824</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
minor update to spreadsheet
</commit_message>
<xml_diff>
--- a/Altium Parts.xlsx
+++ b/Altium Parts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIL-Altium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F93B3C-326B-40A2-8B45-DFF4E426773E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EEF742C-B39B-4C48-B9F3-9B8E3BE79CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="6" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="2" activeTab="6" xr2:uid="{78817FF2-1CC3-4A74-8C91-2AFFF0842C3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome!" sheetId="15" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1427" uniqueCount="831">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1430" uniqueCount="834">
   <si>
     <t>Capacitance</t>
   </si>
@@ -2552,6 +2552,15 @@
   </si>
   <si>
     <t>Connector Header Through Hole 8 position 0.079" (2.00mm)</t>
+  </si>
+  <si>
+    <t>Alcohol Gas Sensor</t>
+  </si>
+  <si>
+    <t>MQ-3B</t>
+  </si>
+  <si>
+    <t>Air Quality Sensor</t>
   </si>
 </sst>
 </file>
@@ -2709,6 +2718,21 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
           <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
@@ -2811,39 +2835,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <extLst>
@@ -3037,19 +3028,37 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
+          <xfpb:DXFComplement i="1"/>
         </ext>
       </extLst>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3095,13 +3104,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}" name="Capacitors" displayName="Capacitors" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{66640DDE-A600-4D40-886A-D93F6DB5FAB3}"/>
   <tableColumns count="9">
-    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="75"/>
+    <tableColumn id="8" xr3:uid="{B97E7FE0-D68A-4659-9DE5-965B7C74FB58}" name="Added to Altium?" dataDxfId="68"/>
     <tableColumn id="1" xr3:uid="{BDC3005D-8889-49B9-B05B-9B4FB822D92C}" name="Capacitance"/>
-    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="74"/>
+    <tableColumn id="2" xr3:uid="{204119AE-0485-4922-A3C8-7CDD048C63F5}" name="Package" dataDxfId="67"/>
     <tableColumn id="3" xr3:uid="{13A5BE24-7E3B-42A7-BB30-CF0EA6F4873D}" name="Max Voltage"/>
     <tableColumn id="4" xr3:uid="{D4BF488D-A80E-4525-A0D1-501D554CEDF7}" name="Tolerance"/>
-    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="73"/>
-    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="72"/>
+    <tableColumn id="5" xr3:uid="{08BCE889-36CA-4A02-9976-7D80BAE9681D}" name="Mounting Type" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{B82114B5-A4D9-4327-9F80-0D9587A64062}" name="Polarity" dataDxfId="65"/>
     <tableColumn id="6" xr3:uid="{31CBAF16-36EA-4251-9AC8-58F6F46900E9}" name="Material"/>
     <tableColumn id="7" xr3:uid="{571D64FC-0F67-4FD0-B071-89D71A56F7C6}" name="Manufacturer Part Number"/>
   </tableColumns>
@@ -3113,11 +3122,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}" name="LEDs" displayName="LEDs" ref="A1:H20" totalsRowShown="0">
   <autoFilter ref="A1:H20" xr:uid="{C732A860-4A42-46A7-A5FA-C00091FE4BA3}"/>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="40"/>
-    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{B2E48D06-BAB0-4133-877E-867AB2EC32E9}" name="Added to Altium?" dataDxfId="33"/>
+    <tableColumn id="8" xr3:uid="{22D7B7BF-E3CF-4637-92B5-B74434B0A877}" name="Type" dataDxfId="32"/>
     <tableColumn id="1" xr3:uid="{727DF6C0-6BC9-4CBC-ACBD-F7D7801F3DED}" name="Color"/>
     <tableColumn id="6" xr3:uid="{2F89F121-2031-4E76-8B64-C6BE1AC4E5A7}" name="Mount Type"/>
-    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{59EEDA5E-A95B-4620-BC5E-79C5C5FB8AFC}" name="Package" dataDxfId="31"/>
     <tableColumn id="3" xr3:uid="{95A3DF17-FA71-419C-9869-87ACAC774187}" name="Dome"/>
     <tableColumn id="4" xr3:uid="{30ACC022-FAF3-44FA-97E2-DA5C989B54D7}" name="Part Number"/>
     <tableColumn id="5" xr3:uid="{BDED051F-FA40-461B-85BB-40EDC316E70C}" name="Description"/>
@@ -3127,10 +3136,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}" name="ICs_10" displayName="ICs_10" ref="A1:G10" totalsRowShown="0" headerRowDxfId="30">
   <autoFilter ref="A1:G10" xr:uid="{EF03BBEA-AE4C-45BB-9CD5-736F7FCCE237}"/>
   <tableColumns count="7">
-    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{2AE73037-16FE-4A0E-B4B4-CF3863388825}" name="Added to Altium?" dataDxfId="29"/>
     <tableColumn id="2" xr3:uid="{D4673AC2-9436-437D-9DE0-521034F11263}" name="Memory Organization"/>
     <tableColumn id="6" xr3:uid="{088605FE-5C4A-4A9F-9607-7699E9A0ED47}" name="Total Capacity"/>
     <tableColumn id="7" xr3:uid="{E9CAAB16-100E-4178-A533-7FCE76F08C9F}" name="Interface"/>
@@ -3149,7 +3158,7 @@
     <sortCondition ref="B1:B13"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{6C04560D-813B-4E79-B81B-87E653E3F958}" name="Added to Altium?" dataDxfId="28"/>
     <tableColumn id="1" xr3:uid="{07652CF2-D7CA-452D-A87D-CEBA35FEC12A}" name="Function"/>
     <tableColumn id="2" xr3:uid="{A9FCB299-A552-4123-B45A-F31F0DC5BB9B}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{2F50D30B-F60A-4BAF-AE6D-0A3909047904}" name="Description"/>
@@ -3159,54 +3168,54 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{A40CA8A6-1C4E-486A-ACF3-77702798EDC5}" name="Mounts_Pads_Vias" displayName="Mounts_Pads_Vias" ref="A1:H11" totalsRowShown="0" headerRowDxfId="77">
   <autoFilter ref="A1:H11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="8">
-    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="32"/>
-    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="29"/>
-    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="28"/>
-    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{AEAC8F87-1C2D-4AB2-AF57-3B985B9984E8}" name="Added to Altium?" dataDxfId="76"/>
+    <tableColumn id="6" xr3:uid="{013363CF-8CB8-438A-8840-8BE5C88DD21A}" name="Type" dataDxfId="75"/>
+    <tableColumn id="1" xr3:uid="{D05BE736-0061-4B08-B525-77CB6D52275D}" name="Name" dataDxfId="74"/>
+    <tableColumn id="2" xr3:uid="{7A597B79-DB0B-4F42-A26A-5BFC2BE446DB}" name="Shape" dataDxfId="73"/>
+    <tableColumn id="3" xr3:uid="{9BE909D1-CB3E-47D8-89BD-A5A9007FC19A}" name="Hole Size (diameter)" dataDxfId="72"/>
+    <tableColumn id="8" xr3:uid="{9D59173A-B663-440B-ABB2-B4420C0F2F76}" name="Copper X-Size" dataDxfId="71"/>
+    <tableColumn id="7" xr3:uid="{0B466DAF-712F-4EDB-BA0B-281F181D75D1}" name="Copper Y-Size" dataDxfId="70"/>
+    <tableColumn id="4" xr3:uid="{63AE9014-61F7-479D-A241-EAA26D52AAA0}" name="Description" dataDxfId="69"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}" name="MCUs" displayName="MCUs" ref="A1:J11" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:J11" xr:uid="{9DA4F768-7F47-4563-8367-8C9704917FC2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J11">
     <sortCondition ref="B1:B11"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="23"/>
-    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="18"/>
-    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{B7904B75-EB47-4AE0-AC16-835BCD406E73}" name="Added to Altium?" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{0881C807-AE0D-4E97-942D-F1BB4BC72740}" name="Name" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{FF11C1E0-268B-4AB9-A529-8334EF2C69FD}" name="# GPIO" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{55162BE7-C291-4B9F-ABE8-A7DE102A5A2F}" name="UART" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{12871EC5-67F1-442C-B9F6-E715FA2B13DA}" name="SPI" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{0676FDA2-81C4-49A9-A3D1-DEE7F28D8014}" name="I2C" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{4D86DECE-60FC-46A0-B57F-AB144D9C1459}" name="PWM" dataDxfId="19"/>
+    <tableColumn id="12" xr3:uid="{F498CA82-C855-4B59-BFFB-E076763E2C7B}" name="USB" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{1C8B55E3-7B48-484B-9DEC-D60D33855BF8}" name="Part Number" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{EB01044E-239A-43EB-B0C2-1F87DDB54160}" name="Description" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}" name="Resistors" displayName="Resistors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:H100" xr:uid="{FE99B236-7512-4792-AE6E-EED4D7BDA003}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H50">
     <sortCondition ref="C1:C50"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="11"/>
-    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="9">
+    <tableColumn id="8" xr3:uid="{5CCC4BAB-E9A7-42D2-BFCF-40A14E4FCFB3}" name="Added to Altium?" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{E2BB1AD3-36C9-4D80-8A78-E46D0D28B43D}" name="Resistance" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{C2F2285A-BFA3-4714-8945-6FE63C9CDE81}" name="Res (Raw)" dataDxfId="11">
       <calculatedColumnFormula>IF(ISNUMBER(B2),
 IF(B2=0,"",B2),
 VALUE(LEFT(B2,LEN(B2)-1))*
@@ -3214,11 +3223,11 @@
 IF(RIGHT(B2,1)="M",1000000,
 IF(RIGHT(B2,1)="m",0.001,1))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{67EED117-D01D-4FE8-BB40-D7D8F55BAB48}" name="Tolerance" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{F1269AFE-5CA5-4F00-93B8-6023E945504D}" name="Package" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{A4374340-1758-433F-80B6-83ABF6D97E11}" name="Wattage" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{7C53E4E9-C23D-4482-9A46-441AB8A4E1B1}" name="Part Number" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{BD8216A4-1B75-4738-A589-0D33231AD075}" name="Description" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium17" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3228,7 +3237,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}" name="Switches" displayName="Switches" ref="A1:G11" totalsRowShown="0">
   <autoFilter ref="A1:G11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="7">
-    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{AC77A4FF-3DCF-4737-ACB4-F75821B19F57}" name="Added to Altium?" dataDxfId="5"/>
     <tableColumn id="1" xr3:uid="{C868B851-3D2D-4863-96B3-5412E9A862E1}" name="Function"/>
     <tableColumn id="6" xr3:uid="{D6EA3AC7-CEF9-4E2A-800B-297C8C002273}" name="Circuit"/>
     <tableColumn id="2" xr3:uid="{5048C5E7-258E-4EC2-B0BD-C338C4D84C91}" name="Part Number"/>
@@ -3241,10 +3250,10 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{C800FF98-41EA-493F-A089-14FECFF39D7A}" name="Test_Points" displayName="Test_Points" ref="A1:F11" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{C800FF98-41EA-493F-A089-14FECFF39D7A}" name="Test_Points" displayName="Test_Points" ref="A1:F11" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="A1:F11" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{5FA1F5D0-B5EA-4DAB-B07A-643BF29E8565}" name="Added to Altium?" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{5FA1F5D0-B5EA-4DAB-B07A-643BF29E8565}" name="Added to Altium?" dataDxfId="3"/>
     <tableColumn id="1" xr3:uid="{CC1FCF46-8E52-4166-BC69-286FE8778BAA}" name="Mounting Type"/>
     <tableColumn id="3" xr3:uid="{25F97020-E67A-4F9F-99D3-71374E9FAEC5}" name="# of pads/points"/>
     <tableColumn id="6" xr3:uid="{6395E911-E7EB-4DC7-B232-C23AAD6F19AF}" name="Series"/>
@@ -3256,10 +3265,10 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{261C41B4-4EE2-4BF0-B2F3-2F2A51D3792A}" name="Transistors" displayName="Transistors" ref="A1:I40" totalsRowShown="0" headerRowDxfId="77">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{261C41B4-4EE2-4BF0-B2F3-2F2A51D3792A}" name="Transistors" displayName="Transistors" ref="A1:I40" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:I40" xr:uid="{EA8CC69A-B6DA-4750-BA77-538662D89C27}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{3A0D6614-B80A-4184-9ADE-5206B38A06E5}" name="Added to Altium?" dataDxfId="76"/>
+    <tableColumn id="7" xr3:uid="{3A0D6614-B80A-4184-9ADE-5206B38A06E5}" name="Added to Altium?" dataDxfId="1"/>
     <tableColumn id="1" xr3:uid="{05D09AC3-5445-495F-8B8E-1C98473F2758}" name="Technology"/>
     <tableColumn id="6" xr3:uid="{F919A207-76D0-435F-BB24-020D391F6DB9}" name="Configuration"/>
     <tableColumn id="8" xr3:uid="{4CC17C6A-1F84-408C-8AAD-69C3E5F234CA}" name="V_DS MAX"/>
@@ -3296,20 +3305,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}" name="Connectors" displayName="Connectors" ref="A1:H100" totalsRowShown="0" headerRowDxfId="64">
   <autoFilter ref="A1:H100" xr:uid="{7090E628-1F8E-4CB3-BC5C-768E76CEFDDC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H100">
     <sortCondition ref="B1:B100"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="70"/>
-    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="69"/>
-    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="68"/>
-    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="67"/>
-    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="66"/>
-    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="65"/>
-    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{CE9E315A-1702-4F78-8ECF-1DA1A2B792AA}" name="Added to Altium?" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{D5AE5A29-FEF0-4556-97F0-002479587894}" name="Series / Family" dataDxfId="62"/>
+    <tableColumn id="2" xr3:uid="{8673F73F-EA18-4F48-837C-C3D933082CD8}" name="# Pins" dataDxfId="61"/>
+    <tableColumn id="3" xr3:uid="{F61E1994-58CD-4ECF-A835-1786BECF70C2}" name="Gender (plug/port)" dataDxfId="60"/>
+    <tableColumn id="4" xr3:uid="{ADD992CB-74CD-4839-9C1F-4CA1C98DDDE6}" name="Part Number" dataDxfId="59"/>
+    <tableColumn id="8" xr3:uid="{0052054B-61D9-4444-933B-4830DE18EF5D}" name="Mating Connector Part Number" dataDxfId="58"/>
+    <tableColumn id="9" xr3:uid="{DF57140F-10E9-43CB-BE16-5AB59D2592F7}" name="Notes" dataDxfId="57"/>
+    <tableColumn id="5" xr3:uid="{E04857DF-CEB1-4D64-87C3-2580C252E44F}" name="Description" dataDxfId="56"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3332,13 +3341,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}" name="Diodes" displayName="Diodes" ref="A1:H20" totalsRowShown="0" headerRowDxfId="55">
   <autoFilter ref="A1:H20" xr:uid="{AC1B69C7-59BA-492E-BEF3-378F8F5A5F42}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H20">
     <sortCondition ref="B1:B20"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="61"/>
+    <tableColumn id="7" xr3:uid="{373BF80E-AE0E-45C8-9A43-A9D96680B6E9}" name="Added to Altium?" dataDxfId="54"/>
     <tableColumn id="1" xr3:uid="{3176E398-8316-4079-97C6-E10CED1CC775}" name="Type"/>
     <tableColumn id="2" xr3:uid="{DFDAC67A-8333-4623-A218-F2BB6C8E25E6}" name="Breakdown voltage"/>
     <tableColumn id="3" xr3:uid="{3A72F6DE-D147-42DD-9C1C-BA3A3545DE11}" name="Max Forward Current"/>
@@ -3358,8 +3367,8 @@
     <sortCondition ref="B1:B50"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="60"/>
-    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="59"/>
+    <tableColumn id="4" xr3:uid="{2DF829CD-290D-41D3-B284-4B22DE33C4AA}" name="Added to Altium?" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{0460994E-DB61-407B-B7D3-3CAA8ED4BC9D}" name="Function" dataDxfId="52"/>
     <tableColumn id="6" xr3:uid="{F86F95F1-F9FE-4146-B379-63E1029BD91F}" name="Notes"/>
     <tableColumn id="1" xr3:uid="{B62DE98C-40C5-4F02-871A-56E6F423B932}" name="Part Number"/>
     <tableColumn id="3" xr3:uid="{613F07FA-6CA3-413B-A8EC-C111F4721AB4}" name="Description"/>
@@ -3369,11 +3378,11 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}" name="Devices" displayName="Devices" ref="A1:F50" totalsRowShown="0" headerRowDxfId="51">
   <autoFilter ref="A1:F50" xr:uid="{C5737D88-F4D8-4117-9BA5-1B2CC31DE11A}"/>
   <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="57"/>
-    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="56"/>
+    <tableColumn id="7" xr3:uid="{6415E46E-CEE3-460F-B779-529E15CD07B6}" name="Added to Altium?" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{A1AE6712-2A25-444F-8418-5CCFC5CDB835}" name="Series" dataDxfId="49"/>
     <tableColumn id="9" xr3:uid="{6F530F3C-B40B-43DA-AB86-21341EB4DAD1}" name="Device"/>
     <tableColumn id="1" xr3:uid="{4AA09E23-76BE-4EAC-BAB7-D19DB7FEF15D}" name="Type"/>
     <tableColumn id="5" xr3:uid="{79DDF2A7-4DA6-48DB-8655-801CD7025B51}" name="Part Number"/>
@@ -3384,25 +3393,25 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}" name="Table6" displayName="Table6" ref="A1:E11" totalsRowShown="0" headerRowDxfId="48">
   <autoFilter ref="A1:E11" xr:uid="{EE7552C4-F486-457F-A2F8-480493B7351C}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="54"/>
-    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{7A1ACCA6-7C12-421C-A8B0-DAF52C5B82F1}" name="Added to Altium?" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{29766E43-A003-4F30-8FBC-98197408FA6D}" name="Part Number" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{9E0E83BD-C619-4B71-B8D8-093D6B07D9D5}" name="Package" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{6C643D04-D582-419C-9C7F-1B57D4315CFE}" name="Resistance" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{67D14711-9F21-4BBC-9182-15BB5F898016}" name="Description" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}" name="Fuses" displayName="Fuses" ref="A1:I10" totalsRowShown="0" headerRowDxfId="42">
   <autoFilter ref="A1:I10" xr:uid="{53E52592-BBF3-4884-BA3C-21683DC4F0F1}"/>
   <tableColumns count="9">
-    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{9030A4FE-0A13-4A65-8271-CB2306DED874}" name="Added to Altium?" dataDxfId="41"/>
+    <tableColumn id="8" xr3:uid="{7A093B6F-93A8-4A04-9A40-8451BE8854E4}" name="Type" dataDxfId="40"/>
     <tableColumn id="4" xr3:uid="{D6AD8AA5-BC88-4F36-A647-B68EB5308316}" name="Automotive Fuse Size"/>
     <tableColumn id="1" xr3:uid="{5D9981C8-F221-4013-A9BA-4E5BF3474E5D}" name="Trip Current"/>
     <tableColumn id="2" xr3:uid="{494ED5E9-E1DA-4E76-9EAF-806837FCC14C}" name="Package"/>
@@ -3416,14 +3425,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}" name="Inductors" displayName="Inductors" ref="A1:E11" totalsRowShown="0" headerRowDxfId="39">
   <autoFilter ref="A1:E11" xr:uid="{8788865D-3714-4394-BD76-99FF24EF6888}"/>
   <tableColumns count="5">
-    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="45"/>
-    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{67CA846A-F07D-4034-8F63-B4E47CA7F931}" name="Added to Altium?" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{EBC427FC-C649-421F-A511-F4C6E090217A}" name="Inductance" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{57FAF0ED-182E-4A05-89A5-EE5FE9CF2C31}" name="Package" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{5B4ACDCC-FB26-4063-91C8-D6D43ABD7134}" name="Part Number" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{CFE06357-AAEA-49E4-8ED8-14478316C7C8}" name="Description" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12078,6 +12087,15 @@
       <c r="A9" s="9" t="b">
         <v>0</v>
       </c>
+      <c r="B9" t="s">
+        <v>833</v>
+      </c>
+      <c r="C9" t="s">
+        <v>832</v>
+      </c>
+      <c r="D9" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="10" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="b">

</xml_diff>